<commit_message>
updated last 3 days details
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -5967,7 +5967,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H87"/>
+  <dimension ref="A1:H90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" style="331" min="1" max="1"/>
@@ -8768,30 +8768,129 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="430" t="inlineStr">
+      <c r="A87" s="430" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B87" s="232" t="inlineStr">
+        <is>
+          <t>Transfer-to-me (customer payment 14-Sep)</t>
+        </is>
+      </c>
+      <c r="C87" s="232" t="inlineStr">
+        <is>
+          <t>Transfer Received</t>
+        </is>
+      </c>
+      <c r="D87" s="232" t="n"/>
+      <c r="E87" s="233" t="n">
+        <v>130</v>
+      </c>
+      <c r="F87" s="233">
+        <f>IFERROR(F86+D87-E87,0)</f>
+        <v/>
+      </c>
+      <c r="G87" s="232" t="inlineStr">
+        <is>
+          <t>✅ Received</t>
+        </is>
+      </c>
+      <c r="H87" s="232" t="inlineStr">
+        <is>
+          <t>Customer paid Lohith personal acct</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="430" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B88" s="232" t="inlineStr">
+        <is>
+          <t>Transfer-to-me (customer payment 17-Sep)</t>
+        </is>
+      </c>
+      <c r="C88" s="232" t="inlineStr">
+        <is>
+          <t>Transfer Received</t>
+        </is>
+      </c>
+      <c r="D88" s="232" t="n"/>
+      <c r="E88" s="233" t="n">
+        <v>260</v>
+      </c>
+      <c r="F88" s="233">
+        <f>IFERROR(F87+D88-E88,0)</f>
+        <v/>
+      </c>
+      <c r="G88" s="232" t="inlineStr">
+        <is>
+          <t>✅ Received</t>
+        </is>
+      </c>
+      <c r="H88" s="232" t="inlineStr">
+        <is>
+          <t>Customer paid Lohith personal acct</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="430" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B89" s="232" t="inlineStr">
+        <is>
+          <t>Pollo $977 (paid by Lohith)</t>
+        </is>
+      </c>
+      <c r="C89" s="232" t="inlineStr">
+        <is>
+          <t>Expense - Personal</t>
+        </is>
+      </c>
+      <c r="D89" s="232" t="n">
+        <v>977</v>
+      </c>
+      <c r="E89" s="233" t="n"/>
+      <c r="F89" s="233">
+        <f>IFERROR(F88+D89-E89,0)</f>
+        <v/>
+      </c>
+      <c r="G89" s="232" t="inlineStr">
+        <is>
+          <t>⏳ Reimburse</t>
+        </is>
+      </c>
+      <c r="H89" s="232" t="inlineStr">
+        <is>
+          <t>Fronted from own pocket; excluded from till via cash_adjust</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="430" t="inlineStr">
         <is>
           <t>TOTALS &amp; CURRENT BALANCE</t>
         </is>
       </c>
-      <c r="B87" s="232" t="n"/>
-      <c r="C87" s="232" t="n"/>
-      <c r="D87" s="232">
-        <f>SUM(D4:D86)</f>
+      <c r="B90" s="232" t="n"/>
+      <c r="C90" s="232" t="n"/>
+      <c r="D90" s="232">
+        <f>SUM(D4:D89)</f>
         <v/>
       </c>
-      <c r="E87" s="233">
-        <f>SUM(E4:E86)</f>
+      <c r="E90" s="233">
+        <f>SUM(E4:E89)</f>
         <v/>
       </c>
-      <c r="F87" s="233">
-        <f>F86</f>
+      <c r="F90" s="233">
+        <f>F89</f>
         <v/>
       </c>
-      <c r="G87" s="232">
-        <f>IF(F86&gt;0,"Restaurant owes Lohith $"&amp;TEXT(F86,"#,##0"),IF(F86&lt;0,"Lohith holds $"&amp;TEXT(ABS(F86),"#,##0"),"Zero balance"))</f>
+      <c r="G90" s="232">
+        <f>IF(F89&gt;0,"Restaurant owes Lohith $"&amp;TEXT(F89,"#,##0"),IF(F89&lt;0,"Lohith holds $"&amp;TEXT(ABS(F89),"#,##0"),"Zero balance"))</f>
         <v/>
       </c>
-      <c r="H87" s="232" t="n"/>
+      <c r="H90" s="232" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -10625,45 +10724,45 @@
       <c r="E6" s="29" t="n"/>
       <c r="F6" s="30">
         <f>SUMIFS($D$8:$D$5000,$B$8:$B$5000,TODAY())+SUMIFS($E$8:$E$5000,$B$8:$B$5000,TODAY())+SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())</f>
-        <v>3345.0</v>
+        <v>4135.0</v>
       </c>
       <c r="G6" s="31">
         <f>SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())</f>
-        <v>1010.0</v>
+        <v>260.0</v>
       </c>
       <c r="H6" s="28">
         <f>SUMIFS($H$8:$H$5000,$B$8:$B$5000,TODAY())</f>
-        <v>45.0</v>
+        <v>1690.0</v>
       </c>
       <c r="I6" s="32">
         <f>F6-H6</f>
-        <v>3300.0</v>
+        <v>2445.0</v>
       </c>
       <c r="J6">
         <f>IFERROR(I6/F6,0)</f>
-        <v>0.986547</v>
+        <v>0.591294</v>
       </c>
       <c r="K6" s="28" t="n"/>
       <c r="L6" s="31" t="n"/>
       <c r="M6" s="28">
         <f>SUMPRODUCT((ISNUMBER($B$8:$B$5000))*($B$8:$B$5000&gt;=TODAY()-MOD(TODAY()-2,7))*($B$8:$B$5000&lt;TODAY()-MOD(TODAY()-2,7)+7)*IF(ISNUMBER($F$8:$F$5000),$F$8:$F$5000,0))</f>
-        <v>17130.0</v>
+        <v>8305.0</v>
       </c>
       <c r="N6" s="33">
         <f>SUMPRODUCT((ISNUMBER($B$8:$B$5000))*($B$8:$B$5000&gt;=TODAY()-MOD(TODAY()-2,7))*($B$8:$B$5000&lt;TODAY()-MOD(TODAY()-2,7)+7)*IF(ISNUMBER($F$8:$F$5000),$F$8:$F$5000,0))</f>
-        <v>17130.0</v>
+        <v>8305.0</v>
       </c>
       <c r="O6" s="33">
         <f>SUMPRODUCT((ISNUMBER($B$8:$B$5000))*(MONTH($B$8:$B$5000)=MONTH(TODAY()))*(YEAR($B$8:$B$5000)=YEAR(TODAY()))*IF(ISNUMBER($F$8:$F$5000),$F$8:$F$5000,0))</f>
-        <v>42674.0</v>
+        <v>53399.0</v>
       </c>
       <c r="P6">
         <f>SUMPRODUCT((ISNUMBER($B$8:$B$5000))*($B$8:$B$5000&gt;=TODAY()-MOD(TODAY()-2,7))*($B$8:$B$5000&lt;TODAY()-MOD(TODAY()-2,7)+7)*IF(ISNUMBER($H$8:$H$5000),$H$8:$H$5000,0))</f>
-        <v>11078.0</v>
+        <v>2350.0</v>
       </c>
       <c r="Q6">
         <f>M6-P6</f>
-        <v>6052.0</v>
+        <v>5955.0</v>
       </c>
     </row>
     <row r="7" ht="27.75" customHeight="1" s="331">
@@ -17625,91 +17724,208 @@
       <c r="AB114" s="324" t="n"/>
     </row>
     <row r="115" ht="16.5" customHeight="1" s="331">
-      <c r="B115" s="34" t="n"/>
-      <c r="C115" s="47" t="n"/>
-      <c r="D115" s="48" t="n"/>
-      <c r="E115" s="49" t="n"/>
-      <c r="F115" s="50" t="n"/>
-      <c r="G115" s="51" t="n"/>
-      <c r="H115" s="52" t="n"/>
-      <c r="I115" s="53" t="n"/>
-      <c r="J115" s="54" t="n"/>
-      <c r="K115" s="55" t="n"/>
-      <c r="L115" s="18" t="n"/>
-      <c r="M115" s="21" t="n"/>
-      <c r="N115" s="56" t="n"/>
-      <c r="O115" s="57" t="n"/>
-      <c r="P115" s="58" t="n"/>
-      <c r="Q115" s="56" t="n"/>
-      <c r="R115" s="56" t="n"/>
-      <c r="S115" s="56" t="n"/>
-      <c r="T115" s="56" t="n"/>
-      <c r="U115" s="56" t="n"/>
-      <c r="V115" s="56" t="n"/>
-      <c r="W115" s="56" t="n"/>
-      <c r="X115" s="56" t="n"/>
-      <c r="Y115" s="56" t="n"/>
-      <c r="Z115" s="56" t="n"/>
-      <c r="AA115" s="56" t="n"/>
-      <c r="AB115" s="56" t="n"/>
+      <c r="B115" s="427" t="n">
+        <v>46277</v>
+      </c>
+      <c r="C115" s="255" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="D115" s="256" t="n">
+        <v>585</v>
+      </c>
+      <c r="E115" s="49" t="n">
+        <v>1835</v>
+      </c>
+      <c r="F115" s="50">
+        <f>IFERROR(D115+E115+G115+U115+Y115,0)</f>
+        <v>2420.0</v>
+      </c>
+      <c r="G115" s="257" t="n">
+        <v>0</v>
+      </c>
+      <c r="H115" s="258">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B115,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B115+1))</f>
+        <v>8813.0</v>
+      </c>
+      <c r="I115" s="259">
+        <f>IFERROR(F115-H115,0)</f>
+        <v>-6393.0</v>
+      </c>
+      <c r="J115" s="260">
+        <f>IFERROR(I115/F115,0)</f>
+        <v>-2.641736</v>
+      </c>
+      <c r="K115" s="254" t="n"/>
+      <c r="L115" s="261" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
+      <c r="M115" s="291" t="n"/>
+      <c r="N115" s="292" t="n"/>
+      <c r="O115" s="293" t="n"/>
+      <c r="P115" s="294" t="n"/>
+      <c r="Q115" s="292" t="n"/>
+      <c r="R115" s="443">
+        <f>IFERROR(D115*$T$7,0)</f>
+        <v>23.75</v>
+      </c>
+      <c r="S115" s="292" t="n"/>
+      <c r="T115" s="292" t="n"/>
+      <c r="U115" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="V115" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="W115" s="292" t="n"/>
+      <c r="X115" s="292" t="n"/>
+      <c r="Y115" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z115" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA115" s="292" t="n"/>
+      <c r="AB115" s="292" t="n"/>
     </row>
     <row r="116" ht="16.5" customHeight="1" s="331">
-      <c r="B116" s="34" t="n"/>
-      <c r="C116" s="35" t="n"/>
-      <c r="D116" s="36" t="n"/>
-      <c r="E116" s="37" t="n"/>
-      <c r="F116" s="38" t="n"/>
-      <c r="G116" s="39" t="n"/>
-      <c r="H116" s="40" t="n"/>
-      <c r="I116" s="41" t="n"/>
-      <c r="J116" s="42" t="n"/>
-      <c r="K116" s="43" t="n"/>
-      <c r="L116" s="9" t="n"/>
-      <c r="M116" s="12" t="n"/>
-      <c r="N116" s="44" t="n"/>
-      <c r="O116" s="45" t="n"/>
-      <c r="P116" s="46" t="n"/>
-      <c r="Q116" s="44" t="n"/>
-      <c r="R116" s="44" t="n"/>
-      <c r="S116" s="44" t="n"/>
-      <c r="T116" s="44" t="n"/>
-      <c r="U116" s="44" t="n"/>
-      <c r="V116" s="44" t="n"/>
-      <c r="W116" s="44" t="n"/>
-      <c r="X116" s="44" t="n"/>
-      <c r="Y116" s="44" t="n"/>
-      <c r="Z116" s="44" t="n"/>
-      <c r="AA116" s="44" t="n"/>
-      <c r="AB116" s="44" t="n"/>
+      <c r="B116" s="427" t="n">
+        <v>46279</v>
+      </c>
+      <c r="C116" s="270" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D116" s="271" t="n">
+        <v>1950</v>
+      </c>
+      <c r="E116" s="37" t="n">
+        <v>2090</v>
+      </c>
+      <c r="F116" s="38">
+        <f>IFERROR(D116+E116+G116+U116+Y116,0)</f>
+        <v>4170.0</v>
+      </c>
+      <c r="G116" s="272" t="n">
+        <v>130</v>
+      </c>
+      <c r="H116" s="273">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B116,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B116+1))</f>
+        <v>660.0</v>
+      </c>
+      <c r="I116" s="274">
+        <f>IFERROR(F116-H116,0)</f>
+        <v>3510.0</v>
+      </c>
+      <c r="J116" s="275">
+        <f>IFERROR(I116/F116,0)</f>
+        <v>0.841727</v>
+      </c>
+      <c r="K116" s="250" t="n"/>
+      <c r="L116" s="276" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
+      <c r="M116" s="323" t="n"/>
+      <c r="N116" s="324" t="n"/>
+      <c r="O116" s="325" t="n"/>
+      <c r="P116" s="326" t="n"/>
+      <c r="Q116" s="324" t="n"/>
+      <c r="R116" s="428">
+        <f>IFERROR(D116*$T$7,0)</f>
+        <v>79.17</v>
+      </c>
+      <c r="S116" s="324" t="n"/>
+      <c r="T116" s="324" t="n"/>
+      <c r="U116" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="V116" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="W116" s="324" t="n"/>
+      <c r="X116" s="324" t="n"/>
+      <c r="Y116" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z116" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA116" s="324" t="n"/>
+      <c r="AB116" s="324" t="n"/>
     </row>
     <row r="117" ht="16.5" customHeight="1" s="331">
-      <c r="B117" s="34" t="n"/>
-      <c r="C117" s="47" t="n"/>
-      <c r="D117" s="48" t="n"/>
-      <c r="E117" s="49" t="n"/>
-      <c r="F117" s="50" t="n"/>
-      <c r="G117" s="51" t="n"/>
-      <c r="H117" s="52" t="n"/>
-      <c r="I117" s="53" t="n"/>
-      <c r="J117" s="54" t="n"/>
-      <c r="K117" s="55" t="n"/>
-      <c r="L117" s="18" t="n"/>
-      <c r="M117" s="21" t="n"/>
-      <c r="N117" s="56" t="n"/>
-      <c r="O117" s="57" t="n"/>
-      <c r="P117" s="58" t="n"/>
-      <c r="Q117" s="56" t="n"/>
-      <c r="R117" s="56" t="n"/>
-      <c r="S117" s="56" t="n"/>
-      <c r="T117" s="56" t="n"/>
-      <c r="U117" s="56" t="n"/>
-      <c r="V117" s="56" t="n"/>
-      <c r="W117" s="56" t="n"/>
-      <c r="X117" s="56" t="n"/>
-      <c r="Y117" s="56" t="n"/>
-      <c r="Z117" s="56" t="n"/>
-      <c r="AA117" s="56" t="n"/>
-      <c r="AB117" s="56" t="n"/>
+      <c r="B117" s="427" t="n">
+        <v>46282</v>
+      </c>
+      <c r="C117" s="255" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D117" s="256" t="n">
+        <v>2875</v>
+      </c>
+      <c r="E117" s="49" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F117" s="50">
+        <f>IFERROR(D117+E117+G117+U117+Y117,0)</f>
+        <v>4135.0</v>
+      </c>
+      <c r="G117" s="257" t="n">
+        <v>260</v>
+      </c>
+      <c r="H117" s="258">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B117,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B117+1))</f>
+        <v>1690.0</v>
+      </c>
+      <c r="I117" s="259">
+        <f>IFERROR(F117-H117,0)</f>
+        <v>2445.0</v>
+      </c>
+      <c r="J117" s="260">
+        <f>IFERROR(I117/F117,0)</f>
+        <v>0.591294</v>
+      </c>
+      <c r="K117" s="254" t="n"/>
+      <c r="L117" s="261" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
+      <c r="M117" s="291" t="n"/>
+      <c r="N117" s="292" t="n"/>
+      <c r="O117" s="293" t="n"/>
+      <c r="P117" s="294" t="n"/>
+      <c r="Q117" s="292" t="n"/>
+      <c r="R117" s="443">
+        <f>IFERROR(D117*$T$7,0)</f>
+        <v>116.72</v>
+      </c>
+      <c r="S117" s="292" t="n"/>
+      <c r="T117" s="292" t="n"/>
+      <c r="U117" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="V117" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="W117" s="292" t="n"/>
+      <c r="X117" s="292" t="n"/>
+      <c r="Y117" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z117" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA117" s="292" t="n"/>
+      <c r="AB117" s="292" t="n"/>
     </row>
     <row r="118" ht="16.5" customHeight="1" s="331">
       <c r="B118" s="34" t="n"/>
@@ -25133,7 +25349,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J764"/>
+  <dimension ref="A1:J774"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="4" customWidth="1" style="331" min="1" max="1"/>
@@ -57488,6 +57704,436 @@
       <c r="J764" s="423" t="inlineStr">
         <is>
           <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="B765" s="429" t="n">
+        <v>46277</v>
+      </c>
+      <c r="C765" s="297" t="inlineStr">
+        <is>
+          <t>Carne</t>
+        </is>
+      </c>
+      <c r="D765" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E765" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat</t>
+        </is>
+      </c>
+      <c r="F765" s="299" t="n">
+        <v>300</v>
+      </c>
+      <c r="G765" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H765" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I765" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J765" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="766">
+      <c r="B766" s="429" t="n">
+        <v>46277</v>
+      </c>
+      <c r="C766" s="297" t="inlineStr">
+        <is>
+          <t>Vegetales</t>
+        </is>
+      </c>
+      <c r="D766" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E766" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Vegetables</t>
+        </is>
+      </c>
+      <c r="F766" s="299" t="n">
+        <v>950</v>
+      </c>
+      <c r="G766" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H766" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I766" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J766" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="B767" s="429" t="n">
+        <v>46277</v>
+      </c>
+      <c r="C767" s="297" t="inlineStr">
+        <is>
+          <t>Chedraui</t>
+        </is>
+      </c>
+      <c r="D767" s="298" t="inlineStr">
+        <is>
+          <t>Chedraui</t>
+        </is>
+      </c>
+      <c r="E767" s="297" t="inlineStr">
+        <is>
+          <t>Supermarket/General</t>
+        </is>
+      </c>
+      <c r="F767" s="299" t="n">
+        <v>153</v>
+      </c>
+      <c r="G767" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H767" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I767" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J767" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="B768" s="429" t="n">
+        <v>46277</v>
+      </c>
+      <c r="C768" s="297" t="inlineStr">
+        <is>
+          <t>Duvi - salary</t>
+        </is>
+      </c>
+      <c r="D768" s="298" t="inlineStr">
+        <is>
+          <t>Payroll</t>
+        </is>
+      </c>
+      <c r="E768" s="297" t="inlineStr">
+        <is>
+          <t>Staff - Salary</t>
+        </is>
+      </c>
+      <c r="F768" s="299" t="n">
+        <v>1460</v>
+      </c>
+      <c r="G768" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H768" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I768" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J768" s="423" t="inlineStr">
+        <is>
+          <t>Weekly salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="B769" s="429" t="n">
+        <v>46277</v>
+      </c>
+      <c r="C769" s="297" t="inlineStr">
+        <is>
+          <t>Armando - salary</t>
+        </is>
+      </c>
+      <c r="D769" s="298" t="inlineStr">
+        <is>
+          <t>Payroll</t>
+        </is>
+      </c>
+      <c r="E769" s="297" t="inlineStr">
+        <is>
+          <t>Staff - Salary</t>
+        </is>
+      </c>
+      <c r="F769" s="299" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G769" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H769" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I769" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J769" s="423" t="inlineStr">
+        <is>
+          <t>Weekly salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="B770" s="429" t="n">
+        <v>46277</v>
+      </c>
+      <c r="C770" s="297" t="inlineStr">
+        <is>
+          <t>Jhon - salary</t>
+        </is>
+      </c>
+      <c r="D770" s="298" t="inlineStr">
+        <is>
+          <t>Payroll</t>
+        </is>
+      </c>
+      <c r="E770" s="297" t="inlineStr">
+        <is>
+          <t>Staff - Salary</t>
+        </is>
+      </c>
+      <c r="F770" s="299" t="n">
+        <v>3750</v>
+      </c>
+      <c r="G770" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H770" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I770" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J770" s="423" t="inlineStr">
+        <is>
+          <t>Weekly salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="B771" s="429" t="n">
+        <v>46279</v>
+      </c>
+      <c r="C771" s="297" t="inlineStr">
+        <is>
+          <t>Queso Panela</t>
+        </is>
+      </c>
+      <c r="D771" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E771" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Dairy</t>
+        </is>
+      </c>
+      <c r="F771" s="299" t="n">
+        <v>590</v>
+      </c>
+      <c r="G771" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H771" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I771" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J771" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="B772" s="429" t="n">
+        <v>46279</v>
+      </c>
+      <c r="C772" s="297" t="inlineStr">
+        <is>
+          <t>oxxo</t>
+        </is>
+      </c>
+      <c r="D772" s="298" t="inlineStr">
+        <is>
+          <t>OXXO</t>
+        </is>
+      </c>
+      <c r="E772" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Pantry</t>
+        </is>
+      </c>
+      <c r="F772" s="299" t="n">
+        <v>70</v>
+      </c>
+      <c r="G772" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H772" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I772" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J772" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="B773" s="429" t="n">
+        <v>46282</v>
+      </c>
+      <c r="C773" s="297" t="inlineStr">
+        <is>
+          <t>Sams Club</t>
+        </is>
+      </c>
+      <c r="D773" s="298" t="inlineStr">
+        <is>
+          <t>Sam's Club</t>
+        </is>
+      </c>
+      <c r="E773" s="297" t="inlineStr">
+        <is>
+          <t>Supermarket/General</t>
+        </is>
+      </c>
+      <c r="F773" s="299" t="n">
+        <v>713</v>
+      </c>
+      <c r="G773" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H773" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I773" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J773" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="B774" s="429" t="n">
+        <v>46282</v>
+      </c>
+      <c r="C774" s="297" t="inlineStr">
+        <is>
+          <t>Pollo</t>
+        </is>
+      </c>
+      <c r="D774" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E774" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat</t>
+        </is>
+      </c>
+      <c r="F774" s="299" t="n">
+        <v>977</v>
+      </c>
+      <c r="G774" s="300" t="inlineStr">
+        <is>
+          <t>Lohith</t>
+        </is>
+      </c>
+      <c r="H774" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I774" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J774" s="423" t="inlineStr">
+        <is>
+          <t>Pagado por Lohith (bolsillo); reembolsable via Owner Ledger</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update todays details and reanchored cash count
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -10887,7 +10887,7 @@
       <c r="E6" s="29" t="n"/>
       <c r="F6" s="30">
         <f>SUMIFS($D$8:$D$5000,$B$8:$B$5000,TODAY())+SUMIFS($E$8:$E$5000,$B$8:$B$5000,TODAY())+SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())+SUMIFS($U$8:$U$5000,$B$8:$B$5000,TODAY())+SUMIFS($Y$8:$Y$5000,$B$8:$B$5000,TODAY())</f>
-        <v>2325.0</v>
+        <v>1960.0</v>
       </c>
       <c r="G6" s="31">
         <f>SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())</f>
@@ -10895,37 +10895,37 @@
       </c>
       <c r="H6" s="28">
         <f>SUMIFS($H$8:$H$5000,$B$8:$B$5000,TODAY())</f>
-        <v>1979.0</v>
+        <v>4626.0</v>
       </c>
       <c r="I6" s="32">
         <f>F6-H6</f>
-        <v>346.0</v>
+        <v>-2666.0</v>
       </c>
       <c r="J6">
         <f>IFERROR(I6/F6,0)</f>
-        <v>0.148817</v>
+        <v>-1.360204</v>
       </c>
       <c r="K6" s="28" t="n"/>
       <c r="L6" s="31" t="n"/>
       <c r="M6" s="28">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>26526.0</v>
+        <v>28486.0</v>
       </c>
       <c r="N6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>26526.0</v>
+        <v>28486.0</v>
       </c>
       <c r="O6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),$B$8:$B$5000,"&lt;"&amp;DATE(YEAR(TODAY()),MONTH(TODAY())+1,1))</f>
-        <v>71620.0</v>
+        <v>73580.0</v>
       </c>
       <c r="P6">
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>5433.0</v>
+        <v>10059.0</v>
       </c>
       <c r="Q6">
         <f>M6-P6</f>
-        <v>21093.0</v>
+        <v>18427.0</v>
       </c>
     </row>
     <row r="7" ht="27.75" customHeight="1" s="331">
@@ -18162,33 +18162,72 @@
       <c r="AB118" s="324" t="n"/>
     </row>
     <row r="119" ht="16.5" customHeight="1" s="331">
-      <c r="B119" s="34" t="n"/>
-      <c r="C119" s="47" t="n"/>
-      <c r="D119" s="48" t="n"/>
-      <c r="E119" s="49" t="n"/>
-      <c r="F119" s="50" t="n"/>
-      <c r="G119" s="51" t="n"/>
-      <c r="H119" s="52" t="n"/>
-      <c r="I119" s="53" t="n"/>
-      <c r="J119" s="54" t="n"/>
-      <c r="K119" s="55" t="n"/>
-      <c r="L119" s="18" t="n"/>
-      <c r="M119" s="21" t="n"/>
-      <c r="N119" s="56" t="n"/>
-      <c r="O119" s="57" t="n"/>
-      <c r="P119" s="58" t="n"/>
-      <c r="Q119" s="56" t="n"/>
-      <c r="R119" s="56" t="n"/>
-      <c r="S119" s="56" t="n"/>
-      <c r="T119" s="56" t="n"/>
-      <c r="U119" s="56" t="n"/>
-      <c r="V119" s="56" t="n"/>
-      <c r="W119" s="56" t="n"/>
-      <c r="X119" s="56" t="n"/>
-      <c r="Y119" s="56" t="n"/>
-      <c r="Z119" s="56" t="n"/>
-      <c r="AA119" s="56" t="n"/>
-      <c r="AB119" s="56" t="n"/>
+      <c r="B119" s="427" t="n">
+        <v>46284</v>
+      </c>
+      <c r="C119" s="255" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="D119" s="256" t="n">
+        <v>625</v>
+      </c>
+      <c r="E119" s="49" t="n">
+        <v>1335</v>
+      </c>
+      <c r="F119" s="50">
+        <f>IFERROR(D119+E119+G119+U119+Y119,0)</f>
+        <v>1960.0</v>
+      </c>
+      <c r="G119" s="257" t="n">
+        <v>0</v>
+      </c>
+      <c r="H119" s="258">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B119,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B119+1))</f>
+        <v>4626.0</v>
+      </c>
+      <c r="I119" s="259">
+        <f>IFERROR(F119-H119,0)</f>
+        <v>-2666.0</v>
+      </c>
+      <c r="J119" s="260">
+        <f>IFERROR(I119/F119,0)</f>
+        <v>-1.360204</v>
+      </c>
+      <c r="K119" s="254" t="n"/>
+      <c r="L119" s="261" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
+      <c r="M119" s="291" t="n"/>
+      <c r="N119" s="292" t="n"/>
+      <c r="O119" s="293" t="n"/>
+      <c r="P119" s="294" t="n"/>
+      <c r="Q119" s="292" t="n"/>
+      <c r="R119" s="443">
+        <f>IFERROR(D119*$T$7,0)</f>
+        <v>25.38</v>
+      </c>
+      <c r="S119" s="292" t="n"/>
+      <c r="T119" s="292" t="n"/>
+      <c r="U119" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="V119" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="W119" s="292" t="n"/>
+      <c r="X119" s="292" t="n"/>
+      <c r="Y119" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z119" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA119" s="292" t="n"/>
+      <c r="AB119" s="292" t="n"/>
     </row>
     <row r="120" ht="16.5" customHeight="1" s="331">
       <c r="B120" s="34" t="n"/>
@@ -25529,9 +25568,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="B5:P5"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="I2:P2"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="B5:P5"/>
     <mergeCell ref="A3:P3"/>
   </mergeCells>
   <conditionalFormatting sqref="I8:I372">
@@ -25554,7 +25593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J782"/>
+  <dimension ref="A1:J784"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="4" customWidth="1" style="331" min="1" max="1"/>
@@ -58683,6 +58722,92 @@
       <c r="J782" s="423" t="inlineStr">
         <is>
           <t>No receipt; cash. Typed as 'Guimar 2333w' on 04-Sep and dropped by eod.py; confirmed $226 by Reddy 18-Sep</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="B783" s="429" t="n">
+        <v>46284</v>
+      </c>
+      <c r="C783" s="297" t="inlineStr">
+        <is>
+          <t>Jhon - salary</t>
+        </is>
+      </c>
+      <c r="D783" s="298" t="inlineStr">
+        <is>
+          <t>Payroll</t>
+        </is>
+      </c>
+      <c r="E783" s="297" t="inlineStr">
+        <is>
+          <t>Staff - Salary</t>
+        </is>
+      </c>
+      <c r="F783" s="299" t="n">
+        <v>3750</v>
+      </c>
+      <c r="G783" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H783" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I783" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J783" s="423" t="inlineStr">
+        <is>
+          <t>Weekly salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="B784" s="429" t="n">
+        <v>46284</v>
+      </c>
+      <c r="C784" s="297" t="inlineStr">
+        <is>
+          <t>Duvi - salary</t>
+        </is>
+      </c>
+      <c r="D784" s="298" t="inlineStr">
+        <is>
+          <t>Payroll</t>
+        </is>
+      </c>
+      <c r="E784" s="297" t="inlineStr">
+        <is>
+          <t>Staff - Salary</t>
+        </is>
+      </c>
+      <c r="F784" s="299" t="n">
+        <v>876</v>
+      </c>
+      <c r="G784" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H784" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I784" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J784" s="423" t="inlineStr">
+        <is>
+          <t>Weekly salary</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
LOKA 05-Oct-2026 | manual push | day 2026-10-05: rev $5,580 exp $29,006 net $-23,426 | bal vs capital $-19,119
Changed: ackup/LOKA_2026-09-17_16-58-42_eod_sep12.xlsx, HOWTO.md, LOKA.bat, LOKA_Restaurant_Manager.xlsx, NOTES.md, dashboard.html, loka.py, tools.py, gdrive_backup.py, git_push.py
+ 18 backup/day file(s)
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -25,7 +25,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="13">
+  <numFmts count="14">
     <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);&quot;-&quot;"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy\ ddd"/>
     <numFmt numFmtId="166" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
@@ -39,6 +39,7 @@
     <numFmt numFmtId="174" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="175" formatCode="dd-mmm-yyyy"/>
     <numFmt numFmtId="176" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="177" formatCode="$#,##0.00;[Red]-$#,##0.00"/>
   </numFmts>
   <fonts count="103">
     <font>
@@ -1366,7 +1367,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25"/>
   </cellStyleXfs>
-  <cellXfs count="454">
+  <cellXfs count="458">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -2517,6 +2518,10 @@
     <xf numFmtId="0" fontId="92" fillId="44" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="176" fontId="95" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="176" fontId="98" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="98" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="177" fontId="98" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="95" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="177" fontId="95" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2960,7 +2965,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H171"/>
+  <dimension ref="A1:H173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="3" customWidth="1" style="331" min="1" max="1"/>
@@ -2981,7 +2986,7 @@
     <row r="2" ht="24" customHeight="1" s="331">
       <c r="B2" s="414" t="inlineStr">
         <is>
-          <t>Last updated: 22 Sep 2026  |  Capital, Acquisition, Pre-Opening, Renovation CapEx &amp; Operations↔Capital</t>
+          <t>Last updated: 05 Oct 2026  |  Capital, Acquisition, Pre-Opening, Renovation CapEx &amp; Operations↔Capital</t>
         </is>
       </c>
     </row>
@@ -5527,11 +5532,11 @@
         </is>
       </c>
       <c r="C147" s="268" t="n">
-        <v>18442</v>
+        <v>0</v>
       </c>
       <c r="E147" s="286" t="inlineStr">
         <is>
-          <t>Operating costs funded from partner capital, net of repayments. Latest addition 22-Sep-2026 $18,442.00. Still owed by Operations: $18,442.00.</t>
+          <t>Legacy (to 22-Sep-2026). From 05-Oct-2026 capital is fixed at $125,934 in the company account; what ops owes Capital = negative Balance vs Capital (row 172). 22-Sep taxes/contador moved to Restaurant.</t>
         </is>
       </c>
     </row>
@@ -5816,7 +5821,7 @@
     <row r="169">
       <c r="B169" s="319" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Moved INTO company account (capital deposits + repayments kept there)</t>
+          <t xml:space="preserve">   CAPITAL held in company account (fixed, moved in 22-Sep-2026)</t>
         </is>
       </c>
       <c r="C169" s="452" t="n">
@@ -5824,29 +5829,29 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>22-Sep-2026: +$125,934.00 Lohith moved all remaining capital to company account.</t>
+          <t>22-Sep-2026: Lohith moved all remaining capital ($125,934) to the company account.</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="B170" s="319" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Drawn from reserve (bills paid with capital from company account)</t>
+          <t xml:space="preserve">   Drawn from capital (retired 05-Oct-2026: all bills are normal company-account expenses)</t>
         </is>
       </c>
       <c r="C170" s="452" t="n">
-        <v>-18442</v>
+        <v>0</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Cumulative draws (menu 5). Negative number. | 22-Sep-2026: -$18,442.00 Impuestos junio, julio y agosto 2026, Honorarios Julio Contador</t>
+          <t>22-Sep taxes/contador draw (-$18,442) reversed 05-Oct-2026 and booked as Restaurant expenses.</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="B171" s="317" t="inlineStr">
         <is>
-          <t>CAPITAL RESERVE BALANCE (in company account)</t>
+          <t>CAPITAL BALANCE (fixed, in company account)</t>
         </is>
       </c>
       <c r="C171" s="453">
@@ -5855,7 +5860,37 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Counted in the bank at a cash count, but NOT operating cash. Recount subtracts it.</t>
+          <t>The pool (company account + cash in hand) must cover this. Difference is row 172.</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="B172" s="454" t="inlineStr">
+        <is>
+          <t>BALANCE vs CAPITAL  (company acct + cash in hand − capital)</t>
+        </is>
+      </c>
+      <c r="C172" s="455" t="n">
+        <v>-19118.92</v>
+      </c>
+      <c r="E172" s="423" t="inlineStr">
+        <is>
+          <t>Negative = the restaurant owes Capital this much. Positive = surplus. Auto-updated by refresh-all.</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="B173" s="456" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Company account + cash in hand (books)</t>
+        </is>
+      </c>
+      <c r="C173" s="457" t="n">
+        <v>106815.08</v>
+      </c>
+      <c r="E173" s="423" t="inlineStr">
+        <is>
+          <t>Last physical count + everything since. Set by menu 13 (cash count). Auto-updated by refresh-all.</t>
         </is>
       </c>
     </row>
@@ -6022,7 +6057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H100"/>
+  <dimension ref="A1:H104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" style="331" min="1" max="1"/>
@@ -9252,30 +9287,162 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="430" t="inlineStr">
+      <c r="A100" s="430" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B100" s="232" t="inlineStr">
+        <is>
+          <t>Transfer-to-me (customer payment 01-Oct)</t>
+        </is>
+      </c>
+      <c r="C100" s="232" t="inlineStr">
+        <is>
+          <t>Transfer Received</t>
+        </is>
+      </c>
+      <c r="D100" s="232" t="n"/>
+      <c r="E100" s="233" t="n">
+        <v>130</v>
+      </c>
+      <c r="F100" s="233">
+        <f>IFERROR(F99+D100-E100,0)</f>
+        <v/>
+      </c>
+      <c r="G100" s="232" t="inlineStr">
+        <is>
+          <t>✅ Received</t>
+        </is>
+      </c>
+      <c r="H100" s="232" t="inlineStr">
+        <is>
+          <t>Customer paid Lohith personal acct</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="430" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B101" s="232" t="inlineStr">
+        <is>
+          <t>Settlement - Lohith returned restaurant money</t>
+        </is>
+      </c>
+      <c r="C101" s="232" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+      <c r="D101" s="232" t="n">
+        <v>1599.47</v>
+      </c>
+      <c r="E101" s="233" t="n"/>
+      <c r="F101" s="233">
+        <f>IFERROR(F100+D101-E101,0)</f>
+        <v/>
+      </c>
+      <c r="G101" s="232" t="inlineStr">
+        <is>
+          <t>✅ Settled</t>
+        </is>
+      </c>
+      <c r="H101" s="232" t="inlineStr">
+        <is>
+          <t>Lohith handed back cash he was holding</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="430" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B102" s="232" t="inlineStr">
+        <is>
+          <t>Transfer-to-me (customer payment 05-Oct)</t>
+        </is>
+      </c>
+      <c r="C102" s="232" t="inlineStr">
+        <is>
+          <t>Transfer Received</t>
+        </is>
+      </c>
+      <c r="D102" s="232" t="n"/>
+      <c r="E102" s="233" t="n">
+        <v>965</v>
+      </c>
+      <c r="F102" s="233">
+        <f>IFERROR(F101+D102-E102,0)</f>
+        <v/>
+      </c>
+      <c r="G102" s="232" t="inlineStr">
+        <is>
+          <t>✅ Received</t>
+        </is>
+      </c>
+      <c r="H102" s="232" t="inlineStr">
+        <is>
+          <t>Customer paid Lohith personal acct</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="430" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B103" s="232" t="inlineStr">
+        <is>
+          <t>Pollo $912 (paid by Lohith)</t>
+        </is>
+      </c>
+      <c r="C103" s="232" t="inlineStr">
+        <is>
+          <t>Expense - Personal</t>
+        </is>
+      </c>
+      <c r="D103" s="232" t="n">
+        <v>912</v>
+      </c>
+      <c r="E103" s="233" t="n"/>
+      <c r="F103" s="233">
+        <f>IFERROR(F102+D103-E103,0)</f>
+        <v/>
+      </c>
+      <c r="G103" s="232" t="inlineStr">
+        <is>
+          <t>⏳ Reimburse</t>
+        </is>
+      </c>
+      <c r="H103" s="232" t="inlineStr">
+        <is>
+          <t>Fronted from own pocket; excluded from till via cash_adjust</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="430" t="inlineStr">
         <is>
           <t>TOTALS &amp; CURRENT BALANCE</t>
         </is>
       </c>
-      <c r="B100" s="232" t="n"/>
-      <c r="C100" s="232" t="n"/>
-      <c r="D100" s="232">
-        <f>SUM(D4:D99)</f>
-        <v/>
-      </c>
-      <c r="E100" s="233">
-        <f>SUM(E4:E99)</f>
-        <v/>
-      </c>
-      <c r="F100" s="233">
-        <f>F99</f>
-        <v/>
-      </c>
-      <c r="G100" s="232">
-        <f>IF(F99&gt;0,"Restaurant owes Lohith $"&amp;TEXT(F99,"#,##0"),IF(F99&lt;0,"Lohith holds $"&amp;TEXT(ABS(F99),"#,##0"),"Zero balance"))</f>
-        <v/>
-      </c>
-      <c r="H100" s="232" t="n"/>
+      <c r="B104" s="232" t="n"/>
+      <c r="C104" s="232" t="n"/>
+      <c r="D104" s="232">
+        <f>SUM(D4:D103)</f>
+        <v/>
+      </c>
+      <c r="E104" s="233">
+        <f>SUM(E4:E103)</f>
+        <v/>
+      </c>
+      <c r="F104" s="233">
+        <f>F103</f>
+        <v/>
+      </c>
+      <c r="G104" s="232">
+        <f>IF(F103&gt;0,"Restaurant owes Lohith $"&amp;TEXT(F103,"#,##0"),IF(F103&lt;0,"Lohith holds $"&amp;TEXT(ABS(F103),"#,##0"),"Zero balance"))</f>
+        <v/>
+      </c>
+      <c r="H104" s="232" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -11109,45 +11276,45 @@
       <c r="E6" s="29" t="n"/>
       <c r="F6" s="30">
         <f>SUMIFS($D$8:$D$5000,$B$8:$B$5000,TODAY())+SUMIFS($E$8:$E$5000,$B$8:$B$5000,TODAY())+SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())+SUMIFS($U$8:$U$5000,$B$8:$B$5000,TODAY())+SUMIFS($Y$8:$Y$5000,$B$8:$B$5000,TODAY())</f>
-        <v>3820.0</v>
+        <v>5580.0</v>
       </c>
       <c r="G6" s="31">
         <f>SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())</f>
-        <v>530.0</v>
+        <v>965.0</v>
       </c>
       <c r="H6" s="28">
         <f>SUMIFS($H$8:$H$5000,$B$8:$B$5000,TODAY())</f>
-        <v>1535.0</v>
+        <v>29005.68</v>
       </c>
       <c r="I6" s="32">
         <f>F6-H6</f>
-        <v>2285.0</v>
+        <v>-23425.68</v>
       </c>
       <c r="J6">
         <f>IFERROR(I6/F6,0)</f>
-        <v>0.598168</v>
+        <v>-4.198151</v>
       </c>
       <c r="K6" s="28" t="n"/>
       <c r="L6" s="31" t="n"/>
       <c r="M6" s="28">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>11142.0</v>
+        <v>5580.0</v>
       </c>
       <c r="N6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>11142.0</v>
+        <v>5580.0</v>
       </c>
       <c r="O6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),$B$8:$B$5000,"&lt;"&amp;DATE(YEAR(TODAY()),MONTH(TODAY())+1,1))</f>
-        <v>106977.0</v>
+        <v>14335.0</v>
       </c>
       <c r="P6">
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>2647.0</v>
+        <v>29005.68</v>
       </c>
       <c r="Q6">
         <f>M6-P6</f>
-        <v>8495.0</v>
+        <v>-23425.68</v>
       </c>
     </row>
     <row r="7" ht="27.75" customHeight="1" s="331">
@@ -19064,91 +19231,208 @@
       <c r="AB128" s="324" t="n"/>
     </row>
     <row r="129" ht="16.5" customHeight="1" s="331">
-      <c r="B129" s="34" t="n"/>
-      <c r="C129" s="47" t="n"/>
-      <c r="D129" s="48" t="n"/>
-      <c r="E129" s="49" t="n"/>
-      <c r="F129" s="50" t="n"/>
-      <c r="G129" s="51" t="n"/>
-      <c r="H129" s="52" t="n"/>
-      <c r="I129" s="53" t="n"/>
-      <c r="J129" s="54" t="n"/>
-      <c r="K129" s="55" t="n"/>
-      <c r="L129" s="18" t="n"/>
-      <c r="M129" s="21" t="n"/>
-      <c r="N129" s="56" t="n"/>
-      <c r="O129" s="57" t="n"/>
-      <c r="P129" s="58" t="n"/>
-      <c r="Q129" s="56" t="n"/>
-      <c r="R129" s="56" t="n"/>
-      <c r="S129" s="56" t="n"/>
-      <c r="T129" s="56" t="n"/>
-      <c r="U129" s="56" t="n"/>
-      <c r="V129" s="56" t="n"/>
-      <c r="W129" s="56" t="n"/>
-      <c r="X129" s="56" t="n"/>
-      <c r="Y129" s="56" t="n"/>
-      <c r="Z129" s="56" t="n"/>
-      <c r="AA129" s="56" t="n"/>
-      <c r="AB129" s="56" t="n"/>
+      <c r="B129" s="427" t="n">
+        <v>46296</v>
+      </c>
+      <c r="C129" s="255" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D129" s="256" t="n">
+        <v>1350</v>
+      </c>
+      <c r="E129" s="49" t="n">
+        <v>940</v>
+      </c>
+      <c r="F129" s="50">
+        <f>IFERROR(D129+E129+G129+U129+Y129,0)</f>
+        <v>2420.0</v>
+      </c>
+      <c r="G129" s="257" t="n">
+        <v>130</v>
+      </c>
+      <c r="H129" s="258">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B129,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B129+1))</f>
+        <v>747.0</v>
+      </c>
+      <c r="I129" s="259">
+        <f>IFERROR(F129-H129,0)</f>
+        <v>1673.0</v>
+      </c>
+      <c r="J129" s="260">
+        <f>IFERROR(I129/F129,0)</f>
+        <v>0.691322</v>
+      </c>
+      <c r="K129" s="254" t="n"/>
+      <c r="L129" s="261" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
+      <c r="M129" s="291" t="n"/>
+      <c r="N129" s="292" t="n"/>
+      <c r="O129" s="293" t="n"/>
+      <c r="P129" s="294" t="n"/>
+      <c r="Q129" s="292" t="n"/>
+      <c r="R129" s="443">
+        <f>IFERROR(D129*$T$7,0)</f>
+        <v>54.81</v>
+      </c>
+      <c r="S129" s="292" t="n"/>
+      <c r="T129" s="292" t="n"/>
+      <c r="U129" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="V129" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="W129" s="292" t="n"/>
+      <c r="X129" s="292" t="n"/>
+      <c r="Y129" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z129" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA129" s="292" t="n"/>
+      <c r="AB129" s="292" t="n"/>
     </row>
     <row r="130" ht="16.5" customHeight="1" s="331">
-      <c r="B130" s="34" t="n"/>
-      <c r="C130" s="35" t="n"/>
-      <c r="D130" s="36" t="n"/>
-      <c r="E130" s="37" t="n"/>
-      <c r="F130" s="38" t="n"/>
-      <c r="G130" s="39" t="n"/>
-      <c r="H130" s="40" t="n"/>
-      <c r="I130" s="41" t="n"/>
-      <c r="J130" s="42" t="n"/>
-      <c r="K130" s="43" t="n"/>
-      <c r="L130" s="9" t="n"/>
-      <c r="M130" s="12" t="n"/>
-      <c r="N130" s="44" t="n"/>
-      <c r="O130" s="45" t="n"/>
-      <c r="P130" s="46" t="n"/>
-      <c r="Q130" s="44" t="n"/>
-      <c r="R130" s="44" t="n"/>
-      <c r="S130" s="44" t="n"/>
-      <c r="T130" s="44" t="n"/>
-      <c r="U130" s="44" t="n"/>
-      <c r="V130" s="44" t="n"/>
-      <c r="W130" s="44" t="n"/>
-      <c r="X130" s="44" t="n"/>
-      <c r="Y130" s="44" t="n"/>
-      <c r="Z130" s="44" t="n"/>
-      <c r="AA130" s="44" t="n"/>
-      <c r="AB130" s="44" t="n"/>
+      <c r="B130" s="427" t="n">
+        <v>46297</v>
+      </c>
+      <c r="C130" s="270" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D130" s="271" t="n">
+        <v>3420</v>
+      </c>
+      <c r="E130" s="37" t="n">
+        <v>2915</v>
+      </c>
+      <c r="F130" s="38">
+        <f>IFERROR(D130+E130+G130+U130+Y130,0)</f>
+        <v>6335.0</v>
+      </c>
+      <c r="G130" s="272" t="n">
+        <v>0</v>
+      </c>
+      <c r="H130" s="273">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B130,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B130+1))</f>
+        <v>5818.0</v>
+      </c>
+      <c r="I130" s="274">
+        <f>IFERROR(F130-H130,0)</f>
+        <v>517.0</v>
+      </c>
+      <c r="J130" s="275">
+        <f>IFERROR(I130/F130,0)</f>
+        <v>0.08161</v>
+      </c>
+      <c r="K130" s="250" t="n"/>
+      <c r="L130" s="276" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
+      <c r="M130" s="323" t="n"/>
+      <c r="N130" s="324" t="n"/>
+      <c r="O130" s="325" t="n"/>
+      <c r="P130" s="326" t="n"/>
+      <c r="Q130" s="324" t="n"/>
+      <c r="R130" s="428">
+        <f>IFERROR(D130*$T$7,0)</f>
+        <v>138.85</v>
+      </c>
+      <c r="S130" s="324" t="n"/>
+      <c r="T130" s="324" t="n"/>
+      <c r="U130" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="V130" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="W130" s="324" t="n"/>
+      <c r="X130" s="324" t="n"/>
+      <c r="Y130" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z130" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA130" s="324" t="n"/>
+      <c r="AB130" s="324" t="n"/>
     </row>
     <row r="131" ht="16.5" customHeight="1" s="331">
-      <c r="B131" s="34" t="n"/>
-      <c r="C131" s="47" t="n"/>
-      <c r="D131" s="48" t="n"/>
-      <c r="E131" s="49" t="n"/>
-      <c r="F131" s="50" t="n"/>
-      <c r="G131" s="51" t="n"/>
-      <c r="H131" s="52" t="n"/>
-      <c r="I131" s="53" t="n"/>
-      <c r="J131" s="54" t="n"/>
-      <c r="K131" s="55" t="n"/>
-      <c r="L131" s="18" t="n"/>
-      <c r="M131" s="21" t="n"/>
-      <c r="N131" s="56" t="n"/>
-      <c r="O131" s="57" t="n"/>
-      <c r="P131" s="58" t="n"/>
-      <c r="Q131" s="56" t="n"/>
-      <c r="R131" s="56" t="n"/>
-      <c r="S131" s="56" t="n"/>
-      <c r="T131" s="56" t="n"/>
-      <c r="U131" s="56" t="n"/>
-      <c r="V131" s="56" t="n"/>
-      <c r="W131" s="56" t="n"/>
-      <c r="X131" s="56" t="n"/>
-      <c r="Y131" s="56" t="n"/>
-      <c r="Z131" s="56" t="n"/>
-      <c r="AA131" s="56" t="n"/>
-      <c r="AB131" s="56" t="n"/>
+      <c r="B131" s="427" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C131" s="255" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D131" s="256" t="n">
+        <v>2042</v>
+      </c>
+      <c r="E131" s="49" t="n">
+        <v>2573</v>
+      </c>
+      <c r="F131" s="50">
+        <f>IFERROR(D131+E131+G131+U131+Y131,0)</f>
+        <v>5580.0</v>
+      </c>
+      <c r="G131" s="257" t="n">
+        <v>965</v>
+      </c>
+      <c r="H131" s="258">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B131,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B131+1))</f>
+        <v>29005.68</v>
+      </c>
+      <c r="I131" s="259">
+        <f>IFERROR(F131-H131,0)</f>
+        <v>-23425.68</v>
+      </c>
+      <c r="J131" s="260">
+        <f>IFERROR(I131/F131,0)</f>
+        <v>-4.198151</v>
+      </c>
+      <c r="K131" s="254" t="n"/>
+      <c r="L131" s="261" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
+      <c r="M131" s="291" t="n"/>
+      <c r="N131" s="292" t="n"/>
+      <c r="O131" s="293" t="n"/>
+      <c r="P131" s="294" t="n"/>
+      <c r="Q131" s="292" t="n"/>
+      <c r="R131" s="443">
+        <f>IFERROR(D131*$T$7,0)</f>
+        <v>82.91</v>
+      </c>
+      <c r="S131" s="292" t="n"/>
+      <c r="T131" s="292" t="n"/>
+      <c r="U131" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="V131" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="W131" s="292" t="n"/>
+      <c r="X131" s="292" t="n"/>
+      <c r="Y131" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z131" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA131" s="292" t="n"/>
+      <c r="AB131" s="292" t="n"/>
     </row>
     <row r="132" ht="16.5" customHeight="1" s="331">
       <c r="B132" s="34" t="n"/>
@@ -26141,9 +26425,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="B5:P5"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="I2:P2"/>
+    <mergeCell ref="B5:P5"/>
     <mergeCell ref="A3:P3"/>
   </mergeCells>
   <conditionalFormatting sqref="I8:I372">
@@ -26166,7 +26450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J820"/>
+  <dimension ref="A1:J832"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="4" customWidth="1" style="331" min="1" max="1"/>
@@ -59752,7 +60036,7 @@
       </c>
       <c r="G793" s="300" t="inlineStr">
         <is>
-          <t>Capital</t>
+          <t>Restaurant</t>
         </is>
       </c>
       <c r="H793" s="300" t="inlineStr">
@@ -59767,7 +60051,7 @@
       </c>
       <c r="J793" s="423" t="inlineStr">
         <is>
-          <t>Impuestos Jun-Ago 2026 pagados con capital - reserva cuenta empresa</t>
+          <t>Impuestos Jun-Ago 2026 pagados desde cuenta empresa</t>
         </is>
       </c>
     </row>
@@ -59795,7 +60079,7 @@
       </c>
       <c r="G794" s="300" t="inlineStr">
         <is>
-          <t>Capital</t>
+          <t>Restaurant</t>
         </is>
       </c>
       <c r="H794" s="300" t="inlineStr">
@@ -59810,7 +60094,7 @@
       </c>
       <c r="J794" s="423" t="inlineStr">
         <is>
-          <t>Honorarios contables pagados con capital - reserva cuenta empresa</t>
+          <t>Honorarios contables pagados desde cuenta empresa</t>
         </is>
       </c>
     </row>
@@ -60929,6 +61213,522 @@
       <c r="J820" s="423" t="inlineStr">
         <is>
           <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="B821" s="429" t="n">
+        <v>46296</v>
+      </c>
+      <c r="C821" s="297" t="inlineStr">
+        <is>
+          <t>Pollo</t>
+        </is>
+      </c>
+      <c r="D821" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E821" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat</t>
+        </is>
+      </c>
+      <c r="F821" s="299" t="n">
+        <v>174</v>
+      </c>
+      <c r="G821" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H821" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I821" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J821" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="B822" s="429" t="n">
+        <v>46296</v>
+      </c>
+      <c r="C822" s="297" t="inlineStr">
+        <is>
+          <t>Oxxo Arrox</t>
+        </is>
+      </c>
+      <c r="D822" s="298" t="inlineStr">
+        <is>
+          <t>OXXO</t>
+        </is>
+      </c>
+      <c r="E822" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Pantry</t>
+        </is>
+      </c>
+      <c r="F822" s="299" t="n">
+        <v>130</v>
+      </c>
+      <c r="G822" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H822" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I822" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J822" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="B823" s="429" t="n">
+        <v>46296</v>
+      </c>
+      <c r="C823" s="297" t="inlineStr">
+        <is>
+          <t>Chedraui</t>
+        </is>
+      </c>
+      <c r="D823" s="298" t="inlineStr">
+        <is>
+          <t>Chedraui</t>
+        </is>
+      </c>
+      <c r="E823" s="297" t="inlineStr">
+        <is>
+          <t>Supermarket/General</t>
+        </is>
+      </c>
+      <c r="F823" s="299" t="n">
+        <v>443</v>
+      </c>
+      <c r="G823" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H823" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I823" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J823" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="B824" s="429" t="n">
+        <v>46297</v>
+      </c>
+      <c r="C824" s="297" t="inlineStr">
+        <is>
+          <t>Pescado</t>
+        </is>
+      </c>
+      <c r="D824" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E824" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat &amp; Fish</t>
+        </is>
+      </c>
+      <c r="F824" s="299" t="n">
+        <v>297</v>
+      </c>
+      <c r="G824" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H824" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I824" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J824" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="B825" s="429" t="n">
+        <v>46297</v>
+      </c>
+      <c r="C825" s="297" t="inlineStr">
+        <is>
+          <t>Duvi - salary</t>
+        </is>
+      </c>
+      <c r="D825" s="298" t="inlineStr">
+        <is>
+          <t>Payroll</t>
+        </is>
+      </c>
+      <c r="E825" s="297" t="inlineStr">
+        <is>
+          <t>Staff - Salary</t>
+        </is>
+      </c>
+      <c r="F825" s="299" t="n">
+        <v>875</v>
+      </c>
+      <c r="G825" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H825" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I825" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J825" s="423" t="inlineStr">
+        <is>
+          <t>Weekly salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="B826" s="429" t="n">
+        <v>46297</v>
+      </c>
+      <c r="C826" s="297" t="inlineStr">
+        <is>
+          <t>Josias - salary</t>
+        </is>
+      </c>
+      <c r="D826" s="298" t="inlineStr">
+        <is>
+          <t>Payroll</t>
+        </is>
+      </c>
+      <c r="E826" s="297" t="inlineStr">
+        <is>
+          <t>Staff - Salary</t>
+        </is>
+      </c>
+      <c r="F826" s="299" t="n">
+        <v>1096</v>
+      </c>
+      <c r="G826" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H826" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I826" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J826" s="423" t="inlineStr">
+        <is>
+          <t>Weekly salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="B827" s="429" t="n">
+        <v>46297</v>
+      </c>
+      <c r="C827" s="297" t="inlineStr">
+        <is>
+          <t>Jhon - salary</t>
+        </is>
+      </c>
+      <c r="D827" s="298" t="inlineStr">
+        <is>
+          <t>Payroll</t>
+        </is>
+      </c>
+      <c r="E827" s="297" t="inlineStr">
+        <is>
+          <t>Staff - Salary</t>
+        </is>
+      </c>
+      <c r="F827" s="299" t="n">
+        <v>3550</v>
+      </c>
+      <c r="G827" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H827" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I827" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J827" s="423" t="inlineStr">
+        <is>
+          <t>Weekly salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="B828" s="429" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C828" s="297" t="inlineStr">
+        <is>
+          <t>Vegetables</t>
+        </is>
+      </c>
+      <c r="D828" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E828" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Vegetables</t>
+        </is>
+      </c>
+      <c r="F828" s="299" t="n">
+        <v>1228</v>
+      </c>
+      <c r="G828" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H828" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I828" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J828" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="B829" s="429" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C829" s="297" t="inlineStr">
+        <is>
+          <t>Chedraui</t>
+        </is>
+      </c>
+      <c r="D829" s="298" t="inlineStr">
+        <is>
+          <t>Chedraui</t>
+        </is>
+      </c>
+      <c r="E829" s="297" t="inlineStr">
+        <is>
+          <t>Supermarket/General</t>
+        </is>
+      </c>
+      <c r="F829" s="299" t="n">
+        <v>89</v>
+      </c>
+      <c r="G829" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H829" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I829" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J829" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="B830" s="429" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C830" s="297" t="inlineStr">
+        <is>
+          <t>Electricity Bill</t>
+        </is>
+      </c>
+      <c r="D830" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E830" s="297" t="inlineStr">
+        <is>
+          <t>Utilities/Electricity</t>
+        </is>
+      </c>
+      <c r="F830" s="299" t="n">
+        <v>7710</v>
+      </c>
+      <c r="G830" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H830" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I830" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J830" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="B831" s="429" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C831" s="297" t="inlineStr">
+        <is>
+          <t>Rent</t>
+        </is>
+      </c>
+      <c r="D831" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E831" s="297" t="inlineStr">
+        <is>
+          <t>Rent</t>
+        </is>
+      </c>
+      <c r="F831" s="299" t="n">
+        <v>19066.68</v>
+      </c>
+      <c r="G831" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H831" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I831" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J831" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="B832" s="429" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C832" s="297" t="inlineStr">
+        <is>
+          <t>Pollo</t>
+        </is>
+      </c>
+      <c r="D832" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E832" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat</t>
+        </is>
+      </c>
+      <c r="F832" s="299" t="n">
+        <v>912</v>
+      </c>
+      <c r="G832" s="300" t="inlineStr">
+        <is>
+          <t>Lohith</t>
+        </is>
+      </c>
+      <c r="H832" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I832" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J832" s="423" t="inlineStr">
+        <is>
+          <t>Pagado por Lohith (bolsillo); reembolsable via Owner Ledger</t>
         </is>
       </c>
     </row>
@@ -71026,7 +71826,7 @@
     <col width="15" customWidth="1" style="331" min="4" max="4"/>
     <col width="15" customWidth="1" style="331" min="5" max="5"/>
     <col width="15" customWidth="1" style="331" min="6" max="14"/>
-    <col width="9" customWidth="1" style="331" min="7" max="7"/>
+    <col width="15" customWidth="1" style="331" min="7" max="7"/>
     <col width="9" customWidth="1" style="331" min="8" max="8"/>
     <col width="9" customWidth="1" style="331" min="9" max="9"/>
     <col width="9" customWidth="1" style="331" min="10" max="10"/>
@@ -71037,17 +71837,17 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" s="331">
-      <c r="A1" s="431" t="inlineStr">
+      <c r="A1" s="441" t="inlineStr">
         <is>
           <t>LOKA — MONTHLY P&amp;L   (live formulas — auto-updates from Daily Log &amp; Expenses)</t>
         </is>
       </c>
-      <c r="B1" s="432" t="n"/>
-      <c r="C1" s="432" t="n"/>
-      <c r="D1" s="432" t="n"/>
-      <c r="E1" s="432" t="n"/>
-      <c r="F1" s="432" t="n"/>
-      <c r="G1" s="433" t="n"/>
+      <c r="B1" s="423" t="n"/>
+      <c r="C1" s="423" t="n"/>
+      <c r="D1" s="423" t="n"/>
+      <c r="E1" s="423" t="n"/>
+      <c r="F1" s="423" t="n"/>
+      <c r="G1" s="423" t="n"/>
       <c r="H1" s="433" t="n"/>
       <c r="I1" s="433" t="n"/>
       <c r="J1" s="433" t="n"/>
@@ -71099,7 +71899,11 @@
           <t>Sep 2026</t>
         </is>
       </c>
-      <c r="G3" s="433" t="n"/>
+      <c r="G3" s="435" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
       <c r="H3" s="433" t="n"/>
       <c r="I3" s="433" t="n"/>
       <c r="J3" s="433" t="n"/>
@@ -71132,7 +71936,10 @@
         <f>SUMIFS('📅 Daily Log'!$F$8:$F$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G4" s="433" t="n"/>
+      <c r="G4" s="437">
+        <f>SUMIFS('📅 Daily Log'!$F$8:$F$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H4" s="433" t="n"/>
       <c r="I4" s="433" t="n"/>
       <c r="J4" s="433" t="n"/>
@@ -71165,7 +71972,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G5" s="433" t="n"/>
+      <c r="G5" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H5" s="433" t="n"/>
       <c r="I5" s="433" t="n"/>
       <c r="J5" s="433" t="n"/>
@@ -71198,7 +72008,10 @@
         <f>F4-F5</f>
         <v/>
       </c>
-      <c r="G6" s="433" t="n"/>
+      <c r="G6" s="438">
+        <f>G4-G5</f>
+        <v/>
+      </c>
       <c r="H6" s="433" t="n"/>
       <c r="I6" s="433" t="n"/>
       <c r="J6" s="433" t="n"/>
@@ -71231,7 +72044,10 @@
         <f>COUNTIFS('📅 Daily Log'!$F$8:$F$5000,"&gt;0",'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G7" s="433" t="n"/>
+      <c r="G7" s="440">
+        <f>COUNTIFS('📅 Daily Log'!$F$8:$F$5000,"&gt;0",'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H7" s="433" t="n"/>
       <c r="I7" s="433" t="n"/>
       <c r="J7" s="433" t="n"/>
@@ -71264,7 +72080,10 @@
         <f>IFERROR(F4/F7,0)</f>
         <v/>
       </c>
-      <c r="G8" s="433" t="n"/>
+      <c r="G8" s="437">
+        <f>IFERROR(G4/G7,0)</f>
+        <v/>
+      </c>
       <c r="H8" s="433" t="n"/>
       <c r="I8" s="433" t="n"/>
       <c r="J8" s="433" t="n"/>
@@ -71316,7 +72135,11 @@
           <t>Sep 2026</t>
         </is>
       </c>
-      <c r="G10" s="433" t="n"/>
+      <c r="G10" s="435" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
       <c r="H10" s="433" t="n"/>
       <c r="I10" s="433" t="n"/>
       <c r="J10" s="433" t="n"/>
@@ -71349,7 +72172,10 @@
         <f>SUMIFS('📅 Daily Log'!$D$8:$D$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))+SUMIFS('📅 Daily Log'!$U$8:$U$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))+SUMIFS('📅 Daily Log'!$Y$8:$Y$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G11" s="433" t="n"/>
+      <c r="G11" s="437">
+        <f>SUMIFS('📅 Daily Log'!$D$8:$D$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))+SUMIFS('📅 Daily Log'!$U$8:$U$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))+SUMIFS('📅 Daily Log'!$Y$8:$Y$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H11" s="433" t="n"/>
       <c r="I11" s="433" t="n"/>
       <c r="J11" s="433" t="n"/>
@@ -71382,7 +72208,10 @@
         <f>SUMIFS('📅 Daily Log'!$E$8:$E$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G12" s="433" t="n"/>
+      <c r="G12" s="437">
+        <f>SUMIFS('📅 Daily Log'!$E$8:$E$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H12" s="433" t="n"/>
       <c r="I12" s="433" t="n"/>
       <c r="J12" s="433" t="n"/>
@@ -71415,7 +72244,10 @@
         <f>SUMIFS('📅 Daily Log'!$G$8:$G$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G13" s="433" t="n"/>
+      <c r="G13" s="437">
+        <f>SUMIFS('📅 Daily Log'!$G$8:$G$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H13" s="433" t="n"/>
       <c r="I13" s="433" t="n"/>
       <c r="J13" s="433" t="n"/>
@@ -71448,7 +72280,10 @@
         <f>F11+F12+F13</f>
         <v/>
       </c>
-      <c r="G14" s="433" t="n"/>
+      <c r="G14" s="438">
+        <f>G11+G12+G13</f>
+        <v/>
+      </c>
       <c r="H14" s="433" t="n"/>
       <c r="I14" s="433" t="n"/>
       <c r="J14" s="433" t="n"/>
@@ -71500,7 +72335,11 @@
           <t>Sep 2026</t>
         </is>
       </c>
-      <c r="G16" s="433" t="n"/>
+      <c r="G16" s="435" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
       <c r="H16" s="433" t="n"/>
       <c r="I16" s="433" t="n"/>
       <c r="J16" s="433" t="n"/>
@@ -71533,7 +72372,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A17,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G17" s="433" t="n"/>
+      <c r="G17" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A17,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H17" s="433" t="n"/>
       <c r="I17" s="433" t="n"/>
       <c r="J17" s="433" t="n"/>
@@ -71566,7 +72408,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A18,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G18" s="433" t="n"/>
+      <c r="G18" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A18,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H18" s="433" t="n"/>
       <c r="I18" s="433" t="n"/>
       <c r="J18" s="433" t="n"/>
@@ -71599,7 +72444,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A19,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G19" s="433" t="n"/>
+      <c r="G19" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A19,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H19" s="433" t="n"/>
       <c r="I19" s="433" t="n"/>
       <c r="J19" s="433" t="n"/>
@@ -71632,7 +72480,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A20,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G20" s="433" t="n"/>
+      <c r="G20" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A20,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H20" s="433" t="n"/>
       <c r="I20" s="433" t="n"/>
       <c r="J20" s="433" t="n"/>
@@ -71665,7 +72516,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A21,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G21" s="433" t="n"/>
+      <c r="G21" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A21,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H21" s="433" t="n"/>
       <c r="I21" s="433" t="n"/>
       <c r="J21" s="433" t="n"/>
@@ -71675,7 +72529,7 @@
     <row r="22">
       <c r="A22" s="439" t="inlineStr">
         <is>
-          <t>Taxes</t>
+          <t>Utilities/Electricity</t>
         </is>
       </c>
       <c r="B22" s="437">
@@ -71698,7 +72552,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A22,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G22" s="433" t="n"/>
+      <c r="G22" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A22,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H22" s="433" t="n"/>
       <c r="I22" s="433" t="n"/>
       <c r="J22" s="433" t="n"/>
@@ -71708,7 +72565,7 @@
     <row r="23">
       <c r="A23" s="439" t="inlineStr">
         <is>
-          <t>Ingredients - Pantry</t>
+          <t>Taxes</t>
         </is>
       </c>
       <c r="B23" s="437">
@@ -71731,7 +72588,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A23,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G23" s="433" t="n"/>
+      <c r="G23" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A23,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H23" s="433" t="n"/>
       <c r="I23" s="433" t="n"/>
       <c r="J23" s="433" t="n"/>
@@ -71741,7 +72601,7 @@
     <row r="24">
       <c r="A24" s="439" t="inlineStr">
         <is>
-          <t>Ingredients - Bread</t>
+          <t>Ingredients - Pantry</t>
         </is>
       </c>
       <c r="B24" s="437">
@@ -71764,7 +72624,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A24,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G24" s="433" t="n"/>
+      <c r="G24" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A24,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H24" s="433" t="n"/>
       <c r="I24" s="433" t="n"/>
       <c r="J24" s="433" t="n"/>
@@ -71774,7 +72637,7 @@
     <row r="25">
       <c r="A25" s="439" t="inlineStr">
         <is>
-          <t>Ingredients - Beverages</t>
+          <t>Ingredients - Bread</t>
         </is>
       </c>
       <c r="B25" s="437">
@@ -71797,7 +72660,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A25,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G25" s="433" t="n"/>
+      <c r="G25" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A25,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H25" s="433" t="n"/>
       <c r="I25" s="433" t="n"/>
       <c r="J25" s="433" t="n"/>
@@ -71807,7 +72673,7 @@
     <row r="26">
       <c r="A26" s="439" t="inlineStr">
         <is>
-          <t>Ingredients - Dairy</t>
+          <t>Ingredients - Beverages</t>
         </is>
       </c>
       <c r="B26" s="437">
@@ -71830,7 +72696,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A26,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G26" s="433" t="n"/>
+      <c r="G26" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A26,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H26" s="433" t="n"/>
       <c r="I26" s="433" t="n"/>
       <c r="J26" s="433" t="n"/>
@@ -71840,7 +72709,7 @@
     <row r="27">
       <c r="A27" s="439" t="inlineStr">
         <is>
-          <t>Utilities/Electricity</t>
+          <t>Ingredients - Dairy</t>
         </is>
       </c>
       <c r="B27" s="437">
@@ -71863,7 +72732,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A27,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G27" s="433" t="n"/>
+      <c r="G27" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A27,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H27" s="433" t="n"/>
       <c r="I27" s="433" t="n"/>
       <c r="J27" s="433" t="n"/>
@@ -71873,7 +72745,7 @@
     <row r="28">
       <c r="A28" s="439" t="inlineStr">
         <is>
-          <t>Supplies/Other</t>
+          <t>Ingredients - Meat &amp; Fish</t>
         </is>
       </c>
       <c r="B28" s="437">
@@ -71896,7 +72768,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A28,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G28" s="433" t="n"/>
+      <c r="G28" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A28,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H28" s="433" t="n"/>
       <c r="I28" s="433" t="n"/>
       <c r="J28" s="433" t="n"/>
@@ -71906,7 +72781,7 @@
     <row r="29">
       <c r="A29" s="439" t="inlineStr">
         <is>
-          <t>Ingredients - Meat &amp; Fish</t>
+          <t>Supplies/Other</t>
         </is>
       </c>
       <c r="B29" s="437">
@@ -71929,7 +72804,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A29,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G29" s="433" t="n"/>
+      <c r="G29" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A29,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H29" s="433" t="n"/>
       <c r="I29" s="433" t="n"/>
       <c r="J29" s="433" t="n"/>
@@ -71962,7 +72840,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A30,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G30" s="433" t="n"/>
+      <c r="G30" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A30,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H30" s="433" t="n"/>
       <c r="I30" s="433" t="n"/>
       <c r="J30" s="433" t="n"/>
@@ -71995,7 +72876,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A31,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G31" s="433" t="n"/>
+      <c r="G31" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A31,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H31" s="433" t="n"/>
       <c r="I31" s="433" t="n"/>
       <c r="J31" s="433" t="n"/>
@@ -72028,7 +72912,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A32,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G32" s="433" t="n"/>
+      <c r="G32" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A32,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H32" s="433" t="n"/>
       <c r="I32" s="433" t="n"/>
       <c r="J32" s="433" t="n"/>
@@ -72061,7 +72948,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A33,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G33" s="433" t="n"/>
+      <c r="G33" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A33,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H33" s="433" t="n"/>
       <c r="I33" s="433" t="n"/>
       <c r="J33" s="433" t="n"/>
@@ -72094,7 +72984,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A34,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G34" s="433" t="n"/>
+      <c r="G34" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A34,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H34" s="433" t="n"/>
       <c r="I34" s="433" t="n"/>
       <c r="J34" s="433" t="n"/>
@@ -72127,7 +73020,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A35,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G35" s="433" t="n"/>
+      <c r="G35" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A35,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H35" s="433" t="n"/>
       <c r="I35" s="433" t="n"/>
       <c r="J35" s="433" t="n"/>
@@ -72160,7 +73056,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A36,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G36" s="433" t="n"/>
+      <c r="G36" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A36,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H36" s="433" t="n"/>
       <c r="I36" s="433" t="n"/>
       <c r="J36" s="433" t="n"/>
@@ -72193,7 +73092,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A37,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G37" s="433" t="n"/>
+      <c r="G37" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A37,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H37" s="433" t="n"/>
       <c r="I37" s="433" t="n"/>
       <c r="J37" s="433" t="n"/>
@@ -72226,7 +73128,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A38,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G38" s="433" t="n"/>
+      <c r="G38" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A38,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H38" s="433" t="n"/>
       <c r="I38" s="433" t="n"/>
       <c r="J38" s="433" t="n"/>
@@ -72259,7 +73164,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A39,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G39" s="433" t="n"/>
+      <c r="G39" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A39,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H39" s="433" t="n"/>
       <c r="I39" s="433" t="n"/>
       <c r="J39" s="433" t="n"/>
@@ -72292,7 +73200,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A40,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G40" s="433" t="n"/>
+      <c r="G40" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A40,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H40" s="433" t="n"/>
       <c r="I40" s="433" t="n"/>
       <c r="J40" s="433" t="n"/>
@@ -72325,7 +73236,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A41,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G41" s="433" t="n"/>
+      <c r="G41" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A41,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H41" s="433" t="n"/>
       <c r="I41" s="433" t="n"/>
       <c r="J41" s="433" t="n"/>
@@ -72358,7 +73272,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A42,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G42" s="433" t="n"/>
+      <c r="G42" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A42,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H42" s="433" t="n"/>
       <c r="I42" s="433" t="n"/>
       <c r="J42" s="433" t="n"/>
@@ -72391,7 +73308,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A43,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G43" s="433" t="n"/>
+      <c r="G43" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A43,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H43" s="433" t="n"/>
       <c r="I43" s="433" t="n"/>
       <c r="J43" s="433" t="n"/>
@@ -72424,7 +73344,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,9,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,10,1))</f>
         <v/>
       </c>
-      <c r="G44" s="433" t="n"/>
+      <c r="G44" s="438">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
       <c r="H44" s="433" t="n"/>
       <c r="I44" s="433" t="n"/>
       <c r="J44" s="433" t="n"/>
@@ -72457,7 +73380,10 @@
         <f>F4-F44</f>
         <v/>
       </c>
-      <c r="G45" s="433" t="n"/>
+      <c r="G45" s="438">
+        <f>G4-G44</f>
+        <v/>
+      </c>
       <c r="H45" s="433" t="n"/>
       <c r="I45" s="433" t="n"/>
       <c r="J45" s="433" t="n"/>
@@ -72676,7 +73602,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
LOKA 06-Oct-2026 | EOD | day 2026-10-06: rev $4,325 exp $5,081 net $-756 | bal vs capital $-20,767
Changed: LOKA_Restaurant_Manager.xlsx, dashboard.html, loka.py, today.txt
+ 2 backup/day file(s)
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -5871,7 +5871,7 @@
         </is>
       </c>
       <c r="C172" s="455" t="n">
-        <v>-19118.92</v>
+        <v>-20767.09</v>
       </c>
       <c r="E172" s="423" t="inlineStr">
         <is>
@@ -5886,7 +5886,7 @@
         </is>
       </c>
       <c r="C173" s="457" t="n">
-        <v>106815.08</v>
+        <v>105166.91</v>
       </c>
       <c r="E173" s="423" t="inlineStr">
         <is>
@@ -6057,7 +6057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H104"/>
+  <dimension ref="A1:H105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" style="331" min="1" max="1"/>
@@ -9419,30 +9419,63 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="430" t="inlineStr">
+      <c r="A104" s="430" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B104" s="232" t="inlineStr">
+        <is>
+          <t>Transfer-to-me (customer payment 06-Oct)</t>
+        </is>
+      </c>
+      <c r="C104" s="232" t="inlineStr">
+        <is>
+          <t>Transfer Received</t>
+        </is>
+      </c>
+      <c r="D104" s="232" t="n"/>
+      <c r="E104" s="233" t="n">
+        <v>840</v>
+      </c>
+      <c r="F104" s="233">
+        <f>IFERROR(F103+D104-E104,0)</f>
+        <v/>
+      </c>
+      <c r="G104" s="232" t="inlineStr">
+        <is>
+          <t>✅ Received</t>
+        </is>
+      </c>
+      <c r="H104" s="232" t="inlineStr">
+        <is>
+          <t>Customer paid Lohith personal acct</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="430" t="inlineStr">
         <is>
           <t>TOTALS &amp; CURRENT BALANCE</t>
         </is>
       </c>
-      <c r="B104" s="232" t="n"/>
-      <c r="C104" s="232" t="n"/>
-      <c r="D104" s="232">
-        <f>SUM(D4:D103)</f>
-        <v/>
-      </c>
-      <c r="E104" s="233">
-        <f>SUM(E4:E103)</f>
-        <v/>
-      </c>
-      <c r="F104" s="233">
-        <f>F103</f>
-        <v/>
-      </c>
-      <c r="G104" s="232">
-        <f>IF(F103&gt;0,"Restaurant owes Lohith $"&amp;TEXT(F103,"#,##0"),IF(F103&lt;0,"Lohith holds $"&amp;TEXT(ABS(F103),"#,##0"),"Zero balance"))</f>
-        <v/>
-      </c>
-      <c r="H104" s="232" t="n"/>
+      <c r="B105" s="232" t="n"/>
+      <c r="C105" s="232" t="n"/>
+      <c r="D105" s="232">
+        <f>SUM(D4:D104)</f>
+        <v/>
+      </c>
+      <c r="E105" s="233">
+        <f>SUM(E4:E104)</f>
+        <v/>
+      </c>
+      <c r="F105" s="233">
+        <f>F104</f>
+        <v/>
+      </c>
+      <c r="G105" s="232">
+        <f>IF(F104&gt;0,"Restaurant owes Lohith $"&amp;TEXT(F104,"#,##0"),IF(F104&lt;0,"Lohith holds $"&amp;TEXT(ABS(F104),"#,##0"),"Zero balance"))</f>
+        <v/>
+      </c>
+      <c r="H105" s="232" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -11276,45 +11309,45 @@
       <c r="E6" s="29" t="n"/>
       <c r="F6" s="30">
         <f>SUMIFS($D$8:$D$5000,$B$8:$B$5000,TODAY())+SUMIFS($E$8:$E$5000,$B$8:$B$5000,TODAY())+SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())+SUMIFS($U$8:$U$5000,$B$8:$B$5000,TODAY())+SUMIFS($Y$8:$Y$5000,$B$8:$B$5000,TODAY())</f>
-        <v>5580.0</v>
+        <v>4325.0</v>
       </c>
       <c r="G6" s="31">
         <f>SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())</f>
-        <v>965.0</v>
+        <v>840.0</v>
       </c>
       <c r="H6" s="28">
         <f>SUMIFS($H$8:$H$5000,$B$8:$B$5000,TODAY())</f>
-        <v>29005.68</v>
+        <v>5081.0</v>
       </c>
       <c r="I6" s="32">
         <f>F6-H6</f>
-        <v>-23425.68</v>
+        <v>-756.0</v>
       </c>
       <c r="J6">
         <f>IFERROR(I6/F6,0)</f>
-        <v>-4.198151</v>
+        <v>-0.174798</v>
       </c>
       <c r="K6" s="28" t="n"/>
       <c r="L6" s="31" t="n"/>
       <c r="M6" s="28">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>5580.0</v>
+        <v>9905.0</v>
       </c>
       <c r="N6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>5580.0</v>
+        <v>9905.0</v>
       </c>
       <c r="O6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),$B$8:$B$5000,"&lt;"&amp;DATE(YEAR(TODAY()),MONTH(TODAY())+1,1))</f>
-        <v>14335.0</v>
+        <v>18660.0</v>
       </c>
       <c r="P6">
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>29005.68</v>
+        <v>34086.68</v>
       </c>
       <c r="Q6">
         <f>M6-P6</f>
-        <v>-23425.68</v>
+        <v>-24181.68</v>
       </c>
     </row>
     <row r="7" ht="27.75" customHeight="1" s="331">
@@ -19435,33 +19468,72 @@
       <c r="AB131" s="292" t="n"/>
     </row>
     <row r="132" ht="16.5" customHeight="1" s="331">
-      <c r="B132" s="34" t="n"/>
-      <c r="C132" s="35" t="n"/>
-      <c r="D132" s="36" t="n"/>
-      <c r="E132" s="37" t="n"/>
-      <c r="F132" s="38" t="n"/>
-      <c r="G132" s="39" t="n"/>
-      <c r="H132" s="40" t="n"/>
-      <c r="I132" s="41" t="n"/>
-      <c r="J132" s="42" t="n"/>
-      <c r="K132" s="43" t="n"/>
-      <c r="L132" s="9" t="n"/>
-      <c r="M132" s="12" t="n"/>
-      <c r="N132" s="44" t="n"/>
-      <c r="O132" s="45" t="n"/>
-      <c r="P132" s="46" t="n"/>
-      <c r="Q132" s="44" t="n"/>
-      <c r="R132" s="44" t="n"/>
-      <c r="S132" s="44" t="n"/>
-      <c r="T132" s="44" t="n"/>
-      <c r="U132" s="44" t="n"/>
-      <c r="V132" s="44" t="n"/>
-      <c r="W132" s="44" t="n"/>
-      <c r="X132" s="44" t="n"/>
-      <c r="Y132" s="44" t="n"/>
-      <c r="Z132" s="44" t="n"/>
-      <c r="AA132" s="44" t="n"/>
-      <c r="AB132" s="44" t="n"/>
+      <c r="B132" s="427" t="n">
+        <v>46301</v>
+      </c>
+      <c r="C132" s="270" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D132" s="271" t="n">
+        <v>1285</v>
+      </c>
+      <c r="E132" s="37" t="n">
+        <v>2200</v>
+      </c>
+      <c r="F132" s="38">
+        <f>IFERROR(D132+E132+G132+U132+Y132,0)</f>
+        <v>4325.0</v>
+      </c>
+      <c r="G132" s="272" t="n">
+        <v>840</v>
+      </c>
+      <c r="H132" s="273">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B132,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B132+1))</f>
+        <v>5081.0</v>
+      </c>
+      <c r="I132" s="274">
+        <f>IFERROR(F132-H132,0)</f>
+        <v>-756.0</v>
+      </c>
+      <c r="J132" s="275">
+        <f>IFERROR(I132/F132,0)</f>
+        <v>-0.174798</v>
+      </c>
+      <c r="K132" s="250" t="n"/>
+      <c r="L132" s="276" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
+      <c r="M132" s="323" t="n"/>
+      <c r="N132" s="324" t="n"/>
+      <c r="O132" s="325" t="n"/>
+      <c r="P132" s="326" t="n"/>
+      <c r="Q132" s="324" t="n"/>
+      <c r="R132" s="428">
+        <f>IFERROR(D132*$T$7,0)</f>
+        <v>52.17</v>
+      </c>
+      <c r="S132" s="324" t="n"/>
+      <c r="T132" s="324" t="n"/>
+      <c r="U132" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="V132" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="W132" s="324" t="n"/>
+      <c r="X132" s="324" t="n"/>
+      <c r="Y132" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z132" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA132" s="324" t="n"/>
+      <c r="AB132" s="324" t="n"/>
     </row>
     <row r="133" ht="16.5" customHeight="1" s="331">
       <c r="B133" s="34" t="n"/>
@@ -26425,9 +26497,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="I2:P2"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="B5:P5"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="I2:P2"/>
     <mergeCell ref="A3:P3"/>
   </mergeCells>
   <conditionalFormatting sqref="I8:I372">
@@ -26450,7 +26522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J832"/>
+  <dimension ref="A1:J840"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="4" customWidth="1" style="331" min="1" max="1"/>
@@ -61729,6 +61801,350 @@
       <c r="J832" s="423" t="inlineStr">
         <is>
           <t>Pagado por Lohith (bolsillo); reembolsable via Owner Ledger</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="B833" s="429" t="n">
+        <v>46301</v>
+      </c>
+      <c r="C833" s="297" t="inlineStr">
+        <is>
+          <t>Chedraui</t>
+        </is>
+      </c>
+      <c r="D833" s="298" t="inlineStr">
+        <is>
+          <t>Chedraui</t>
+        </is>
+      </c>
+      <c r="E833" s="297" t="inlineStr">
+        <is>
+          <t>Supermarket/General</t>
+        </is>
+      </c>
+      <c r="F833" s="299" t="n">
+        <v>49</v>
+      </c>
+      <c r="G833" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H833" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I833" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J833" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="B834" s="429" t="n">
+        <v>46301</v>
+      </c>
+      <c r="C834" s="297" t="inlineStr">
+        <is>
+          <t>Oxxo panela</t>
+        </is>
+      </c>
+      <c r="D834" s="298" t="inlineStr">
+        <is>
+          <t>OXXO</t>
+        </is>
+      </c>
+      <c r="E834" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Dairy</t>
+        </is>
+      </c>
+      <c r="F834" s="299" t="n">
+        <v>45</v>
+      </c>
+      <c r="G834" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H834" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I834" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J834" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="B835" s="429" t="n">
+        <v>46301</v>
+      </c>
+      <c r="C835" s="297" t="inlineStr">
+        <is>
+          <t>Pan</t>
+        </is>
+      </c>
+      <c r="D835" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E835" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Bread</t>
+        </is>
+      </c>
+      <c r="F835" s="299" t="n">
+        <v>25</v>
+      </c>
+      <c r="G835" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H835" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I835" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J835" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="B836" s="429" t="n">
+        <v>46301</v>
+      </c>
+      <c r="C836" s="297" t="inlineStr">
+        <is>
+          <t>Carne</t>
+        </is>
+      </c>
+      <c r="D836" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E836" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat</t>
+        </is>
+      </c>
+      <c r="F836" s="299" t="n">
+        <v>1056</v>
+      </c>
+      <c r="G836" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H836" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I836" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J836" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="B837" s="429" t="n">
+        <v>46301</v>
+      </c>
+      <c r="C837" s="297" t="inlineStr">
+        <is>
+          <t>Sams club</t>
+        </is>
+      </c>
+      <c r="D837" s="298" t="inlineStr">
+        <is>
+          <t>Sam's Club</t>
+        </is>
+      </c>
+      <c r="E837" s="297" t="inlineStr">
+        <is>
+          <t>Supermarket/General</t>
+        </is>
+      </c>
+      <c r="F837" s="299" t="n">
+        <v>1909</v>
+      </c>
+      <c r="G837" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H837" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I837" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J837" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="B838" s="429" t="n">
+        <v>46301</v>
+      </c>
+      <c r="C838" s="297" t="inlineStr">
+        <is>
+          <t>guimar</t>
+        </is>
+      </c>
+      <c r="D838" s="298" t="inlineStr">
+        <is>
+          <t>Guimar Polietilenos</t>
+        </is>
+      </c>
+      <c r="E838" s="297" t="inlineStr">
+        <is>
+          <t>Packaging/Disposables</t>
+        </is>
+      </c>
+      <c r="F838" s="299" t="n">
+        <v>604</v>
+      </c>
+      <c r="G838" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H838" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I838" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J838" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="B839" s="429" t="n">
+        <v>46301</v>
+      </c>
+      <c r="C839" s="297" t="inlineStr">
+        <is>
+          <t>Carne</t>
+        </is>
+      </c>
+      <c r="D839" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E839" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat</t>
+        </is>
+      </c>
+      <c r="F839" s="299" t="n">
+        <v>583</v>
+      </c>
+      <c r="G839" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H839" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I839" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J839" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="B840" s="429" t="n">
+        <v>46301</v>
+      </c>
+      <c r="C840" s="297" t="inlineStr">
+        <is>
+          <t>soft app</t>
+        </is>
+      </c>
+      <c r="D840" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E840" s="297" t="inlineStr">
+        <is>
+          <t>Software/Subscription</t>
+        </is>
+      </c>
+      <c r="F840" s="299" t="n">
+        <v>810</v>
+      </c>
+      <c r="G840" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H840" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I840" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J840" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
         </is>
       </c>
     </row>
@@ -73033,7 +73449,7 @@
     <row r="36">
       <c r="A36" s="439" t="inlineStr">
         <is>
-          <t>Utilities/Internet</t>
+          <t>Software/Subscription</t>
         </is>
       </c>
       <c r="B36" s="437">
@@ -73069,7 +73485,7 @@
     <row r="37">
       <c r="A37" s="439" t="inlineStr">
         <is>
-          <t>Office Supplies</t>
+          <t>Utilities/Internet</t>
         </is>
       </c>
       <c r="B37" s="437">
@@ -73105,7 +73521,7 @@
     <row r="38">
       <c r="A38" s="439" t="inlineStr">
         <is>
-          <t>Ingredients - Other</t>
+          <t>Office Supplies</t>
         </is>
       </c>
       <c r="B38" s="437">
@@ -73141,7 +73557,7 @@
     <row r="39">
       <c r="A39" s="439" t="inlineStr">
         <is>
-          <t>Software/Subscription</t>
+          <t>Ingredients - Other</t>
         </is>
       </c>
       <c r="B39" s="437">

</xml_diff>

<commit_message>
LOKA 12-Oct-2026 | EOD | day 2026-10-07: rev $1,455 exp $1,085 net $370 | bal vs capital $-20,412
Changed: LOKA_Restaurant_Manager.xlsx, dashboard.html, today.txt
+ 3 backup/day file(s)
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -5871,7 +5871,7 @@
         </is>
       </c>
       <c r="C172" s="455" t="n">
-        <v>-20767.09</v>
+        <v>-20411.71</v>
       </c>
       <c r="E172" s="423" t="inlineStr">
         <is>
@@ -5886,7 +5886,7 @@
         </is>
       </c>
       <c r="C173" s="457" t="n">
-        <v>105166.91</v>
+        <v>105522.29</v>
       </c>
       <c r="E173" s="423" t="inlineStr">
         <is>
@@ -11309,45 +11309,45 @@
       <c r="E6" s="29" t="n"/>
       <c r="F6" s="30">
         <f>SUMIFS($D$8:$D$5000,$B$8:$B$5000,TODAY())+SUMIFS($E$8:$E$5000,$B$8:$B$5000,TODAY())+SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())+SUMIFS($U$8:$U$5000,$B$8:$B$5000,TODAY())+SUMIFS($Y$8:$Y$5000,$B$8:$B$5000,TODAY())</f>
-        <v>4325.0</v>
+        <v>1455.0</v>
       </c>
       <c r="G6" s="31">
         <f>SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())</f>
-        <v>840.0</v>
+        <v>0.0</v>
       </c>
       <c r="H6" s="28">
         <f>SUMIFS($H$8:$H$5000,$B$8:$B$5000,TODAY())</f>
-        <v>5081.0</v>
+        <v>1085.0</v>
       </c>
       <c r="I6" s="32">
         <f>F6-H6</f>
-        <v>-756.0</v>
+        <v>370.0</v>
       </c>
       <c r="J6">
         <f>IFERROR(I6/F6,0)</f>
-        <v>-0.174798</v>
+        <v>0.254296</v>
       </c>
       <c r="K6" s="28" t="n"/>
       <c r="L6" s="31" t="n"/>
       <c r="M6" s="28">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>9905.0</v>
+        <v>11360.0</v>
       </c>
       <c r="N6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>9905.0</v>
+        <v>11360.0</v>
       </c>
       <c r="O6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),$B$8:$B$5000,"&lt;"&amp;DATE(YEAR(TODAY()),MONTH(TODAY())+1,1))</f>
-        <v>18660.0</v>
+        <v>20115.0</v>
       </c>
       <c r="P6">
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>34086.68</v>
+        <v>35171.68</v>
       </c>
       <c r="Q6">
         <f>M6-P6</f>
-        <v>-24181.68</v>
+        <v>-23811.68</v>
       </c>
     </row>
     <row r="7" ht="27.75" customHeight="1" s="331">
@@ -19536,33 +19536,72 @@
       <c r="AB132" s="324" t="n"/>
     </row>
     <row r="133" ht="16.5" customHeight="1" s="331">
-      <c r="B133" s="34" t="n"/>
-      <c r="C133" s="47" t="n"/>
-      <c r="D133" s="48" t="n"/>
-      <c r="E133" s="49" t="n"/>
-      <c r="F133" s="50" t="n"/>
-      <c r="G133" s="51" t="n"/>
-      <c r="H133" s="52" t="n"/>
-      <c r="I133" s="53" t="n"/>
-      <c r="J133" s="54" t="n"/>
-      <c r="K133" s="55" t="n"/>
-      <c r="L133" s="18" t="n"/>
-      <c r="M133" s="21" t="n"/>
-      <c r="N133" s="56" t="n"/>
-      <c r="O133" s="57" t="n"/>
-      <c r="P133" s="58" t="n"/>
-      <c r="Q133" s="56" t="n"/>
-      <c r="R133" s="56" t="n"/>
-      <c r="S133" s="56" t="n"/>
-      <c r="T133" s="56" t="n"/>
-      <c r="U133" s="56" t="n"/>
-      <c r="V133" s="56" t="n"/>
-      <c r="W133" s="56" t="n"/>
-      <c r="X133" s="56" t="n"/>
-      <c r="Y133" s="56" t="n"/>
-      <c r="Z133" s="56" t="n"/>
-      <c r="AA133" s="56" t="n"/>
-      <c r="AB133" s="56" t="n"/>
+      <c r="B133" s="427" t="n">
+        <v>46302</v>
+      </c>
+      <c r="C133" s="255" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="D133" s="256" t="n">
+        <v>360</v>
+      </c>
+      <c r="E133" s="49" t="n">
+        <v>1095</v>
+      </c>
+      <c r="F133" s="50">
+        <f>IFERROR(D133+E133+G133+U133+Y133,0)</f>
+        <v>1455.0</v>
+      </c>
+      <c r="G133" s="257" t="n">
+        <v>0</v>
+      </c>
+      <c r="H133" s="258">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B133,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B133+1))</f>
+        <v>1085.0</v>
+      </c>
+      <c r="I133" s="259">
+        <f>IFERROR(F133-H133,0)</f>
+        <v>370.0</v>
+      </c>
+      <c r="J133" s="260">
+        <f>IFERROR(I133/F133,0)</f>
+        <v>0.254296</v>
+      </c>
+      <c r="K133" s="254" t="n"/>
+      <c r="L133" s="261" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
+      <c r="M133" s="291" t="n"/>
+      <c r="N133" s="292" t="n"/>
+      <c r="O133" s="293" t="n"/>
+      <c r="P133" s="294" t="n"/>
+      <c r="Q133" s="292" t="n"/>
+      <c r="R133" s="443">
+        <f>IFERROR(D133*$T$7,0)</f>
+        <v>14.62</v>
+      </c>
+      <c r="S133" s="292" t="n"/>
+      <c r="T133" s="292" t="n"/>
+      <c r="U133" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="V133" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="W133" s="292" t="n"/>
+      <c r="X133" s="292" t="n"/>
+      <c r="Y133" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z133" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA133" s="292" t="n"/>
+      <c r="AB133" s="292" t="n"/>
     </row>
     <row r="134" ht="16.5" customHeight="1" s="331">
       <c r="B134" s="34" t="n"/>
@@ -26497,9 +26536,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="B5:P5"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="I2:P2"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="B5:P5"/>
     <mergeCell ref="A3:P3"/>
   </mergeCells>
   <conditionalFormatting sqref="I8:I372">
@@ -26522,7 +26561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J840"/>
+  <dimension ref="A1:J843"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="4" customWidth="1" style="331" min="1" max="1"/>
@@ -62143,6 +62182,135 @@
         </is>
       </c>
       <c r="J840" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="B841" s="429" t="n">
+        <v>46302</v>
+      </c>
+      <c r="C841" s="297" t="inlineStr">
+        <is>
+          <t>Carne</t>
+        </is>
+      </c>
+      <c r="D841" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E841" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat</t>
+        </is>
+      </c>
+      <c r="F841" s="299" t="n">
+        <v>189</v>
+      </c>
+      <c r="G841" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H841" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I841" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J841" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="B842" s="429" t="n">
+        <v>46302</v>
+      </c>
+      <c r="C842" s="297" t="inlineStr">
+        <is>
+          <t>Guimar</t>
+        </is>
+      </c>
+      <c r="D842" s="298" t="inlineStr">
+        <is>
+          <t>Guimar Polietilenos</t>
+        </is>
+      </c>
+      <c r="E842" s="297" t="inlineStr">
+        <is>
+          <t>Packaging/Disposables</t>
+        </is>
+      </c>
+      <c r="F842" s="299" t="n">
+        <v>146</v>
+      </c>
+      <c r="G842" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H842" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I842" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J842" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="B843" s="429" t="n">
+        <v>46302</v>
+      </c>
+      <c r="C843" s="297" t="inlineStr">
+        <is>
+          <t>Avia Reca</t>
+        </is>
+      </c>
+      <c r="D843" s="298" t="inlineStr">
+        <is>
+          <t>Reca</t>
+        </is>
+      </c>
+      <c r="E843" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Beverages</t>
+        </is>
+      </c>
+      <c r="F843" s="299" t="n">
+        <v>750</v>
+      </c>
+      <c r="G843" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H843" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I843" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J843" s="423" t="inlineStr">
         <is>
           <t>No receipt; cash</t>
         </is>
@@ -73053,7 +73221,7 @@
     <row r="25">
       <c r="A25" s="439" t="inlineStr">
         <is>
-          <t>Ingredients - Bread</t>
+          <t>Ingredients - Beverages</t>
         </is>
       </c>
       <c r="B25" s="437">
@@ -73089,7 +73257,7 @@
     <row r="26">
       <c r="A26" s="439" t="inlineStr">
         <is>
-          <t>Ingredients - Beverages</t>
+          <t>Ingredients - Bread</t>
         </is>
       </c>
       <c r="B26" s="437">

</xml_diff>

<commit_message>
LOKA 12-Oct-2026 | EOD | day 2026-10-08: rev $2,665 exp $296 net $2,369 | bal vs capital $-18,191
Changed: LOKA_Restaurant_Manager.xlsx, dashboard.html, loka.py, today.txt
+ 3 backup/day file(s)
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -5871,7 +5871,7 @@
         </is>
       </c>
       <c r="C172" s="455" t="n">
-        <v>-20411.71</v>
+        <v>-18191.25</v>
       </c>
       <c r="E172" s="423" t="inlineStr">
         <is>
@@ -5886,7 +5886,7 @@
         </is>
       </c>
       <c r="C173" s="457" t="n">
-        <v>105522.29</v>
+        <v>107742.75</v>
       </c>
       <c r="E173" s="423" t="inlineStr">
         <is>
@@ -6057,7 +6057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H105"/>
+  <dimension ref="A1:H106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" style="331" min="1" max="1"/>
@@ -9452,30 +9452,63 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="430" t="inlineStr">
+      <c r="A105" s="430" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B105" s="232" t="inlineStr">
+        <is>
+          <t>Transfer-to-me (customer payment 08-Oct)</t>
+        </is>
+      </c>
+      <c r="C105" s="232" t="inlineStr">
+        <is>
+          <t>Transfer Received</t>
+        </is>
+      </c>
+      <c r="D105" s="232" t="n"/>
+      <c r="E105" s="233" t="n">
+        <v>85</v>
+      </c>
+      <c r="F105" s="233">
+        <f>IFERROR(F104+D105-E105,0)</f>
+        <v/>
+      </c>
+      <c r="G105" s="232" t="inlineStr">
+        <is>
+          <t>✅ Received</t>
+        </is>
+      </c>
+      <c r="H105" s="232" t="inlineStr">
+        <is>
+          <t>Customer paid Lohith personal acct</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="430" t="inlineStr">
         <is>
           <t>TOTALS &amp; CURRENT BALANCE</t>
         </is>
       </c>
-      <c r="B105" s="232" t="n"/>
-      <c r="C105" s="232" t="n"/>
-      <c r="D105" s="232">
-        <f>SUM(D4:D104)</f>
-        <v/>
-      </c>
-      <c r="E105" s="233">
-        <f>SUM(E4:E104)</f>
-        <v/>
-      </c>
-      <c r="F105" s="233">
-        <f>F104</f>
-        <v/>
-      </c>
-      <c r="G105" s="232">
-        <f>IF(F104&gt;0,"Restaurant owes Lohith $"&amp;TEXT(F104,"#,##0"),IF(F104&lt;0,"Lohith holds $"&amp;TEXT(ABS(F104),"#,##0"),"Zero balance"))</f>
-        <v/>
-      </c>
-      <c r="H105" s="232" t="n"/>
+      <c r="B106" s="232" t="n"/>
+      <c r="C106" s="232" t="n"/>
+      <c r="D106" s="232">
+        <f>SUM(D4:D105)</f>
+        <v/>
+      </c>
+      <c r="E106" s="233">
+        <f>SUM(E4:E105)</f>
+        <v/>
+      </c>
+      <c r="F106" s="233">
+        <f>F105</f>
+        <v/>
+      </c>
+      <c r="G106" s="232">
+        <f>IF(F105&gt;0,"Restaurant owes Lohith $"&amp;TEXT(F105,"#,##0"),IF(F105&lt;0,"Lohith holds $"&amp;TEXT(ABS(F105),"#,##0"),"Zero balance"))</f>
+        <v/>
+      </c>
+      <c r="H106" s="232" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -11309,45 +11342,45 @@
       <c r="E6" s="29" t="n"/>
       <c r="F6" s="30">
         <f>SUMIFS($D$8:$D$5000,$B$8:$B$5000,TODAY())+SUMIFS($E$8:$E$5000,$B$8:$B$5000,TODAY())+SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())+SUMIFS($U$8:$U$5000,$B$8:$B$5000,TODAY())+SUMIFS($Y$8:$Y$5000,$B$8:$B$5000,TODAY())</f>
-        <v>1455.0</v>
+        <v>2665.0</v>
       </c>
       <c r="G6" s="31">
         <f>SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())</f>
-        <v>0.0</v>
+        <v>85.0</v>
       </c>
       <c r="H6" s="28">
         <f>SUMIFS($H$8:$H$5000,$B$8:$B$5000,TODAY())</f>
-        <v>1085.0</v>
+        <v>296.0</v>
       </c>
       <c r="I6" s="32">
         <f>F6-H6</f>
-        <v>370.0</v>
+        <v>2369.0</v>
       </c>
       <c r="J6">
         <f>IFERROR(I6/F6,0)</f>
-        <v>0.254296</v>
+        <v>0.888931</v>
       </c>
       <c r="K6" s="28" t="n"/>
       <c r="L6" s="31" t="n"/>
       <c r="M6" s="28">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>11360.0</v>
+        <v>14025.0</v>
       </c>
       <c r="N6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>11360.0</v>
+        <v>14025.0</v>
       </c>
       <c r="O6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),$B$8:$B$5000,"&lt;"&amp;DATE(YEAR(TODAY()),MONTH(TODAY())+1,1))</f>
-        <v>20115.0</v>
+        <v>22780.0</v>
       </c>
       <c r="P6">
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>35171.68</v>
+        <v>35467.68</v>
       </c>
       <c r="Q6">
         <f>M6-P6</f>
-        <v>-23811.68</v>
+        <v>-21442.68</v>
       </c>
     </row>
     <row r="7" ht="27.75" customHeight="1" s="331">
@@ -19604,33 +19637,72 @@
       <c r="AB133" s="292" t="n"/>
     </row>
     <row r="134" ht="16.5" customHeight="1" s="331">
-      <c r="B134" s="34" t="n"/>
-      <c r="C134" s="35" t="n"/>
-      <c r="D134" s="36" t="n"/>
-      <c r="E134" s="37" t="n"/>
-      <c r="F134" s="38" t="n"/>
-      <c r="G134" s="39" t="n"/>
-      <c r="H134" s="40" t="n"/>
-      <c r="I134" s="41" t="n"/>
-      <c r="J134" s="42" t="n"/>
-      <c r="K134" s="43" t="n"/>
-      <c r="L134" s="9" t="n"/>
-      <c r="M134" s="12" t="n"/>
-      <c r="N134" s="44" t="n"/>
-      <c r="O134" s="45" t="n"/>
-      <c r="P134" s="46" t="n"/>
-      <c r="Q134" s="44" t="n"/>
-      <c r="R134" s="44" t="n"/>
-      <c r="S134" s="44" t="n"/>
-      <c r="T134" s="44" t="n"/>
-      <c r="U134" s="44" t="n"/>
-      <c r="V134" s="44" t="n"/>
-      <c r="W134" s="44" t="n"/>
-      <c r="X134" s="44" t="n"/>
-      <c r="Y134" s="44" t="n"/>
-      <c r="Z134" s="44" t="n"/>
-      <c r="AA134" s="44" t="n"/>
-      <c r="AB134" s="44" t="n"/>
+      <c r="B134" s="427" t="n">
+        <v>46303</v>
+      </c>
+      <c r="C134" s="270" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D134" s="271" t="n">
+        <v>1565</v>
+      </c>
+      <c r="E134" s="37" t="n">
+        <v>1015</v>
+      </c>
+      <c r="F134" s="38">
+        <f>IFERROR(D134+E134+G134+U134+Y134,0)</f>
+        <v>2665.0</v>
+      </c>
+      <c r="G134" s="272" t="n">
+        <v>85</v>
+      </c>
+      <c r="H134" s="273">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B134,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B134+1))</f>
+        <v>296.0</v>
+      </c>
+      <c r="I134" s="274">
+        <f>IFERROR(F134-H134,0)</f>
+        <v>2369.0</v>
+      </c>
+      <c r="J134" s="275">
+        <f>IFERROR(I134/F134,0)</f>
+        <v>0.888931</v>
+      </c>
+      <c r="K134" s="250" t="n"/>
+      <c r="L134" s="276" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
+      <c r="M134" s="323" t="n"/>
+      <c r="N134" s="324" t="n"/>
+      <c r="O134" s="325" t="n"/>
+      <c r="P134" s="326" t="n"/>
+      <c r="Q134" s="324" t="n"/>
+      <c r="R134" s="428">
+        <f>IFERROR(D134*$T$7,0)</f>
+        <v>63.54</v>
+      </c>
+      <c r="S134" s="324" t="n"/>
+      <c r="T134" s="324" t="n"/>
+      <c r="U134" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="V134" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="W134" s="324" t="n"/>
+      <c r="X134" s="324" t="n"/>
+      <c r="Y134" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z134" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA134" s="324" t="n"/>
+      <c r="AB134" s="324" t="n"/>
     </row>
     <row r="135" ht="16.5" customHeight="1" s="331">
       <c r="B135" s="34" t="n"/>
@@ -26536,9 +26608,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="I2:P2"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="B5:P5"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="I2:P2"/>
     <mergeCell ref="A3:P3"/>
   </mergeCells>
   <conditionalFormatting sqref="I8:I372">
@@ -26561,7 +26633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J843"/>
+  <dimension ref="A1:J846"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="4" customWidth="1" style="331" min="1" max="1"/>
@@ -62311,6 +62383,135 @@
         </is>
       </c>
       <c r="J843" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="844">
+      <c r="B844" s="429" t="n">
+        <v>46303</v>
+      </c>
+      <c r="C844" s="297" t="inlineStr">
+        <is>
+          <t>Oxxo Arroz</t>
+        </is>
+      </c>
+      <c r="D844" s="298" t="inlineStr">
+        <is>
+          <t>OXXO</t>
+        </is>
+      </c>
+      <c r="E844" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Pantry</t>
+        </is>
+      </c>
+      <c r="F844" s="299" t="n">
+        <v>130</v>
+      </c>
+      <c r="G844" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H844" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I844" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J844" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="B845" s="429" t="n">
+        <v>46303</v>
+      </c>
+      <c r="C845" s="297" t="inlineStr">
+        <is>
+          <t>Agua</t>
+        </is>
+      </c>
+      <c r="D845" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E845" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Beverages</t>
+        </is>
+      </c>
+      <c r="F845" s="299" t="n">
+        <v>45</v>
+      </c>
+      <c r="G845" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H845" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I845" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J845" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="B846" s="429" t="n">
+        <v>46303</v>
+      </c>
+      <c r="C846" s="297" t="inlineStr">
+        <is>
+          <t>Chedraui</t>
+        </is>
+      </c>
+      <c r="D846" s="298" t="inlineStr">
+        <is>
+          <t>Chedraui</t>
+        </is>
+      </c>
+      <c r="E846" s="297" t="inlineStr">
+        <is>
+          <t>Supermarket/General</t>
+        </is>
+      </c>
+      <c r="F846" s="299" t="n">
+        <v>121</v>
+      </c>
+      <c r="G846" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H846" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I846" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J846" s="423" t="inlineStr">
         <is>
           <t>No receipt; cash</t>
         </is>

</xml_diff>

<commit_message>
LOKA 12-Oct-2026 | EOD | day 2026-10-09: rev $4,480 exp $1,460 net $3,020 | bal vs capital $-15,418
Changed: LOKA_Restaurant_Manager.xlsx, dashboard.html, loka.py, today.txt
+ 3 backup/day file(s)
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -5871,7 +5871,7 @@
         </is>
       </c>
       <c r="C172" s="455" t="n">
-        <v>-18191.25</v>
+        <v>-15417.81</v>
       </c>
       <c r="E172" s="423" t="inlineStr">
         <is>
@@ -5886,7 +5886,7 @@
         </is>
       </c>
       <c r="C173" s="457" t="n">
-        <v>107742.75</v>
+        <v>110516.19</v>
       </c>
       <c r="E173" s="423" t="inlineStr">
         <is>
@@ -6057,7 +6057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H106"/>
+  <dimension ref="A1:H107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" style="331" min="1" max="1"/>
@@ -9485,30 +9485,63 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="430" t="inlineStr">
+      <c r="A106" s="430" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B106" s="232" t="inlineStr">
+        <is>
+          <t>Transfer-to-me (customer payment 09-Oct)</t>
+        </is>
+      </c>
+      <c r="C106" s="232" t="inlineStr">
+        <is>
+          <t>Transfer Received</t>
+        </is>
+      </c>
+      <c r="D106" s="232" t="n"/>
+      <c r="E106" s="233" t="n">
+        <v>130</v>
+      </c>
+      <c r="F106" s="233">
+        <f>IFERROR(F105+D106-E106,0)</f>
+        <v/>
+      </c>
+      <c r="G106" s="232" t="inlineStr">
+        <is>
+          <t>✅ Received</t>
+        </is>
+      </c>
+      <c r="H106" s="232" t="inlineStr">
+        <is>
+          <t>Customer paid Lohith personal acct</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="430" t="inlineStr">
         <is>
           <t>TOTALS &amp; CURRENT BALANCE</t>
         </is>
       </c>
-      <c r="B106" s="232" t="n"/>
-      <c r="C106" s="232" t="n"/>
-      <c r="D106" s="232">
-        <f>SUM(D4:D105)</f>
-        <v/>
-      </c>
-      <c r="E106" s="233">
-        <f>SUM(E4:E105)</f>
-        <v/>
-      </c>
-      <c r="F106" s="233">
-        <f>F105</f>
-        <v/>
-      </c>
-      <c r="G106" s="232">
-        <f>IF(F105&gt;0,"Restaurant owes Lohith $"&amp;TEXT(F105,"#,##0"),IF(F105&lt;0,"Lohith holds $"&amp;TEXT(ABS(F105),"#,##0"),"Zero balance"))</f>
-        <v/>
-      </c>
-      <c r="H106" s="232" t="n"/>
+      <c r="B107" s="232" t="n"/>
+      <c r="C107" s="232" t="n"/>
+      <c r="D107" s="232">
+        <f>SUM(D4:D106)</f>
+        <v/>
+      </c>
+      <c r="E107" s="233">
+        <f>SUM(E4:E106)</f>
+        <v/>
+      </c>
+      <c r="F107" s="233">
+        <f>F106</f>
+        <v/>
+      </c>
+      <c r="G107" s="232">
+        <f>IF(F106&gt;0,"Restaurant owes Lohith $"&amp;TEXT(F106,"#,##0"),IF(F106&lt;0,"Lohith holds $"&amp;TEXT(ABS(F106),"#,##0"),"Zero balance"))</f>
+        <v/>
+      </c>
+      <c r="H107" s="232" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -11342,45 +11375,45 @@
       <c r="E6" s="29" t="n"/>
       <c r="F6" s="30">
         <f>SUMIFS($D$8:$D$5000,$B$8:$B$5000,TODAY())+SUMIFS($E$8:$E$5000,$B$8:$B$5000,TODAY())+SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())+SUMIFS($U$8:$U$5000,$B$8:$B$5000,TODAY())+SUMIFS($Y$8:$Y$5000,$B$8:$B$5000,TODAY())</f>
-        <v>2665.0</v>
+        <v>4480.0</v>
       </c>
       <c r="G6" s="31">
         <f>SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())</f>
-        <v>85.0</v>
+        <v>130.0</v>
       </c>
       <c r="H6" s="28">
         <f>SUMIFS($H$8:$H$5000,$B$8:$B$5000,TODAY())</f>
-        <v>296.0</v>
+        <v>1460.0</v>
       </c>
       <c r="I6" s="32">
         <f>F6-H6</f>
-        <v>2369.0</v>
+        <v>3020.0</v>
       </c>
       <c r="J6">
         <f>IFERROR(I6/F6,0)</f>
-        <v>0.888931</v>
+        <v>0.674107</v>
       </c>
       <c r="K6" s="28" t="n"/>
       <c r="L6" s="31" t="n"/>
       <c r="M6" s="28">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>14025.0</v>
+        <v>18505.0</v>
       </c>
       <c r="N6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>14025.0</v>
+        <v>18505.0</v>
       </c>
       <c r="O6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),$B$8:$B$5000,"&lt;"&amp;DATE(YEAR(TODAY()),MONTH(TODAY())+1,1))</f>
-        <v>22780.0</v>
+        <v>27260.0</v>
       </c>
       <c r="P6">
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>35467.68</v>
+        <v>36927.68</v>
       </c>
       <c r="Q6">
         <f>M6-P6</f>
-        <v>-21442.68</v>
+        <v>-18422.68</v>
       </c>
     </row>
     <row r="7" ht="27.75" customHeight="1" s="331">
@@ -19705,33 +19738,72 @@
       <c r="AB134" s="324" t="n"/>
     </row>
     <row r="135" ht="16.5" customHeight="1" s="331">
-      <c r="B135" s="34" t="n"/>
-      <c r="C135" s="47" t="n"/>
-      <c r="D135" s="48" t="n"/>
-      <c r="E135" s="49" t="n"/>
-      <c r="F135" s="50" t="n"/>
-      <c r="G135" s="51" t="n"/>
-      <c r="H135" s="52" t="n"/>
-      <c r="I135" s="53" t="n"/>
-      <c r="J135" s="54" t="n"/>
-      <c r="K135" s="55" t="n"/>
-      <c r="L135" s="18" t="n"/>
-      <c r="M135" s="21" t="n"/>
-      <c r="N135" s="56" t="n"/>
-      <c r="O135" s="57" t="n"/>
-      <c r="P135" s="58" t="n"/>
-      <c r="Q135" s="56" t="n"/>
-      <c r="R135" s="56" t="n"/>
-      <c r="S135" s="56" t="n"/>
-      <c r="T135" s="56" t="n"/>
-      <c r="U135" s="56" t="n"/>
-      <c r="V135" s="56" t="n"/>
-      <c r="W135" s="56" t="n"/>
-      <c r="X135" s="56" t="n"/>
-      <c r="Y135" s="56" t="n"/>
-      <c r="Z135" s="56" t="n"/>
-      <c r="AA135" s="56" t="n"/>
-      <c r="AB135" s="56" t="n"/>
+      <c r="B135" s="427" t="n">
+        <v>46304</v>
+      </c>
+      <c r="C135" s="255" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D135" s="256" t="n">
+        <v>2871</v>
+      </c>
+      <c r="E135" s="49" t="n">
+        <v>1479</v>
+      </c>
+      <c r="F135" s="50">
+        <f>IFERROR(D135+E135+G135+U135+Y135,0)</f>
+        <v>4480.0</v>
+      </c>
+      <c r="G135" s="257" t="n">
+        <v>130</v>
+      </c>
+      <c r="H135" s="258">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B135,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B135+1))</f>
+        <v>1460.0</v>
+      </c>
+      <c r="I135" s="259">
+        <f>IFERROR(F135-H135,0)</f>
+        <v>3020.0</v>
+      </c>
+      <c r="J135" s="260">
+        <f>IFERROR(I135/F135,0)</f>
+        <v>0.674107</v>
+      </c>
+      <c r="K135" s="254" t="n"/>
+      <c r="L135" s="261" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
+      <c r="M135" s="291" t="n"/>
+      <c r="N135" s="292" t="n"/>
+      <c r="O135" s="293" t="n"/>
+      <c r="P135" s="294" t="n"/>
+      <c r="Q135" s="292" t="n"/>
+      <c r="R135" s="443">
+        <f>IFERROR(D135*$T$7,0)</f>
+        <v>116.56</v>
+      </c>
+      <c r="S135" s="292" t="n"/>
+      <c r="T135" s="292" t="n"/>
+      <c r="U135" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="V135" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="W135" s="292" t="n"/>
+      <c r="X135" s="292" t="n"/>
+      <c r="Y135" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z135" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA135" s="292" t="n"/>
+      <c r="AB135" s="292" t="n"/>
     </row>
     <row r="136" ht="16.5" customHeight="1" s="331">
       <c r="B136" s="34" t="n"/>
@@ -26608,8 +26680,8 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="I2:P2"/>
-    <mergeCell ref="A2:H2"/>
     <mergeCell ref="B5:P5"/>
     <mergeCell ref="A3:P3"/>
   </mergeCells>
@@ -26633,7 +26705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J846"/>
+  <dimension ref="A1:J847"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="4" customWidth="1" style="331" min="1" max="1"/>
@@ -62514,6 +62586,49 @@
       <c r="J846" s="423" t="inlineStr">
         <is>
           <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="B847" s="429" t="n">
+        <v>46304</v>
+      </c>
+      <c r="C847" s="297" t="inlineStr">
+        <is>
+          <t>Duvi - salary</t>
+        </is>
+      </c>
+      <c r="D847" s="298" t="inlineStr">
+        <is>
+          <t>Payroll</t>
+        </is>
+      </c>
+      <c r="E847" s="297" t="inlineStr">
+        <is>
+          <t>Staff - Salary</t>
+        </is>
+      </c>
+      <c r="F847" s="299" t="n">
+        <v>1460</v>
+      </c>
+      <c r="G847" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H847" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I847" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J847" s="423" t="inlineStr">
+        <is>
+          <t>Weekly salary</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
LOKA 12-Oct-2026 | EOD | day 2026-10-10: rev $3,260 exp $13,069 net $-9,809 | bal vs capital $-24,438
Changed: LOKA_Restaurant_Manager.xlsx, dashboard.html, loka.py, today.txt
+ 3 backup/day file(s)
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -5871,7 +5871,7 @@
         </is>
       </c>
       <c r="C172" s="455" t="n">
-        <v>-15417.81</v>
+        <v>-24438.09</v>
       </c>
       <c r="E172" s="423" t="inlineStr">
         <is>
@@ -5886,7 +5886,7 @@
         </is>
       </c>
       <c r="C173" s="457" t="n">
-        <v>110516.19</v>
+        <v>101495.91</v>
       </c>
       <c r="E173" s="423" t="inlineStr">
         <is>
@@ -6057,7 +6057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H107"/>
+  <dimension ref="A1:H109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" style="331" min="1" max="1"/>
@@ -9518,30 +9518,96 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="430" t="inlineStr">
+      <c r="A107" s="430" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B107" s="232" t="inlineStr">
+        <is>
+          <t>Transfer-to-me (customer payment 10-Oct)</t>
+        </is>
+      </c>
+      <c r="C107" s="232" t="inlineStr">
+        <is>
+          <t>Transfer Received</t>
+        </is>
+      </c>
+      <c r="D107" s="232" t="n"/>
+      <c r="E107" s="233" t="n">
+        <v>220</v>
+      </c>
+      <c r="F107" s="233">
+        <f>IFERROR(F106+D107-E107,0)</f>
+        <v/>
+      </c>
+      <c r="G107" s="232" t="inlineStr">
+        <is>
+          <t>✅ Received</t>
+        </is>
+      </c>
+      <c r="H107" s="232" t="inlineStr">
+        <is>
+          <t>Customer paid Lohith personal acct</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="430" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B108" s="232" t="inlineStr">
+        <is>
+          <t>Pollo $1,055 (paid by Lohith)</t>
+        </is>
+      </c>
+      <c r="C108" s="232" t="inlineStr">
+        <is>
+          <t>Expense - Personal</t>
+        </is>
+      </c>
+      <c r="D108" s="232" t="n">
+        <v>1055</v>
+      </c>
+      <c r="E108" s="233" t="n"/>
+      <c r="F108" s="233">
+        <f>IFERROR(F107+D108-E108,0)</f>
+        <v/>
+      </c>
+      <c r="G108" s="232" t="inlineStr">
+        <is>
+          <t>⏳ Reimburse</t>
+        </is>
+      </c>
+      <c r="H108" s="232" t="inlineStr">
+        <is>
+          <t>Fronted from own pocket; excluded from till via cash_adjust</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="430" t="inlineStr">
         <is>
           <t>TOTALS &amp; CURRENT BALANCE</t>
         </is>
       </c>
-      <c r="B107" s="232" t="n"/>
-      <c r="C107" s="232" t="n"/>
-      <c r="D107" s="232">
-        <f>SUM(D4:D106)</f>
-        <v/>
-      </c>
-      <c r="E107" s="233">
-        <f>SUM(E4:E106)</f>
-        <v/>
-      </c>
-      <c r="F107" s="233">
-        <f>F106</f>
-        <v/>
-      </c>
-      <c r="G107" s="232">
-        <f>IF(F106&gt;0,"Restaurant owes Lohith $"&amp;TEXT(F106,"#,##0"),IF(F106&lt;0,"Lohith holds $"&amp;TEXT(ABS(F106),"#,##0"),"Zero balance"))</f>
-        <v/>
-      </c>
-      <c r="H107" s="232" t="n"/>
+      <c r="B109" s="232" t="n"/>
+      <c r="C109" s="232" t="n"/>
+      <c r="D109" s="232">
+        <f>SUM(D4:D108)</f>
+        <v/>
+      </c>
+      <c r="E109" s="233">
+        <f>SUM(E4:E108)</f>
+        <v/>
+      </c>
+      <c r="F109" s="233">
+        <f>F108</f>
+        <v/>
+      </c>
+      <c r="G109" s="232">
+        <f>IF(F108&gt;0,"Restaurant owes Lohith $"&amp;TEXT(F108,"#,##0"),IF(F108&lt;0,"Lohith holds $"&amp;TEXT(ABS(F108),"#,##0"),"Zero balance"))</f>
+        <v/>
+      </c>
+      <c r="H109" s="232" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -11375,45 +11441,45 @@
       <c r="E6" s="29" t="n"/>
       <c r="F6" s="30">
         <f>SUMIFS($D$8:$D$5000,$B$8:$B$5000,TODAY())+SUMIFS($E$8:$E$5000,$B$8:$B$5000,TODAY())+SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())+SUMIFS($U$8:$U$5000,$B$8:$B$5000,TODAY())+SUMIFS($Y$8:$Y$5000,$B$8:$B$5000,TODAY())</f>
-        <v>4480.0</v>
+        <v>3260.0</v>
       </c>
       <c r="G6" s="31">
         <f>SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())</f>
-        <v>130.0</v>
+        <v>220.0</v>
       </c>
       <c r="H6" s="28">
         <f>SUMIFS($H$8:$H$5000,$B$8:$B$5000,TODAY())</f>
-        <v>1460.0</v>
+        <v>13069.0</v>
       </c>
       <c r="I6" s="32">
         <f>F6-H6</f>
-        <v>3020.0</v>
+        <v>-9809.0</v>
       </c>
       <c r="J6">
         <f>IFERROR(I6/F6,0)</f>
-        <v>0.674107</v>
+        <v>-3.008896</v>
       </c>
       <c r="K6" s="28" t="n"/>
       <c r="L6" s="31" t="n"/>
       <c r="M6" s="28">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>18505.0</v>
+        <v>21765.0</v>
       </c>
       <c r="N6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>18505.0</v>
+        <v>21765.0</v>
       </c>
       <c r="O6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),$B$8:$B$5000,"&lt;"&amp;DATE(YEAR(TODAY()),MONTH(TODAY())+1,1))</f>
-        <v>27260.0</v>
+        <v>30520.0</v>
       </c>
       <c r="P6">
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>36927.68</v>
+        <v>49996.68</v>
       </c>
       <c r="Q6">
         <f>M6-P6</f>
-        <v>-18422.68</v>
+        <v>-28231.68</v>
       </c>
     </row>
     <row r="7" ht="27.75" customHeight="1" s="331">
@@ -19806,33 +19872,72 @@
       <c r="AB135" s="292" t="n"/>
     </row>
     <row r="136" ht="16.5" customHeight="1" s="331">
-      <c r="B136" s="34" t="n"/>
-      <c r="C136" s="35" t="n"/>
-      <c r="D136" s="36" t="n"/>
-      <c r="E136" s="37" t="n"/>
-      <c r="F136" s="38" t="n"/>
-      <c r="G136" s="39" t="n"/>
-      <c r="H136" s="40" t="n"/>
-      <c r="I136" s="41" t="n"/>
-      <c r="J136" s="42" t="n"/>
-      <c r="K136" s="43" t="n"/>
-      <c r="L136" s="9" t="n"/>
-      <c r="M136" s="12" t="n"/>
-      <c r="N136" s="44" t="n"/>
-      <c r="O136" s="45" t="n"/>
-      <c r="P136" s="46" t="n"/>
-      <c r="Q136" s="44" t="n"/>
-      <c r="R136" s="44" t="n"/>
-      <c r="S136" s="44" t="n"/>
-      <c r="T136" s="44" t="n"/>
-      <c r="U136" s="44" t="n"/>
-      <c r="V136" s="44" t="n"/>
-      <c r="W136" s="44" t="n"/>
-      <c r="X136" s="44" t="n"/>
-      <c r="Y136" s="44" t="n"/>
-      <c r="Z136" s="44" t="n"/>
-      <c r="AA136" s="44" t="n"/>
-      <c r="AB136" s="44" t="n"/>
+      <c r="B136" s="427" t="n">
+        <v>46305</v>
+      </c>
+      <c r="C136" s="270" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="D136" s="271" t="n">
+        <v>1140</v>
+      </c>
+      <c r="E136" s="37" t="n">
+        <v>1900</v>
+      </c>
+      <c r="F136" s="38">
+        <f>IFERROR(D136+E136+G136+U136+Y136,0)</f>
+        <v>3260.0</v>
+      </c>
+      <c r="G136" s="272" t="n">
+        <v>220</v>
+      </c>
+      <c r="H136" s="273">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B136,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B136+1))</f>
+        <v>13069.0</v>
+      </c>
+      <c r="I136" s="274">
+        <f>IFERROR(F136-H136,0)</f>
+        <v>-9809.0</v>
+      </c>
+      <c r="J136" s="275">
+        <f>IFERROR(I136/F136,0)</f>
+        <v>-3.008896</v>
+      </c>
+      <c r="K136" s="250" t="n"/>
+      <c r="L136" s="276" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
+      <c r="M136" s="323" t="n"/>
+      <c r="N136" s="324" t="n"/>
+      <c r="O136" s="325" t="n"/>
+      <c r="P136" s="326" t="n"/>
+      <c r="Q136" s="324" t="n"/>
+      <c r="R136" s="428">
+        <f>IFERROR(D136*$T$7,0)</f>
+        <v>46.28</v>
+      </c>
+      <c r="S136" s="324" t="n"/>
+      <c r="T136" s="324" t="n"/>
+      <c r="U136" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="V136" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="W136" s="324" t="n"/>
+      <c r="X136" s="324" t="n"/>
+      <c r="Y136" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z136" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA136" s="324" t="n"/>
+      <c r="AB136" s="324" t="n"/>
     </row>
     <row r="137" ht="16.5" customHeight="1" s="331">
       <c r="B137" s="34" t="n"/>
@@ -26705,7 +26810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J847"/>
+  <dimension ref="A1:J857"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="4" customWidth="1" style="331" min="1" max="1"/>
@@ -62627,6 +62732,436 @@
         </is>
       </c>
       <c r="J847" s="423" t="inlineStr">
+        <is>
+          <t>Weekly salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="B848" s="429" t="n">
+        <v>46305</v>
+      </c>
+      <c r="C848" s="297" t="inlineStr">
+        <is>
+          <t>Vegetables</t>
+        </is>
+      </c>
+      <c r="D848" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E848" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Vegetables</t>
+        </is>
+      </c>
+      <c r="F848" s="299" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G848" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H848" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I848" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J848" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="B849" s="429" t="n">
+        <v>46305</v>
+      </c>
+      <c r="C849" s="297" t="inlineStr">
+        <is>
+          <t>Molino</t>
+        </is>
+      </c>
+      <c r="D849" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E849" s="297" t="inlineStr">
+        <is>
+          <t>Supermarket/General</t>
+        </is>
+      </c>
+      <c r="F849" s="299" t="n">
+        <v>72</v>
+      </c>
+      <c r="G849" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H849" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I849" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J849" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="B850" s="429" t="n">
+        <v>46305</v>
+      </c>
+      <c r="C850" s="297" t="inlineStr">
+        <is>
+          <t>Carne</t>
+        </is>
+      </c>
+      <c r="D850" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E850" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat</t>
+        </is>
+      </c>
+      <c r="F850" s="299" t="n">
+        <v>297</v>
+      </c>
+      <c r="G850" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H850" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I850" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J850" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="B851" s="429" t="n">
+        <v>46305</v>
+      </c>
+      <c r="C851" s="297" t="inlineStr">
+        <is>
+          <t>3B</t>
+        </is>
+      </c>
+      <c r="D851" s="298" t="inlineStr">
+        <is>
+          <t>Tres B</t>
+        </is>
+      </c>
+      <c r="E851" s="297" t="inlineStr">
+        <is>
+          <t>Supermarket/General</t>
+        </is>
+      </c>
+      <c r="F851" s="299" t="n">
+        <v>938</v>
+      </c>
+      <c r="G851" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H851" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I851" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J851" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="B852" s="429" t="n">
+        <v>46305</v>
+      </c>
+      <c r="C852" s="297" t="inlineStr">
+        <is>
+          <t>Gas</t>
+        </is>
+      </c>
+      <c r="D852" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E852" s="297" t="inlineStr">
+        <is>
+          <t>Utilities/Gas</t>
+        </is>
+      </c>
+      <c r="F852" s="299" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G852" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H852" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I852" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J852" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="B853" s="429" t="n">
+        <v>46305</v>
+      </c>
+      <c r="C853" s="297" t="inlineStr">
+        <is>
+          <t>Queso Bodega</t>
+        </is>
+      </c>
+      <c r="D853" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E853" s="297" t="inlineStr">
+        <is>
+          <t>Supermarket/General</t>
+        </is>
+      </c>
+      <c r="F853" s="299" t="n">
+        <v>570</v>
+      </c>
+      <c r="G853" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H853" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I853" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J853" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="B854" s="429" t="n">
+        <v>46305</v>
+      </c>
+      <c r="C854" s="297" t="inlineStr">
+        <is>
+          <t>Queso Panela</t>
+        </is>
+      </c>
+      <c r="D854" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E854" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Dairy</t>
+        </is>
+      </c>
+      <c r="F854" s="299" t="n">
+        <v>687</v>
+      </c>
+      <c r="G854" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H854" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I854" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J854" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="B855" s="429" t="n">
+        <v>46305</v>
+      </c>
+      <c r="C855" s="297" t="inlineStr">
+        <is>
+          <t>Pollo</t>
+        </is>
+      </c>
+      <c r="D855" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E855" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat</t>
+        </is>
+      </c>
+      <c r="F855" s="299" t="n">
+        <v>1055</v>
+      </c>
+      <c r="G855" s="300" t="inlineStr">
+        <is>
+          <t>Lohith</t>
+        </is>
+      </c>
+      <c r="H855" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I855" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J855" s="423" t="inlineStr">
+        <is>
+          <t>Pagado por Lohith (bolsillo); reembolsable via Owner Ledger</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="B856" s="429" t="n">
+        <v>46305</v>
+      </c>
+      <c r="C856" s="297" t="inlineStr">
+        <is>
+          <t>Josias - salary</t>
+        </is>
+      </c>
+      <c r="D856" s="298" t="inlineStr">
+        <is>
+          <t>Payroll</t>
+        </is>
+      </c>
+      <c r="E856" s="297" t="inlineStr">
+        <is>
+          <t>Staff - Salary</t>
+        </is>
+      </c>
+      <c r="F856" s="299" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G856" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H856" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I856" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J856" s="423" t="inlineStr">
+        <is>
+          <t>Weekly salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="B857" s="429" t="n">
+        <v>46305</v>
+      </c>
+      <c r="C857" s="297" t="inlineStr">
+        <is>
+          <t>Jhon - salary</t>
+        </is>
+      </c>
+      <c r="D857" s="298" t="inlineStr">
+        <is>
+          <t>Payroll</t>
+        </is>
+      </c>
+      <c r="E857" s="297" t="inlineStr">
+        <is>
+          <t>Staff - Salary</t>
+        </is>
+      </c>
+      <c r="F857" s="299" t="n">
+        <v>3750</v>
+      </c>
+      <c r="G857" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H857" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I857" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J857" s="423" t="inlineStr">
         <is>
           <t>Weekly salary</t>
         </is>
@@ -73573,7 +74108,7 @@
     <row r="26">
       <c r="A26" s="439" t="inlineStr">
         <is>
-          <t>Ingredients - Bread</t>
+          <t>Ingredients - Dairy</t>
         </is>
       </c>
       <c r="B26" s="437">
@@ -73609,7 +74144,7 @@
     <row r="27">
       <c r="A27" s="439" t="inlineStr">
         <is>
-          <t>Ingredients - Dairy</t>
+          <t>Ingredients - Bread</t>
         </is>
       </c>
       <c r="B27" s="437">
@@ -73753,7 +74288,7 @@
     <row r="31">
       <c r="A31" s="439" t="inlineStr">
         <is>
-          <t>Packaging/Disposables</t>
+          <t>Utilities/Gas</t>
         </is>
       </c>
       <c r="B31" s="437">
@@ -73789,7 +74324,7 @@
     <row r="32">
       <c r="A32" s="439" t="inlineStr">
         <is>
-          <t>Utilities/Gas</t>
+          <t>Packaging/Disposables</t>
         </is>
       </c>
       <c r="B32" s="437">

</xml_diff>

<commit_message>
LOKA 12-Oct-2026 | EOD | day 2026-10-12: rev $4,930 exp $3,040 net $1,890 | bal vs capital $-22,714
Changed: LOKA_Restaurant_Manager.xlsx, dashboard.html, loka.py, today.txt
+ 3 backup/day file(s)
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -5871,7 +5871,7 @@
         </is>
       </c>
       <c r="C172" s="455" t="n">
-        <v>-24438.09</v>
+        <v>-22713.89</v>
       </c>
       <c r="E172" s="423" t="inlineStr">
         <is>
@@ -5886,7 +5886,7 @@
         </is>
       </c>
       <c r="C173" s="457" t="n">
-        <v>101495.91</v>
+        <v>103220.11</v>
       </c>
       <c r="E173" s="423" t="inlineStr">
         <is>
@@ -6057,7 +6057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H109"/>
+  <dimension ref="A1:H110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" style="331" min="1" max="1"/>
@@ -9584,30 +9584,63 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="430" t="inlineStr">
+      <c r="A109" s="430" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B109" s="232" t="inlineStr">
+        <is>
+          <t>Transfer-to-me (customer payment 12-Oct)</t>
+        </is>
+      </c>
+      <c r="C109" s="232" t="inlineStr">
+        <is>
+          <t>Transfer Received</t>
+        </is>
+      </c>
+      <c r="D109" s="232" t="n"/>
+      <c r="E109" s="233" t="n">
+        <v>85</v>
+      </c>
+      <c r="F109" s="233">
+        <f>IFERROR(F108+D109-E109,0)</f>
+        <v/>
+      </c>
+      <c r="G109" s="232" t="inlineStr">
+        <is>
+          <t>✅ Received</t>
+        </is>
+      </c>
+      <c r="H109" s="232" t="inlineStr">
+        <is>
+          <t>Customer paid Lohith personal acct</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="430" t="inlineStr">
         <is>
           <t>TOTALS &amp; CURRENT BALANCE</t>
         </is>
       </c>
-      <c r="B109" s="232" t="n"/>
-      <c r="C109" s="232" t="n"/>
-      <c r="D109" s="232">
-        <f>SUM(D4:D108)</f>
-        <v/>
-      </c>
-      <c r="E109" s="233">
-        <f>SUM(E4:E108)</f>
-        <v/>
-      </c>
-      <c r="F109" s="233">
-        <f>F108</f>
-        <v/>
-      </c>
-      <c r="G109" s="232">
-        <f>IF(F108&gt;0,"Restaurant owes Lohith $"&amp;TEXT(F108,"#,##0"),IF(F108&lt;0,"Lohith holds $"&amp;TEXT(ABS(F108),"#,##0"),"Zero balance"))</f>
-        <v/>
-      </c>
-      <c r="H109" s="232" t="n"/>
+      <c r="B110" s="232" t="n"/>
+      <c r="C110" s="232" t="n"/>
+      <c r="D110" s="232">
+        <f>SUM(D4:D109)</f>
+        <v/>
+      </c>
+      <c r="E110" s="233">
+        <f>SUM(E4:E109)</f>
+        <v/>
+      </c>
+      <c r="F110" s="233">
+        <f>F109</f>
+        <v/>
+      </c>
+      <c r="G110" s="232">
+        <f>IF(F109&gt;0,"Restaurant owes Lohith $"&amp;TEXT(F109,"#,##0"),IF(F109&lt;0,"Lohith holds $"&amp;TEXT(ABS(F109),"#,##0"),"Zero balance"))</f>
+        <v/>
+      </c>
+      <c r="H110" s="232" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -11441,45 +11474,45 @@
       <c r="E6" s="29" t="n"/>
       <c r="F6" s="30">
         <f>SUMIFS($D$8:$D$5000,$B$8:$B$5000,TODAY())+SUMIFS($E$8:$E$5000,$B$8:$B$5000,TODAY())+SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())+SUMIFS($U$8:$U$5000,$B$8:$B$5000,TODAY())+SUMIFS($Y$8:$Y$5000,$B$8:$B$5000,TODAY())</f>
-        <v>3260.0</v>
+        <v>4930.0</v>
       </c>
       <c r="G6" s="31">
         <f>SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())</f>
-        <v>220.0</v>
+        <v>85.0</v>
       </c>
       <c r="H6" s="28">
         <f>SUMIFS($H$8:$H$5000,$B$8:$B$5000,TODAY())</f>
-        <v>13069.0</v>
+        <v>3040.0</v>
       </c>
       <c r="I6" s="32">
         <f>F6-H6</f>
-        <v>-9809.0</v>
+        <v>1890.0</v>
       </c>
       <c r="J6">
         <f>IFERROR(I6/F6,0)</f>
-        <v>-3.008896</v>
+        <v>0.383367</v>
       </c>
       <c r="K6" s="28" t="n"/>
       <c r="L6" s="31" t="n"/>
       <c r="M6" s="28">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>21765.0</v>
+        <v>4930.0</v>
       </c>
       <c r="N6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>21765.0</v>
+        <v>4930.0</v>
       </c>
       <c r="O6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),$B$8:$B$5000,"&lt;"&amp;DATE(YEAR(TODAY()),MONTH(TODAY())+1,1))</f>
-        <v>30520.0</v>
+        <v>35450.0</v>
       </c>
       <c r="P6">
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>49996.68</v>
+        <v>3040.0</v>
       </c>
       <c r="Q6">
         <f>M6-P6</f>
-        <v>-28231.68</v>
+        <v>1890.0</v>
       </c>
     </row>
     <row r="7" ht="27.75" customHeight="1" s="331">
@@ -19940,33 +19973,72 @@
       <c r="AB136" s="324" t="n"/>
     </row>
     <row r="137" ht="16.5" customHeight="1" s="331">
-      <c r="B137" s="34" t="n"/>
-      <c r="C137" s="47" t="n"/>
-      <c r="D137" s="48" t="n"/>
-      <c r="E137" s="49" t="n"/>
-      <c r="F137" s="50" t="n"/>
-      <c r="G137" s="51" t="n"/>
-      <c r="H137" s="52" t="n"/>
-      <c r="I137" s="53" t="n"/>
-      <c r="J137" s="54" t="n"/>
-      <c r="K137" s="55" t="n"/>
-      <c r="L137" s="18" t="n"/>
-      <c r="M137" s="21" t="n"/>
-      <c r="N137" s="56" t="n"/>
-      <c r="O137" s="57" t="n"/>
-      <c r="P137" s="58" t="n"/>
-      <c r="Q137" s="56" t="n"/>
-      <c r="R137" s="56" t="n"/>
-      <c r="S137" s="56" t="n"/>
-      <c r="T137" s="56" t="n"/>
-      <c r="U137" s="56" t="n"/>
-      <c r="V137" s="56" t="n"/>
-      <c r="W137" s="56" t="n"/>
-      <c r="X137" s="56" t="n"/>
-      <c r="Y137" s="56" t="n"/>
-      <c r="Z137" s="56" t="n"/>
-      <c r="AA137" s="56" t="n"/>
-      <c r="AB137" s="56" t="n"/>
+      <c r="B137" s="427" t="n">
+        <v>46307</v>
+      </c>
+      <c r="C137" s="255" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D137" s="256" t="n">
+        <v>1990</v>
+      </c>
+      <c r="E137" s="49" t="n">
+        <v>2855</v>
+      </c>
+      <c r="F137" s="50">
+        <f>IFERROR(D137+E137+G137+U137+Y137,0)</f>
+        <v>4930.0</v>
+      </c>
+      <c r="G137" s="257" t="n">
+        <v>85</v>
+      </c>
+      <c r="H137" s="258">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B137,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B137+1))</f>
+        <v>3040.0</v>
+      </c>
+      <c r="I137" s="259">
+        <f>IFERROR(F137-H137,0)</f>
+        <v>1890.0</v>
+      </c>
+      <c r="J137" s="260">
+        <f>IFERROR(I137/F137,0)</f>
+        <v>0.383367</v>
+      </c>
+      <c r="K137" s="254" t="n"/>
+      <c r="L137" s="261" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
+      <c r="M137" s="291" t="n"/>
+      <c r="N137" s="292" t="n"/>
+      <c r="O137" s="293" t="n"/>
+      <c r="P137" s="294" t="n"/>
+      <c r="Q137" s="292" t="n"/>
+      <c r="R137" s="443">
+        <f>IFERROR(D137*$T$7,0)</f>
+        <v>80.79</v>
+      </c>
+      <c r="S137" s="292" t="n"/>
+      <c r="T137" s="292" t="n"/>
+      <c r="U137" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="V137" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="W137" s="292" t="n"/>
+      <c r="X137" s="292" t="n"/>
+      <c r="Y137" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z137" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA137" s="292" t="n"/>
+      <c r="AB137" s="292" t="n"/>
     </row>
     <row r="138" ht="16.5" customHeight="1" s="331">
       <c r="B138" s="34" t="n"/>
@@ -26785,9 +26857,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="B5:P5"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="I2:P2"/>
-    <mergeCell ref="B5:P5"/>
     <mergeCell ref="A3:P3"/>
   </mergeCells>
   <conditionalFormatting sqref="I8:I372">
@@ -26810,7 +26882,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J857"/>
+  <dimension ref="A1:J859"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="4" customWidth="1" style="331" min="1" max="1"/>
@@ -63164,6 +63236,92 @@
       <c r="J857" s="423" t="inlineStr">
         <is>
           <t>Weekly salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="B858" s="429" t="n">
+        <v>46307</v>
+      </c>
+      <c r="C858" s="297" t="inlineStr">
+        <is>
+          <t>Electric Issue</t>
+        </is>
+      </c>
+      <c r="D858" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E858" s="297" t="inlineStr">
+        <is>
+          <t>Utilities/Electricity</t>
+        </is>
+      </c>
+      <c r="F858" s="299" t="n">
+        <v>2700</v>
+      </c>
+      <c r="G858" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H858" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I858" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J858" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="B859" s="429" t="n">
+        <v>46307</v>
+      </c>
+      <c r="C859" s="297" t="inlineStr">
+        <is>
+          <t>Chedraui</t>
+        </is>
+      </c>
+      <c r="D859" s="298" t="inlineStr">
+        <is>
+          <t>Chedraui</t>
+        </is>
+      </c>
+      <c r="E859" s="297" t="inlineStr">
+        <is>
+          <t>Supermarket/General</t>
+        </is>
+      </c>
+      <c r="F859" s="299" t="n">
+        <v>340</v>
+      </c>
+      <c r="G859" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H859" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I859" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J859" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
LOKA 14-Oct-2026 | EOD | day 2026-10-13: rev $4,435 exp $1,389 net $3,046 | bal vs capital $-19,890
Changed: LOKA_Restaurant_Manager.xlsx, dashboard.html, loka.py, today.txt
+ 2 backup/day file(s)
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -5871,7 +5871,7 @@
         </is>
       </c>
       <c r="C172" s="455" t="n">
-        <v>-22713.89</v>
+        <v>-19890.4</v>
       </c>
       <c r="E172" s="423" t="inlineStr">
         <is>
@@ -5886,7 +5886,7 @@
         </is>
       </c>
       <c r="C173" s="457" t="n">
-        <v>103220.11</v>
+        <v>106043.6</v>
       </c>
       <c r="E173" s="423" t="inlineStr">
         <is>
@@ -6057,7 +6057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H110"/>
+  <dimension ref="A1:H111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" style="331" min="1" max="1"/>
@@ -9617,30 +9617,63 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="430" t="inlineStr">
+      <c r="A110" s="430" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B110" s="232" t="inlineStr">
+        <is>
+          <t>Transfer-to-me (customer payment 13-Oct)</t>
+        </is>
+      </c>
+      <c r="C110" s="232" t="inlineStr">
+        <is>
+          <t>Transfer Received</t>
+        </is>
+      </c>
+      <c r="D110" s="232" t="n"/>
+      <c r="E110" s="233" t="n">
+        <v>120</v>
+      </c>
+      <c r="F110" s="233">
+        <f>IFERROR(F109+D110-E110,0)</f>
+        <v/>
+      </c>
+      <c r="G110" s="232" t="inlineStr">
+        <is>
+          <t>✅ Received</t>
+        </is>
+      </c>
+      <c r="H110" s="232" t="inlineStr">
+        <is>
+          <t>Customer paid Lohith personal acct</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="430" t="inlineStr">
         <is>
           <t>TOTALS &amp; CURRENT BALANCE</t>
         </is>
       </c>
-      <c r="B110" s="232" t="n"/>
-      <c r="C110" s="232" t="n"/>
-      <c r="D110" s="232">
-        <f>SUM(D4:D109)</f>
-        <v/>
-      </c>
-      <c r="E110" s="233">
-        <f>SUM(E4:E109)</f>
-        <v/>
-      </c>
-      <c r="F110" s="233">
-        <f>F109</f>
-        <v/>
-      </c>
-      <c r="G110" s="232">
-        <f>IF(F109&gt;0,"Restaurant owes Lohith $"&amp;TEXT(F109,"#,##0"),IF(F109&lt;0,"Lohith holds $"&amp;TEXT(ABS(F109),"#,##0"),"Zero balance"))</f>
-        <v/>
-      </c>
-      <c r="H110" s="232" t="n"/>
+      <c r="B111" s="232" t="n"/>
+      <c r="C111" s="232" t="n"/>
+      <c r="D111" s="232">
+        <f>SUM(D4:D110)</f>
+        <v/>
+      </c>
+      <c r="E111" s="233">
+        <f>SUM(E4:E110)</f>
+        <v/>
+      </c>
+      <c r="F111" s="233">
+        <f>F110</f>
+        <v/>
+      </c>
+      <c r="G111" s="232">
+        <f>IF(F110&gt;0,"Restaurant owes Lohith $"&amp;TEXT(F110,"#,##0"),IF(F110&lt;0,"Lohith holds $"&amp;TEXT(ABS(F110),"#,##0"),"Zero balance"))</f>
+        <v/>
+      </c>
+      <c r="H111" s="232" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -11474,45 +11507,45 @@
       <c r="E6" s="29" t="n"/>
       <c r="F6" s="30">
         <f>SUMIFS($D$8:$D$5000,$B$8:$B$5000,TODAY())+SUMIFS($E$8:$E$5000,$B$8:$B$5000,TODAY())+SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())+SUMIFS($U$8:$U$5000,$B$8:$B$5000,TODAY())+SUMIFS($Y$8:$Y$5000,$B$8:$B$5000,TODAY())</f>
-        <v>4930.0</v>
+        <v>4435.0</v>
       </c>
       <c r="G6" s="31">
         <f>SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())</f>
-        <v>85.0</v>
+        <v>120.0</v>
       </c>
       <c r="H6" s="28">
         <f>SUMIFS($H$8:$H$5000,$B$8:$B$5000,TODAY())</f>
-        <v>3040.0</v>
+        <v>1389.0</v>
       </c>
       <c r="I6" s="32">
         <f>F6-H6</f>
-        <v>1890.0</v>
+        <v>3046.0</v>
       </c>
       <c r="J6">
         <f>IFERROR(I6/F6,0)</f>
-        <v>0.383367</v>
+        <v>0.686809</v>
       </c>
       <c r="K6" s="28" t="n"/>
       <c r="L6" s="31" t="n"/>
       <c r="M6" s="28">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>4930.0</v>
+        <v>9365.0</v>
       </c>
       <c r="N6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>4930.0</v>
+        <v>9365.0</v>
       </c>
       <c r="O6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),$B$8:$B$5000,"&lt;"&amp;DATE(YEAR(TODAY()),MONTH(TODAY())+1,1))</f>
-        <v>35450.0</v>
+        <v>39885.0</v>
       </c>
       <c r="P6">
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>3040.0</v>
+        <v>4429.0</v>
       </c>
       <c r="Q6">
         <f>M6-P6</f>
-        <v>1890.0</v>
+        <v>4936.0</v>
       </c>
     </row>
     <row r="7" ht="27.75" customHeight="1" s="331">
@@ -20041,33 +20074,72 @@
       <c r="AB137" s="292" t="n"/>
     </row>
     <row r="138" ht="16.5" customHeight="1" s="331">
-      <c r="B138" s="34" t="n"/>
-      <c r="C138" s="35" t="n"/>
-      <c r="D138" s="36" t="n"/>
-      <c r="E138" s="37" t="n"/>
-      <c r="F138" s="38" t="n"/>
-      <c r="G138" s="39" t="n"/>
-      <c r="H138" s="40" t="n"/>
-      <c r="I138" s="41" t="n"/>
-      <c r="J138" s="42" t="n"/>
-      <c r="K138" s="43" t="n"/>
-      <c r="L138" s="9" t="n"/>
-      <c r="M138" s="12" t="n"/>
-      <c r="N138" s="44" t="n"/>
-      <c r="O138" s="45" t="n"/>
-      <c r="P138" s="46" t="n"/>
-      <c r="Q138" s="44" t="n"/>
-      <c r="R138" s="44" t="n"/>
-      <c r="S138" s="44" t="n"/>
-      <c r="T138" s="44" t="n"/>
-      <c r="U138" s="44" t="n"/>
-      <c r="V138" s="44" t="n"/>
-      <c r="W138" s="44" t="n"/>
-      <c r="X138" s="44" t="n"/>
-      <c r="Y138" s="44" t="n"/>
-      <c r="Z138" s="44" t="n"/>
-      <c r="AA138" s="44" t="n"/>
-      <c r="AB138" s="44" t="n"/>
+      <c r="B138" s="427" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C138" s="270" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D138" s="271" t="n">
+        <v>2525</v>
+      </c>
+      <c r="E138" s="37" t="n">
+        <v>1790</v>
+      </c>
+      <c r="F138" s="38">
+        <f>IFERROR(D138+E138+G138+U138+Y138,0)</f>
+        <v>4435.0</v>
+      </c>
+      <c r="G138" s="272" t="n">
+        <v>120</v>
+      </c>
+      <c r="H138" s="273">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B138,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B138+1))</f>
+        <v>1389.0</v>
+      </c>
+      <c r="I138" s="274">
+        <f>IFERROR(F138-H138,0)</f>
+        <v>3046.0</v>
+      </c>
+      <c r="J138" s="275">
+        <f>IFERROR(I138/F138,0)</f>
+        <v>0.686809</v>
+      </c>
+      <c r="K138" s="250" t="n"/>
+      <c r="L138" s="276" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
+      <c r="M138" s="323" t="n"/>
+      <c r="N138" s="324" t="n"/>
+      <c r="O138" s="325" t="n"/>
+      <c r="P138" s="326" t="n"/>
+      <c r="Q138" s="324" t="n"/>
+      <c r="R138" s="428">
+        <f>IFERROR(D138*$T$7,0)</f>
+        <v>102.51</v>
+      </c>
+      <c r="S138" s="324" t="n"/>
+      <c r="T138" s="324" t="n"/>
+      <c r="U138" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="V138" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="W138" s="324" t="n"/>
+      <c r="X138" s="324" t="n"/>
+      <c r="Y138" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z138" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA138" s="324" t="n"/>
+      <c r="AB138" s="324" t="n"/>
     </row>
     <row r="139" ht="16.5" customHeight="1" s="331">
       <c r="B139" s="34" t="n"/>
@@ -26857,9 +26929,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="I2:P2"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="B5:P5"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="I2:P2"/>
     <mergeCell ref="A3:P3"/>
   </mergeCells>
   <conditionalFormatting sqref="I8:I372">
@@ -26882,7 +26954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J859"/>
+  <dimension ref="A1:J863"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="4" customWidth="1" style="331" min="1" max="1"/>
@@ -63320,6 +63392,178 @@
         </is>
       </c>
       <c r="J859" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="B860" s="429" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C860" s="297" t="inlineStr">
+        <is>
+          <t>Molino</t>
+        </is>
+      </c>
+      <c r="D860" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E860" s="297" t="inlineStr">
+        <is>
+          <t>Supermarket/General</t>
+        </is>
+      </c>
+      <c r="F860" s="299" t="n">
+        <v>116</v>
+      </c>
+      <c r="G860" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H860" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I860" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J860" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="B861" s="429" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C861" s="297" t="inlineStr">
+        <is>
+          <t>Carne</t>
+        </is>
+      </c>
+      <c r="D861" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E861" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat</t>
+        </is>
+      </c>
+      <c r="F861" s="299" t="n">
+        <v>826</v>
+      </c>
+      <c r="G861" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H861" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I861" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J861" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="B862" s="429" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C862" s="297" t="inlineStr">
+        <is>
+          <t>Carne Hamburguesa</t>
+        </is>
+      </c>
+      <c r="D862" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E862" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat</t>
+        </is>
+      </c>
+      <c r="F862" s="299" t="n">
+        <v>380</v>
+      </c>
+      <c r="G862" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H862" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I862" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J862" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="B863" s="429" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C863" s="297" t="inlineStr">
+        <is>
+          <t>Chedraui</t>
+        </is>
+      </c>
+      <c r="D863" s="298" t="inlineStr">
+        <is>
+          <t>Chedraui</t>
+        </is>
+      </c>
+      <c r="E863" s="297" t="inlineStr">
+        <is>
+          <t>Supermarket/General</t>
+        </is>
+      </c>
+      <c r="F863" s="299" t="n">
+        <v>67</v>
+      </c>
+      <c r="G863" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H863" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I863" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J863" s="423" t="inlineStr">
         <is>
           <t>No receipt; cash</t>
         </is>

</xml_diff>

<commit_message>
LOKA 14-Oct-2026 | EOD | day 2026-10-14: rev $2,270 exp $481 net $1,789 | bal vs capital $-18,139
Changed: LOKA_Restaurant_Manager.xlsx, dashboard.html, today.txt
+ 3 backup/day file(s)
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -5871,7 +5871,7 @@
         </is>
       </c>
       <c r="C172" s="455" t="n">
-        <v>-19890.4</v>
+        <v>-18138.96</v>
       </c>
       <c r="E172" s="423" t="inlineStr">
         <is>
@@ -5886,7 +5886,7 @@
         </is>
       </c>
       <c r="C173" s="457" t="n">
-        <v>106043.6</v>
+        <v>107795.04</v>
       </c>
       <c r="E173" s="423" t="inlineStr">
         <is>
@@ -11507,45 +11507,45 @@
       <c r="E6" s="29" t="n"/>
       <c r="F6" s="30">
         <f>SUMIFS($D$8:$D$5000,$B$8:$B$5000,TODAY())+SUMIFS($E$8:$E$5000,$B$8:$B$5000,TODAY())+SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())+SUMIFS($U$8:$U$5000,$B$8:$B$5000,TODAY())+SUMIFS($Y$8:$Y$5000,$B$8:$B$5000,TODAY())</f>
-        <v>4435.0</v>
+        <v>2270.0</v>
       </c>
       <c r="G6" s="31">
         <f>SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())</f>
-        <v>120.0</v>
+        <v>0.0</v>
       </c>
       <c r="H6" s="28">
         <f>SUMIFS($H$8:$H$5000,$B$8:$B$5000,TODAY())</f>
-        <v>1389.0</v>
+        <v>481.0</v>
       </c>
       <c r="I6" s="32">
         <f>F6-H6</f>
-        <v>3046.0</v>
+        <v>1789.0</v>
       </c>
       <c r="J6">
         <f>IFERROR(I6/F6,0)</f>
-        <v>0.686809</v>
+        <v>0.788106</v>
       </c>
       <c r="K6" s="28" t="n"/>
       <c r="L6" s="31" t="n"/>
       <c r="M6" s="28">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>9365.0</v>
+        <v>11635.0</v>
       </c>
       <c r="N6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>9365.0</v>
+        <v>11635.0</v>
       </c>
       <c r="O6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),$B$8:$B$5000,"&lt;"&amp;DATE(YEAR(TODAY()),MONTH(TODAY())+1,1))</f>
-        <v>39885.0</v>
+        <v>42155.0</v>
       </c>
       <c r="P6">
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>4429.0</v>
+        <v>4910.0</v>
       </c>
       <c r="Q6">
         <f>M6-P6</f>
-        <v>4936.0</v>
+        <v>6725.0</v>
       </c>
     </row>
     <row r="7" ht="27.75" customHeight="1" s="331">
@@ -20142,33 +20142,72 @@
       <c r="AB138" s="324" t="n"/>
     </row>
     <row r="139" ht="16.5" customHeight="1" s="331">
-      <c r="B139" s="34" t="n"/>
-      <c r="C139" s="47" t="n"/>
-      <c r="D139" s="48" t="n"/>
-      <c r="E139" s="49" t="n"/>
-      <c r="F139" s="50" t="n"/>
-      <c r="G139" s="51" t="n"/>
-      <c r="H139" s="52" t="n"/>
-      <c r="I139" s="53" t="n"/>
-      <c r="J139" s="54" t="n"/>
-      <c r="K139" s="55" t="n"/>
-      <c r="L139" s="18" t="n"/>
-      <c r="M139" s="21" t="n"/>
-      <c r="N139" s="56" t="n"/>
-      <c r="O139" s="57" t="n"/>
-      <c r="P139" s="58" t="n"/>
-      <c r="Q139" s="56" t="n"/>
-      <c r="R139" s="56" t="n"/>
-      <c r="S139" s="56" t="n"/>
-      <c r="T139" s="56" t="n"/>
-      <c r="U139" s="56" t="n"/>
-      <c r="V139" s="56" t="n"/>
-      <c r="W139" s="56" t="n"/>
-      <c r="X139" s="56" t="n"/>
-      <c r="Y139" s="56" t="n"/>
-      <c r="Z139" s="56" t="n"/>
-      <c r="AA139" s="56" t="n"/>
-      <c r="AB139" s="56" t="n"/>
+      <c r="B139" s="427" t="n">
+        <v>46309</v>
+      </c>
+      <c r="C139" s="255" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="D139" s="256" t="n">
+        <v>925</v>
+      </c>
+      <c r="E139" s="49" t="n">
+        <v>1345</v>
+      </c>
+      <c r="F139" s="50">
+        <f>IFERROR(D139+E139+G139+U139+Y139,0)</f>
+        <v>2270.0</v>
+      </c>
+      <c r="G139" s="257" t="n">
+        <v>0</v>
+      </c>
+      <c r="H139" s="258">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B139,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B139+1))</f>
+        <v>481.0</v>
+      </c>
+      <c r="I139" s="259">
+        <f>IFERROR(F139-H139,0)</f>
+        <v>1789.0</v>
+      </c>
+      <c r="J139" s="260">
+        <f>IFERROR(I139/F139,0)</f>
+        <v>0.788106</v>
+      </c>
+      <c r="K139" s="254" t="n"/>
+      <c r="L139" s="261" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
+      <c r="M139" s="291" t="n"/>
+      <c r="N139" s="292" t="n"/>
+      <c r="O139" s="293" t="n"/>
+      <c r="P139" s="294" t="n"/>
+      <c r="Q139" s="292" t="n"/>
+      <c r="R139" s="443">
+        <f>IFERROR(D139*$T$7,0)</f>
+        <v>37.55</v>
+      </c>
+      <c r="S139" s="292" t="n"/>
+      <c r="T139" s="292" t="n"/>
+      <c r="U139" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="V139" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="W139" s="292" t="n"/>
+      <c r="X139" s="292" t="n"/>
+      <c r="Y139" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z139" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA139" s="292" t="n"/>
+      <c r="AB139" s="292" t="n"/>
     </row>
     <row r="140" ht="16.5" customHeight="1" s="331">
       <c r="B140" s="34" t="n"/>
@@ -26929,9 +26968,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="B5:P5"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="I2:P2"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="B5:P5"/>
     <mergeCell ref="A3:P3"/>
   </mergeCells>
   <conditionalFormatting sqref="I8:I372">
@@ -26954,7 +26993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J863"/>
+  <dimension ref="A1:J866"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="4" customWidth="1" style="331" min="1" max="1"/>
@@ -63564,6 +63603,135 @@
         </is>
       </c>
       <c r="J863" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="B864" s="429" t="n">
+        <v>46309</v>
+      </c>
+      <c r="C864" s="297" t="inlineStr">
+        <is>
+          <t>Pescado</t>
+        </is>
+      </c>
+      <c r="D864" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E864" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat &amp; Fish</t>
+        </is>
+      </c>
+      <c r="F864" s="299" t="n">
+        <v>313</v>
+      </c>
+      <c r="G864" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H864" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I864" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J864" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="B865" s="429" t="n">
+        <v>46309</v>
+      </c>
+      <c r="C865" s="297" t="inlineStr">
+        <is>
+          <t>Molino</t>
+        </is>
+      </c>
+      <c r="D865" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E865" s="297" t="inlineStr">
+        <is>
+          <t>Supermarket/General</t>
+        </is>
+      </c>
+      <c r="F865" s="299" t="n">
+        <v>28</v>
+      </c>
+      <c r="G865" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H865" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I865" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J865" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="B866" s="429" t="n">
+        <v>46309</v>
+      </c>
+      <c r="C866" s="297" t="inlineStr">
+        <is>
+          <t>Vegetables</t>
+        </is>
+      </c>
+      <c r="D866" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E866" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Vegetables</t>
+        </is>
+      </c>
+      <c r="F866" s="299" t="n">
+        <v>140</v>
+      </c>
+      <c r="G866" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H866" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I866" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J866" s="423" t="inlineStr">
         <is>
           <t>No receipt; cash</t>
         </is>

</xml_diff>

<commit_message>
LOKA 21-Oct-2026 | EOD | day 2026-10-15: rev $3,975 exp $2,075 net $1,900 | bal vs capital $-16,346
Changed: LOKA_Restaurant_Manager.xlsx, dashboard.html, today.txt
+ 2 backup/day file(s)
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -5871,7 +5871,7 @@
         </is>
       </c>
       <c r="C172" s="455" t="n">
-        <v>-18138.96</v>
+        <v>-16345.53</v>
       </c>
       <c r="E172" s="423" t="inlineStr">
         <is>
@@ -5886,7 +5886,7 @@
         </is>
       </c>
       <c r="C173" s="457" t="n">
-        <v>107795.04</v>
+        <v>109588.47</v>
       </c>
       <c r="E173" s="423" t="inlineStr">
         <is>
@@ -11507,7 +11507,7 @@
       <c r="E6" s="29" t="n"/>
       <c r="F6" s="30">
         <f>SUMIFS($D$8:$D$5000,$B$8:$B$5000,TODAY())+SUMIFS($E$8:$E$5000,$B$8:$B$5000,TODAY())+SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())+SUMIFS($U$8:$U$5000,$B$8:$B$5000,TODAY())+SUMIFS($Y$8:$Y$5000,$B$8:$B$5000,TODAY())</f>
-        <v>2270.0</v>
+        <v>3975.0</v>
       </c>
       <c r="G6" s="31">
         <f>SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())</f>
@@ -11515,37 +11515,37 @@
       </c>
       <c r="H6" s="28">
         <f>SUMIFS($H$8:$H$5000,$B$8:$B$5000,TODAY())</f>
-        <v>481.0</v>
+        <v>2075.0</v>
       </c>
       <c r="I6" s="32">
         <f>F6-H6</f>
-        <v>1789.0</v>
+        <v>1900.0</v>
       </c>
       <c r="J6">
         <f>IFERROR(I6/F6,0)</f>
-        <v>0.788106</v>
+        <v>0.477987</v>
       </c>
       <c r="K6" s="28" t="n"/>
       <c r="L6" s="31" t="n"/>
       <c r="M6" s="28">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>11635.0</v>
+        <v>15610.0</v>
       </c>
       <c r="N6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>11635.0</v>
+        <v>15610.0</v>
       </c>
       <c r="O6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),$B$8:$B$5000,"&lt;"&amp;DATE(YEAR(TODAY()),MONTH(TODAY())+1,1))</f>
-        <v>42155.0</v>
+        <v>46130.0</v>
       </c>
       <c r="P6">
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>4910.0</v>
+        <v>6985.0</v>
       </c>
       <c r="Q6">
         <f>M6-P6</f>
-        <v>6725.0</v>
+        <v>8625.0</v>
       </c>
     </row>
     <row r="7" ht="27.75" customHeight="1" s="331">
@@ -20210,33 +20210,72 @@
       <c r="AB139" s="292" t="n"/>
     </row>
     <row r="140" ht="16.5" customHeight="1" s="331">
-      <c r="B140" s="34" t="n"/>
-      <c r="C140" s="35" t="n"/>
-      <c r="D140" s="36" t="n"/>
-      <c r="E140" s="37" t="n"/>
-      <c r="F140" s="38" t="n"/>
-      <c r="G140" s="39" t="n"/>
-      <c r="H140" s="40" t="n"/>
-      <c r="I140" s="41" t="n"/>
-      <c r="J140" s="42" t="n"/>
-      <c r="K140" s="43" t="n"/>
-      <c r="L140" s="9" t="n"/>
-      <c r="M140" s="12" t="n"/>
-      <c r="N140" s="44" t="n"/>
-      <c r="O140" s="45" t="n"/>
-      <c r="P140" s="46" t="n"/>
-      <c r="Q140" s="44" t="n"/>
-      <c r="R140" s="44" t="n"/>
-      <c r="S140" s="44" t="n"/>
-      <c r="T140" s="44" t="n"/>
-      <c r="U140" s="44" t="n"/>
-      <c r="V140" s="44" t="n"/>
-      <c r="W140" s="44" t="n"/>
-      <c r="X140" s="44" t="n"/>
-      <c r="Y140" s="44" t="n"/>
-      <c r="Z140" s="44" t="n"/>
-      <c r="AA140" s="44" t="n"/>
-      <c r="AB140" s="44" t="n"/>
+      <c r="B140" s="427" t="n">
+        <v>46310</v>
+      </c>
+      <c r="C140" s="270" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D140" s="271" t="n">
+        <v>2625</v>
+      </c>
+      <c r="E140" s="37" t="n">
+        <v>1350</v>
+      </c>
+      <c r="F140" s="38">
+        <f>IFERROR(D140+E140+G140+U140+Y140,0)</f>
+        <v>3975.0</v>
+      </c>
+      <c r="G140" s="272" t="n">
+        <v>0</v>
+      </c>
+      <c r="H140" s="273">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B140,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B140+1))</f>
+        <v>2075.0</v>
+      </c>
+      <c r="I140" s="274">
+        <f>IFERROR(F140-H140,0)</f>
+        <v>1900.0</v>
+      </c>
+      <c r="J140" s="275">
+        <f>IFERROR(I140/F140,0)</f>
+        <v>0.477987</v>
+      </c>
+      <c r="K140" s="250" t="n"/>
+      <c r="L140" s="276" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
+      <c r="M140" s="323" t="n"/>
+      <c r="N140" s="324" t="n"/>
+      <c r="O140" s="325" t="n"/>
+      <c r="P140" s="326" t="n"/>
+      <c r="Q140" s="324" t="n"/>
+      <c r="R140" s="428">
+        <f>IFERROR(D140*$T$7,0)</f>
+        <v>106.57</v>
+      </c>
+      <c r="S140" s="324" t="n"/>
+      <c r="T140" s="324" t="n"/>
+      <c r="U140" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="V140" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="W140" s="324" t="n"/>
+      <c r="X140" s="324" t="n"/>
+      <c r="Y140" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z140" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA140" s="324" t="n"/>
+      <c r="AB140" s="324" t="n"/>
     </row>
     <row r="141" ht="16.5" customHeight="1" s="331">
       <c r="B141" s="34" t="n"/>
@@ -26968,9 +27007,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="B5:P5"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="I2:P2"/>
+    <mergeCell ref="B5:P5"/>
     <mergeCell ref="A3:P3"/>
   </mergeCells>
   <conditionalFormatting sqref="I8:I372">
@@ -26993,7 +27032,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J866"/>
+  <dimension ref="A1:J870"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="4" customWidth="1" style="331" min="1" max="1"/>
@@ -63734,6 +63773,178 @@
       <c r="J866" s="423" t="inlineStr">
         <is>
           <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="B867" s="429" t="n">
+        <v>46310</v>
+      </c>
+      <c r="C867" s="297" t="inlineStr">
+        <is>
+          <t>Vegetables</t>
+        </is>
+      </c>
+      <c r="D867" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E867" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Vegetables</t>
+        </is>
+      </c>
+      <c r="F867" s="299" t="n">
+        <v>198</v>
+      </c>
+      <c r="G867" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H867" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I867" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J867" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="B868" s="429" t="n">
+        <v>46310</v>
+      </c>
+      <c r="C868" s="297" t="inlineStr">
+        <is>
+          <t>Carne</t>
+        </is>
+      </c>
+      <c r="D868" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E868" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat</t>
+        </is>
+      </c>
+      <c r="F868" s="299" t="n">
+        <v>378</v>
+      </c>
+      <c r="G868" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H868" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I868" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J868" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="B869" s="429" t="n">
+        <v>46310</v>
+      </c>
+      <c r="C869" s="297" t="inlineStr">
+        <is>
+          <t>Chedraui</t>
+        </is>
+      </c>
+      <c r="D869" s="298" t="inlineStr">
+        <is>
+          <t>Chedraui</t>
+        </is>
+      </c>
+      <c r="E869" s="297" t="inlineStr">
+        <is>
+          <t>Supermarket/General</t>
+        </is>
+      </c>
+      <c r="F869" s="299" t="n">
+        <v>149</v>
+      </c>
+      <c r="G869" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H869" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I869" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J869" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="B870" s="429" t="n">
+        <v>46310</v>
+      </c>
+      <c r="C870" s="297" t="inlineStr">
+        <is>
+          <t>Josias - salary</t>
+        </is>
+      </c>
+      <c r="D870" s="298" t="inlineStr">
+        <is>
+          <t>Payroll</t>
+        </is>
+      </c>
+      <c r="E870" s="297" t="inlineStr">
+        <is>
+          <t>Staff - Salary</t>
+        </is>
+      </c>
+      <c r="F870" s="299" t="n">
+        <v>1350</v>
+      </c>
+      <c r="G870" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H870" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I870" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J870" s="423" t="inlineStr">
+        <is>
+          <t>Weekly salary</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
LOKA 21-Oct-2026 | EOD | day 2026-10-16: rev $5,825 exp $1,420 net $4,405 | bal vs capital $-12,028
Changed: LOKA_Restaurant_Manager.xlsx, dashboard.html, today.txt
+ 3 backup/day file(s)
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -5871,7 +5871,7 @@
         </is>
       </c>
       <c r="C172" s="455" t="n">
-        <v>-16345.53</v>
+        <v>-12027.62</v>
       </c>
       <c r="E172" s="423" t="inlineStr">
         <is>
@@ -5886,7 +5886,7 @@
         </is>
       </c>
       <c r="C173" s="457" t="n">
-        <v>109588.47</v>
+        <v>113906.38</v>
       </c>
       <c r="E173" s="423" t="inlineStr">
         <is>
@@ -11507,7 +11507,7 @@
       <c r="E6" s="29" t="n"/>
       <c r="F6" s="30">
         <f>SUMIFS($D$8:$D$5000,$B$8:$B$5000,TODAY())+SUMIFS($E$8:$E$5000,$B$8:$B$5000,TODAY())+SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())+SUMIFS($U$8:$U$5000,$B$8:$B$5000,TODAY())+SUMIFS($Y$8:$Y$5000,$B$8:$B$5000,TODAY())</f>
-        <v>3975.0</v>
+        <v>5825.0</v>
       </c>
       <c r="G6" s="31">
         <f>SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())</f>
@@ -11515,37 +11515,37 @@
       </c>
       <c r="H6" s="28">
         <f>SUMIFS($H$8:$H$5000,$B$8:$B$5000,TODAY())</f>
-        <v>2075.0</v>
+        <v>1420.0</v>
       </c>
       <c r="I6" s="32">
         <f>F6-H6</f>
-        <v>1900.0</v>
+        <v>4405.0</v>
       </c>
       <c r="J6">
         <f>IFERROR(I6/F6,0)</f>
-        <v>0.477987</v>
+        <v>0.756223</v>
       </c>
       <c r="K6" s="28" t="n"/>
       <c r="L6" s="31" t="n"/>
       <c r="M6" s="28">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>15610.0</v>
+        <v>21435.0</v>
       </c>
       <c r="N6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>15610.0</v>
+        <v>21435.0</v>
       </c>
       <c r="O6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),$B$8:$B$5000,"&lt;"&amp;DATE(YEAR(TODAY()),MONTH(TODAY())+1,1))</f>
-        <v>46130.0</v>
+        <v>51955.0</v>
       </c>
       <c r="P6">
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>6985.0</v>
+        <v>8405.0</v>
       </c>
       <c r="Q6">
         <f>M6-P6</f>
-        <v>8625.0</v>
+        <v>13030.0</v>
       </c>
     </row>
     <row r="7" ht="27.75" customHeight="1" s="331">
@@ -20278,33 +20278,72 @@
       <c r="AB140" s="324" t="n"/>
     </row>
     <row r="141" ht="16.5" customHeight="1" s="331">
-      <c r="B141" s="34" t="n"/>
-      <c r="C141" s="47" t="n"/>
-      <c r="D141" s="48" t="n"/>
-      <c r="E141" s="49" t="n"/>
-      <c r="F141" s="50" t="n"/>
-      <c r="G141" s="51" t="n"/>
-      <c r="H141" s="52" t="n"/>
-      <c r="I141" s="53" t="n"/>
-      <c r="J141" s="54" t="n"/>
-      <c r="K141" s="55" t="n"/>
-      <c r="L141" s="18" t="n"/>
-      <c r="M141" s="21" t="n"/>
-      <c r="N141" s="56" t="n"/>
-      <c r="O141" s="57" t="n"/>
-      <c r="P141" s="58" t="n"/>
-      <c r="Q141" s="56" t="n"/>
-      <c r="R141" s="56" t="n"/>
-      <c r="S141" s="56" t="n"/>
-      <c r="T141" s="56" t="n"/>
-      <c r="U141" s="56" t="n"/>
-      <c r="V141" s="56" t="n"/>
-      <c r="W141" s="56" t="n"/>
-      <c r="X141" s="56" t="n"/>
-      <c r="Y141" s="56" t="n"/>
-      <c r="Z141" s="56" t="n"/>
-      <c r="AA141" s="56" t="n"/>
-      <c r="AB141" s="56" t="n"/>
+      <c r="B141" s="427" t="n">
+        <v>46311</v>
+      </c>
+      <c r="C141" s="255" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D141" s="256" t="n">
+        <v>2145</v>
+      </c>
+      <c r="E141" s="49" t="n">
+        <v>3680</v>
+      </c>
+      <c r="F141" s="50">
+        <f>IFERROR(D141+E141+G141+U141+Y141,0)</f>
+        <v>5825.0</v>
+      </c>
+      <c r="G141" s="257" t="n">
+        <v>0</v>
+      </c>
+      <c r="H141" s="258">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B141,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B141+1))</f>
+        <v>1420.0</v>
+      </c>
+      <c r="I141" s="259">
+        <f>IFERROR(F141-H141,0)</f>
+        <v>4405.0</v>
+      </c>
+      <c r="J141" s="260">
+        <f>IFERROR(I141/F141,0)</f>
+        <v>0.756223</v>
+      </c>
+      <c r="K141" s="254" t="n"/>
+      <c r="L141" s="261" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
+      <c r="M141" s="291" t="n"/>
+      <c r="N141" s="292" t="n"/>
+      <c r="O141" s="293" t="n"/>
+      <c r="P141" s="294" t="n"/>
+      <c r="Q141" s="292" t="n"/>
+      <c r="R141" s="443">
+        <f>IFERROR(D141*$T$7,0)</f>
+        <v>87.09</v>
+      </c>
+      <c r="S141" s="292" t="n"/>
+      <c r="T141" s="292" t="n"/>
+      <c r="U141" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="V141" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="W141" s="292" t="n"/>
+      <c r="X141" s="292" t="n"/>
+      <c r="Y141" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z141" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA141" s="292" t="n"/>
+      <c r="AB141" s="292" t="n"/>
     </row>
     <row r="142" ht="16.5" customHeight="1" s="331">
       <c r="B142" s="34" t="n"/>
@@ -27007,8 +27046,8 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="I2:P2"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="I2:P2"/>
     <mergeCell ref="B5:P5"/>
     <mergeCell ref="A3:P3"/>
   </mergeCells>
@@ -27032,7 +27071,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J870"/>
+  <dimension ref="A1:J872"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="4" customWidth="1" style="331" min="1" max="1"/>
@@ -63943,6 +63982,92 @@
         </is>
       </c>
       <c r="J870" s="423" t="inlineStr">
+        <is>
+          <t>Weekly salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="B871" s="429" t="n">
+        <v>46311</v>
+      </c>
+      <c r="C871" s="297" t="inlineStr">
+        <is>
+          <t>Vegetables</t>
+        </is>
+      </c>
+      <c r="D871" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E871" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Vegetables</t>
+        </is>
+      </c>
+      <c r="F871" s="299" t="n">
+        <v>120</v>
+      </c>
+      <c r="G871" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H871" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I871" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J871" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="B872" s="429" t="n">
+        <v>46311</v>
+      </c>
+      <c r="C872" s="297" t="inlineStr">
+        <is>
+          <t>Duvi - salary</t>
+        </is>
+      </c>
+      <c r="D872" s="298" t="inlineStr">
+        <is>
+          <t>Payroll</t>
+        </is>
+      </c>
+      <c r="E872" s="297" t="inlineStr">
+        <is>
+          <t>Staff - Salary</t>
+        </is>
+      </c>
+      <c r="F872" s="299" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G872" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H872" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I872" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J872" s="423" t="inlineStr">
         <is>
           <t>Weekly salary</t>
         </is>

</xml_diff>

<commit_message>
LOKA 21-Oct-2026 | EOD | day 2026-10-17: rev $4,515 exp $7,037 net $-2,522 | bal vs capital $-14,648
Changed: LOKA_Restaurant_Manager.xlsx, dashboard.html, today.txt
+ 3 backup/day file(s)
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -5871,7 +5871,7 @@
         </is>
       </c>
       <c r="C172" s="455" t="n">
-        <v>-12027.62</v>
+        <v>-14648.07</v>
       </c>
       <c r="E172" s="423" t="inlineStr">
         <is>
@@ -5886,7 +5886,7 @@
         </is>
       </c>
       <c r="C173" s="457" t="n">
-        <v>113906.38</v>
+        <v>111285.93</v>
       </c>
       <c r="E173" s="423" t="inlineStr">
         <is>
@@ -11507,7 +11507,7 @@
       <c r="E6" s="29" t="n"/>
       <c r="F6" s="30">
         <f>SUMIFS($D$8:$D$5000,$B$8:$B$5000,TODAY())+SUMIFS($E$8:$E$5000,$B$8:$B$5000,TODAY())+SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())+SUMIFS($U$8:$U$5000,$B$8:$B$5000,TODAY())+SUMIFS($Y$8:$Y$5000,$B$8:$B$5000,TODAY())</f>
-        <v>5825.0</v>
+        <v>4515.0</v>
       </c>
       <c r="G6" s="31">
         <f>SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())</f>
@@ -11515,37 +11515,37 @@
       </c>
       <c r="H6" s="28">
         <f>SUMIFS($H$8:$H$5000,$B$8:$B$5000,TODAY())</f>
-        <v>1420.0</v>
+        <v>7037.0</v>
       </c>
       <c r="I6" s="32">
         <f>F6-H6</f>
-        <v>4405.0</v>
+        <v>-2522.0</v>
       </c>
       <c r="J6">
         <f>IFERROR(I6/F6,0)</f>
-        <v>0.756223</v>
+        <v>-0.558583</v>
       </c>
       <c r="K6" s="28" t="n"/>
       <c r="L6" s="31" t="n"/>
       <c r="M6" s="28">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>21435.0</v>
+        <v>25950.0</v>
       </c>
       <c r="N6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>21435.0</v>
+        <v>25950.0</v>
       </c>
       <c r="O6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),$B$8:$B$5000,"&lt;"&amp;DATE(YEAR(TODAY()),MONTH(TODAY())+1,1))</f>
-        <v>51955.0</v>
+        <v>56470.0</v>
       </c>
       <c r="P6">
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>8405.0</v>
+        <v>15442.0</v>
       </c>
       <c r="Q6">
         <f>M6-P6</f>
-        <v>13030.0</v>
+        <v>10508.0</v>
       </c>
     </row>
     <row r="7" ht="27.75" customHeight="1" s="331">
@@ -20346,33 +20346,72 @@
       <c r="AB141" s="292" t="n"/>
     </row>
     <row r="142" ht="16.5" customHeight="1" s="331">
-      <c r="B142" s="34" t="n"/>
-      <c r="C142" s="35" t="n"/>
-      <c r="D142" s="36" t="n"/>
-      <c r="E142" s="37" t="n"/>
-      <c r="F142" s="38" t="n"/>
-      <c r="G142" s="39" t="n"/>
-      <c r="H142" s="40" t="n"/>
-      <c r="I142" s="41" t="n"/>
-      <c r="J142" s="42" t="n"/>
-      <c r="K142" s="43" t="n"/>
-      <c r="L142" s="9" t="n"/>
-      <c r="M142" s="12" t="n"/>
-      <c r="N142" s="44" t="n"/>
-      <c r="O142" s="45" t="n"/>
-      <c r="P142" s="46" t="n"/>
-      <c r="Q142" s="44" t="n"/>
-      <c r="R142" s="44" t="n"/>
-      <c r="S142" s="44" t="n"/>
-      <c r="T142" s="44" t="n"/>
-      <c r="U142" s="44" t="n"/>
-      <c r="V142" s="44" t="n"/>
-      <c r="W142" s="44" t="n"/>
-      <c r="X142" s="44" t="n"/>
-      <c r="Y142" s="44" t="n"/>
-      <c r="Z142" s="44" t="n"/>
-      <c r="AA142" s="44" t="n"/>
-      <c r="AB142" s="44" t="n"/>
+      <c r="B142" s="427" t="n">
+        <v>46312</v>
+      </c>
+      <c r="C142" s="270" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="D142" s="271" t="n">
+        <v>2425</v>
+      </c>
+      <c r="E142" s="37" t="n">
+        <v>2090</v>
+      </c>
+      <c r="F142" s="38">
+        <f>IFERROR(D142+E142+G142+U142+Y142,0)</f>
+        <v>4515.0</v>
+      </c>
+      <c r="G142" s="272" t="n">
+        <v>0</v>
+      </c>
+      <c r="H142" s="273">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B142,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B142+1))</f>
+        <v>7037.0</v>
+      </c>
+      <c r="I142" s="274">
+        <f>IFERROR(F142-H142,0)</f>
+        <v>-2522.0</v>
+      </c>
+      <c r="J142" s="275">
+        <f>IFERROR(I142/F142,0)</f>
+        <v>-0.558583</v>
+      </c>
+      <c r="K142" s="250" t="n"/>
+      <c r="L142" s="276" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
+      <c r="M142" s="323" t="n"/>
+      <c r="N142" s="324" t="n"/>
+      <c r="O142" s="325" t="n"/>
+      <c r="P142" s="326" t="n"/>
+      <c r="Q142" s="324" t="n"/>
+      <c r="R142" s="428">
+        <f>IFERROR(D142*$T$7,0)</f>
+        <v>98.45</v>
+      </c>
+      <c r="S142" s="324" t="n"/>
+      <c r="T142" s="324" t="n"/>
+      <c r="U142" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="V142" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="W142" s="324" t="n"/>
+      <c r="X142" s="324" t="n"/>
+      <c r="Y142" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z142" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA142" s="324" t="n"/>
+      <c r="AB142" s="324" t="n"/>
     </row>
     <row r="143" ht="16.5" customHeight="1" s="331">
       <c r="B143" s="34" t="n"/>
@@ -27046,9 +27085,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="B5:P5"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="I2:P2"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="B5:P5"/>
     <mergeCell ref="A3:P3"/>
   </mergeCells>
   <conditionalFormatting sqref="I8:I372">
@@ -27071,7 +27110,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J872"/>
+  <dimension ref="A1:J876"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="4" customWidth="1" style="331" min="1" max="1"/>
@@ -64068,6 +64107,178 @@
         </is>
       </c>
       <c r="J872" s="423" t="inlineStr">
+        <is>
+          <t>Weekly salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="B873" s="429" t="n">
+        <v>46312</v>
+      </c>
+      <c r="C873" s="297" t="inlineStr">
+        <is>
+          <t>Hielo</t>
+        </is>
+      </c>
+      <c r="D873" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E873" s="297" t="inlineStr">
+        <is>
+          <t>Kitchen Supplies</t>
+        </is>
+      </c>
+      <c r="F873" s="299" t="n">
+        <v>125</v>
+      </c>
+      <c r="G873" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H873" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I873" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J873" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="B874" s="429" t="n">
+        <v>46312</v>
+      </c>
+      <c r="C874" s="297" t="inlineStr">
+        <is>
+          <t>Vegetables</t>
+        </is>
+      </c>
+      <c r="D874" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E874" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Vegetables</t>
+        </is>
+      </c>
+      <c r="F874" s="299" t="n">
+        <v>1662</v>
+      </c>
+      <c r="G874" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H874" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I874" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J874" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="B875" s="429" t="n">
+        <v>46312</v>
+      </c>
+      <c r="C875" s="297" t="inlineStr">
+        <is>
+          <t>Jhon - salary</t>
+        </is>
+      </c>
+      <c r="D875" s="298" t="inlineStr">
+        <is>
+          <t>Payroll</t>
+        </is>
+      </c>
+      <c r="E875" s="297" t="inlineStr">
+        <is>
+          <t>Staff - Salary</t>
+        </is>
+      </c>
+      <c r="F875" s="299" t="n">
+        <v>3750</v>
+      </c>
+      <c r="G875" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H875" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I875" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J875" s="423" t="inlineStr">
+        <is>
+          <t>Weekly salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="B876" s="429" t="n">
+        <v>46312</v>
+      </c>
+      <c r="C876" s="297" t="inlineStr">
+        <is>
+          <t>Rodrigo - salary</t>
+        </is>
+      </c>
+      <c r="D876" s="298" t="inlineStr">
+        <is>
+          <t>Payroll</t>
+        </is>
+      </c>
+      <c r="E876" s="297" t="inlineStr">
+        <is>
+          <t>Staff - Salary</t>
+        </is>
+      </c>
+      <c r="F876" s="299" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G876" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H876" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I876" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J876" s="423" t="inlineStr">
         <is>
           <t>Weekly salary</t>
         </is>

</xml_diff>

<commit_message>
LOKA 21-Oct-2026 | EOD | day 2026-10-19: rev $5,685 exp $1,402 net $4,283 | bal vs capital $-10,139
Changed: LOKA_Restaurant_Manager.xlsx, dashboard.html, loka.py, today.txt
+ 3 backup/day file(s)
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -5871,7 +5871,7 @@
         </is>
       </c>
       <c r="C172" s="455" t="n">
-        <v>-14648.07</v>
+        <v>-10139.3</v>
       </c>
       <c r="E172" s="423" t="inlineStr">
         <is>
@@ -5886,7 +5886,7 @@
         </is>
       </c>
       <c r="C173" s="457" t="n">
-        <v>111285.93</v>
+        <v>115794.7</v>
       </c>
       <c r="E173" s="423" t="inlineStr">
         <is>
@@ -6057,7 +6057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H111"/>
+  <dimension ref="A1:H112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" style="331" min="1" max="1"/>
@@ -9650,30 +9650,63 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="430" t="inlineStr">
+      <c r="A111" s="430" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B111" s="232" t="inlineStr">
+        <is>
+          <t>Telmex $349 (paid by Lohith)</t>
+        </is>
+      </c>
+      <c r="C111" s="232" t="inlineStr">
+        <is>
+          <t>Expense - Personal</t>
+        </is>
+      </c>
+      <c r="D111" s="232" t="n">
+        <v>349</v>
+      </c>
+      <c r="E111" s="233" t="n"/>
+      <c r="F111" s="233">
+        <f>IFERROR(F110+D111-E111,0)</f>
+        <v/>
+      </c>
+      <c r="G111" s="232" t="inlineStr">
+        <is>
+          <t>⏳ Reimburse</t>
+        </is>
+      </c>
+      <c r="H111" s="232" t="inlineStr">
+        <is>
+          <t>Fronted from own pocket; excluded from till via cash_adjust</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="430" t="inlineStr">
         <is>
           <t>TOTALS &amp; CURRENT BALANCE</t>
         </is>
       </c>
-      <c r="B111" s="232" t="n"/>
-      <c r="C111" s="232" t="n"/>
-      <c r="D111" s="232">
-        <f>SUM(D4:D110)</f>
-        <v/>
-      </c>
-      <c r="E111" s="233">
-        <f>SUM(E4:E110)</f>
-        <v/>
-      </c>
-      <c r="F111" s="233">
-        <f>F110</f>
-        <v/>
-      </c>
-      <c r="G111" s="232">
-        <f>IF(F110&gt;0,"Restaurant owes Lohith $"&amp;TEXT(F110,"#,##0"),IF(F110&lt;0,"Lohith holds $"&amp;TEXT(ABS(F110),"#,##0"),"Zero balance"))</f>
-        <v/>
-      </c>
-      <c r="H111" s="232" t="n"/>
+      <c r="B112" s="232" t="n"/>
+      <c r="C112" s="232" t="n"/>
+      <c r="D112" s="232">
+        <f>SUM(D4:D111)</f>
+        <v/>
+      </c>
+      <c r="E112" s="233">
+        <f>SUM(E4:E111)</f>
+        <v/>
+      </c>
+      <c r="F112" s="233">
+        <f>F111</f>
+        <v/>
+      </c>
+      <c r="G112" s="232">
+        <f>IF(F111&gt;0,"Restaurant owes Lohith $"&amp;TEXT(F111,"#,##0"),IF(F111&lt;0,"Lohith holds $"&amp;TEXT(ABS(F111),"#,##0"),"Zero balance"))</f>
+        <v/>
+      </c>
+      <c r="H112" s="232" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -11507,7 +11540,7 @@
       <c r="E6" s="29" t="n"/>
       <c r="F6" s="30">
         <f>SUMIFS($D$8:$D$5000,$B$8:$B$5000,TODAY())+SUMIFS($E$8:$E$5000,$B$8:$B$5000,TODAY())+SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())+SUMIFS($U$8:$U$5000,$B$8:$B$5000,TODAY())+SUMIFS($Y$8:$Y$5000,$B$8:$B$5000,TODAY())</f>
-        <v>4515.0</v>
+        <v>5685.0</v>
       </c>
       <c r="G6" s="31">
         <f>SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())</f>
@@ -11515,37 +11548,37 @@
       </c>
       <c r="H6" s="28">
         <f>SUMIFS($H$8:$H$5000,$B$8:$B$5000,TODAY())</f>
-        <v>7037.0</v>
+        <v>1402.0</v>
       </c>
       <c r="I6" s="32">
         <f>F6-H6</f>
-        <v>-2522.0</v>
+        <v>4283.0</v>
       </c>
       <c r="J6">
         <f>IFERROR(I6/F6,0)</f>
-        <v>-0.558583</v>
+        <v>0.753386</v>
       </c>
       <c r="K6" s="28" t="n"/>
       <c r="L6" s="31" t="n"/>
       <c r="M6" s="28">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>25950.0</v>
+        <v>5685.0</v>
       </c>
       <c r="N6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>25950.0</v>
+        <v>5685.0</v>
       </c>
       <c r="O6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),$B$8:$B$5000,"&lt;"&amp;DATE(YEAR(TODAY()),MONTH(TODAY())+1,1))</f>
-        <v>56470.0</v>
+        <v>62155.0</v>
       </c>
       <c r="P6">
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>15442.0</v>
+        <v>1402.0</v>
       </c>
       <c r="Q6">
         <f>M6-P6</f>
-        <v>10508.0</v>
+        <v>4283.0</v>
       </c>
     </row>
     <row r="7" ht="27.75" customHeight="1" s="331">
@@ -20414,33 +20447,72 @@
       <c r="AB142" s="324" t="n"/>
     </row>
     <row r="143" ht="16.5" customHeight="1" s="331">
-      <c r="B143" s="34" t="n"/>
-      <c r="C143" s="47" t="n"/>
-      <c r="D143" s="48" t="n"/>
-      <c r="E143" s="49" t="n"/>
-      <c r="F143" s="50" t="n"/>
-      <c r="G143" s="51" t="n"/>
-      <c r="H143" s="52" t="n"/>
-      <c r="I143" s="53" t="n"/>
-      <c r="J143" s="54" t="n"/>
-      <c r="K143" s="55" t="n"/>
-      <c r="L143" s="18" t="n"/>
-      <c r="M143" s="21" t="n"/>
-      <c r="N143" s="56" t="n"/>
-      <c r="O143" s="57" t="n"/>
-      <c r="P143" s="58" t="n"/>
-      <c r="Q143" s="56" t="n"/>
-      <c r="R143" s="56" t="n"/>
-      <c r="S143" s="56" t="n"/>
-      <c r="T143" s="56" t="n"/>
-      <c r="U143" s="56" t="n"/>
-      <c r="V143" s="56" t="n"/>
-      <c r="W143" s="56" t="n"/>
-      <c r="X143" s="56" t="n"/>
-      <c r="Y143" s="56" t="n"/>
-      <c r="Z143" s="56" t="n"/>
-      <c r="AA143" s="56" t="n"/>
-      <c r="AB143" s="56" t="n"/>
+      <c r="B143" s="427" t="n">
+        <v>46314</v>
+      </c>
+      <c r="C143" s="255" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D143" s="256" t="n">
+        <v>3035</v>
+      </c>
+      <c r="E143" s="49" t="n">
+        <v>2650</v>
+      </c>
+      <c r="F143" s="50">
+        <f>IFERROR(D143+E143+G143+U143+Y143,0)</f>
+        <v>5685.0</v>
+      </c>
+      <c r="G143" s="257" t="n">
+        <v>0</v>
+      </c>
+      <c r="H143" s="258">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B143,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B143+1))</f>
+        <v>1402.0</v>
+      </c>
+      <c r="I143" s="259">
+        <f>IFERROR(F143-H143,0)</f>
+        <v>4283.0</v>
+      </c>
+      <c r="J143" s="260">
+        <f>IFERROR(I143/F143,0)</f>
+        <v>0.753386</v>
+      </c>
+      <c r="K143" s="254" t="n"/>
+      <c r="L143" s="261" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
+      <c r="M143" s="291" t="n"/>
+      <c r="N143" s="292" t="n"/>
+      <c r="O143" s="293" t="n"/>
+      <c r="P143" s="294" t="n"/>
+      <c r="Q143" s="292" t="n"/>
+      <c r="R143" s="443">
+        <f>IFERROR(D143*$T$7,0)</f>
+        <v>123.22</v>
+      </c>
+      <c r="S143" s="292" t="n"/>
+      <c r="T143" s="292" t="n"/>
+      <c r="U143" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="V143" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="W143" s="292" t="n"/>
+      <c r="X143" s="292" t="n"/>
+      <c r="Y143" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z143" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA143" s="292" t="n"/>
+      <c r="AB143" s="292" t="n"/>
     </row>
     <row r="144" ht="16.5" customHeight="1" s="331">
       <c r="B144" s="34" t="n"/>
@@ -27085,9 +27157,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="I2:P2"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="B5:P5"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="I2:P2"/>
     <mergeCell ref="A3:P3"/>
   </mergeCells>
   <conditionalFormatting sqref="I8:I372">
@@ -27110,7 +27182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J876"/>
+  <dimension ref="A1:J882"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="4" customWidth="1" style="331" min="1" max="1"/>
@@ -64281,6 +64353,264 @@
       <c r="J876" s="423" t="inlineStr">
         <is>
           <t>Weekly salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="877">
+      <c r="B877" s="429" t="n">
+        <v>46314</v>
+      </c>
+      <c r="C877" s="297" t="inlineStr">
+        <is>
+          <t>Pan Dulce</t>
+        </is>
+      </c>
+      <c r="D877" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E877" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Bread</t>
+        </is>
+      </c>
+      <c r="F877" s="299" t="n">
+        <v>80</v>
+      </c>
+      <c r="G877" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H877" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I877" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J877" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="878">
+      <c r="B878" s="429" t="n">
+        <v>46314</v>
+      </c>
+      <c r="C878" s="297" t="inlineStr">
+        <is>
+          <t>Tortillas</t>
+        </is>
+      </c>
+      <c r="D878" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E878" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Bread</t>
+        </is>
+      </c>
+      <c r="F878" s="299" t="n">
+        <v>27</v>
+      </c>
+      <c r="G878" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H878" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I878" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J878" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="879">
+      <c r="B879" s="429" t="n">
+        <v>46314</v>
+      </c>
+      <c r="C879" s="297" t="inlineStr">
+        <is>
+          <t>Carne</t>
+        </is>
+      </c>
+      <c r="D879" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E879" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat</t>
+        </is>
+      </c>
+      <c r="F879" s="299" t="n">
+        <v>771</v>
+      </c>
+      <c r="G879" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H879" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I879" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J879" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="B880" s="429" t="n">
+        <v>46314</v>
+      </c>
+      <c r="C880" s="297" t="inlineStr">
+        <is>
+          <t>Guimar</t>
+        </is>
+      </c>
+      <c r="D880" s="298" t="inlineStr">
+        <is>
+          <t>Guimar Polietilenos</t>
+        </is>
+      </c>
+      <c r="E880" s="297" t="inlineStr">
+        <is>
+          <t>Packaging/Disposables</t>
+        </is>
+      </c>
+      <c r="F880" s="299" t="n">
+        <v>108</v>
+      </c>
+      <c r="G880" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H880" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I880" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J880" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="881">
+      <c r="B881" s="429" t="n">
+        <v>46314</v>
+      </c>
+      <c r="C881" s="297" t="inlineStr">
+        <is>
+          <t>Oxxo Arroz</t>
+        </is>
+      </c>
+      <c r="D881" s="298" t="inlineStr">
+        <is>
+          <t>OXXO</t>
+        </is>
+      </c>
+      <c r="E881" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Pantry</t>
+        </is>
+      </c>
+      <c r="F881" s="299" t="n">
+        <v>67</v>
+      </c>
+      <c r="G881" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H881" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I881" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J881" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="882">
+      <c r="B882" s="429" t="n">
+        <v>46314</v>
+      </c>
+      <c r="C882" s="297" t="inlineStr">
+        <is>
+          <t>Telmex</t>
+        </is>
+      </c>
+      <c r="D882" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E882" s="297" t="inlineStr">
+        <is>
+          <t>Utilities/Internet</t>
+        </is>
+      </c>
+      <c r="F882" s="299" t="n">
+        <v>349</v>
+      </c>
+      <c r="G882" s="300" t="inlineStr">
+        <is>
+          <t>Lohith</t>
+        </is>
+      </c>
+      <c r="H882" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I882" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J882" s="423" t="inlineStr">
+        <is>
+          <t>Pagado por Lohith (bolsillo); reembolsable via Owner Ledger</t>
         </is>
       </c>
     </row>
@@ -75585,7 +75915,7 @@
     <row r="36">
       <c r="A36" s="439" t="inlineStr">
         <is>
-          <t>Software/Subscription</t>
+          <t>Utilities/Internet</t>
         </is>
       </c>
       <c r="B36" s="437">
@@ -75621,7 +75951,7 @@
     <row r="37">
       <c r="A37" s="439" t="inlineStr">
         <is>
-          <t>Utilities/Internet</t>
+          <t>Software/Subscription</t>
         </is>
       </c>
       <c r="B37" s="437">

</xml_diff>

<commit_message>
LOKA 21-Oct-2026 | EOD | day 2026-10-20: rev $4,395 exp $11,580 net $-7,185 | bal vs capital $-16,094
Changed: LOKA_Restaurant_Manager.xlsx, dashboard.html, loka.py, today.txt
+ 3 backup/day file(s)
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -5871,7 +5871,7 @@
         </is>
       </c>
       <c r="C172" s="455" t="n">
-        <v>-10139.3</v>
+        <v>-16094.43</v>
       </c>
       <c r="E172" s="423" t="inlineStr">
         <is>
@@ -5886,7 +5886,7 @@
         </is>
       </c>
       <c r="C173" s="457" t="n">
-        <v>115794.7</v>
+        <v>109839.57</v>
       </c>
       <c r="E173" s="423" t="inlineStr">
         <is>
@@ -6057,7 +6057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H112"/>
+  <dimension ref="A1:H113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" style="331" min="1" max="1"/>
@@ -9683,30 +9683,63 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="430" t="inlineStr">
+      <c r="A112" s="430" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B112" s="232" t="inlineStr">
+        <is>
+          <t>Pollo $1,334 (paid by Lohith)</t>
+        </is>
+      </c>
+      <c r="C112" s="232" t="inlineStr">
+        <is>
+          <t>Expense - Personal</t>
+        </is>
+      </c>
+      <c r="D112" s="232" t="n">
+        <v>1334</v>
+      </c>
+      <c r="E112" s="233" t="n"/>
+      <c r="F112" s="233">
+        <f>IFERROR(F111+D112-E112,0)</f>
+        <v/>
+      </c>
+      <c r="G112" s="232" t="inlineStr">
+        <is>
+          <t>⏳ Reimburse</t>
+        </is>
+      </c>
+      <c r="H112" s="232" t="inlineStr">
+        <is>
+          <t>Fronted from own pocket; excluded from till via cash_adjust</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="430" t="inlineStr">
         <is>
           <t>TOTALS &amp; CURRENT BALANCE</t>
         </is>
       </c>
-      <c r="B112" s="232" t="n"/>
-      <c r="C112" s="232" t="n"/>
-      <c r="D112" s="232">
-        <f>SUM(D4:D111)</f>
-        <v/>
-      </c>
-      <c r="E112" s="233">
-        <f>SUM(E4:E111)</f>
-        <v/>
-      </c>
-      <c r="F112" s="233">
-        <f>F111</f>
-        <v/>
-      </c>
-      <c r="G112" s="232">
-        <f>IF(F111&gt;0,"Restaurant owes Lohith $"&amp;TEXT(F111,"#,##0"),IF(F111&lt;0,"Lohith holds $"&amp;TEXT(ABS(F111),"#,##0"),"Zero balance"))</f>
-        <v/>
-      </c>
-      <c r="H112" s="232" t="n"/>
+      <c r="B113" s="232" t="n"/>
+      <c r="C113" s="232" t="n"/>
+      <c r="D113" s="232">
+        <f>SUM(D4:D112)</f>
+        <v/>
+      </c>
+      <c r="E113" s="233">
+        <f>SUM(E4:E112)</f>
+        <v/>
+      </c>
+      <c r="F113" s="233">
+        <f>F112</f>
+        <v/>
+      </c>
+      <c r="G113" s="232">
+        <f>IF(F112&gt;0,"Restaurant owes Lohith $"&amp;TEXT(F112,"#,##0"),IF(F112&lt;0,"Lohith holds $"&amp;TEXT(ABS(F112),"#,##0"),"Zero balance"))</f>
+        <v/>
+      </c>
+      <c r="H113" s="232" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -11540,7 +11573,7 @@
       <c r="E6" s="29" t="n"/>
       <c r="F6" s="30">
         <f>SUMIFS($D$8:$D$5000,$B$8:$B$5000,TODAY())+SUMIFS($E$8:$E$5000,$B$8:$B$5000,TODAY())+SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())+SUMIFS($U$8:$U$5000,$B$8:$B$5000,TODAY())+SUMIFS($Y$8:$Y$5000,$B$8:$B$5000,TODAY())</f>
-        <v>5685.0</v>
+        <v>4395.0</v>
       </c>
       <c r="G6" s="31">
         <f>SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())</f>
@@ -11548,37 +11581,37 @@
       </c>
       <c r="H6" s="28">
         <f>SUMIFS($H$8:$H$5000,$B$8:$B$5000,TODAY())</f>
-        <v>1402.0</v>
+        <v>11580.0</v>
       </c>
       <c r="I6" s="32">
         <f>F6-H6</f>
-        <v>4283.0</v>
+        <v>-7185.0</v>
       </c>
       <c r="J6">
         <f>IFERROR(I6/F6,0)</f>
-        <v>0.753386</v>
+        <v>-1.634812</v>
       </c>
       <c r="K6" s="28" t="n"/>
       <c r="L6" s="31" t="n"/>
       <c r="M6" s="28">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>5685.0</v>
+        <v>10080.0</v>
       </c>
       <c r="N6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>5685.0</v>
+        <v>10080.0</v>
       </c>
       <c r="O6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),$B$8:$B$5000,"&lt;"&amp;DATE(YEAR(TODAY()),MONTH(TODAY())+1,1))</f>
-        <v>62155.0</v>
+        <v>66550.0</v>
       </c>
       <c r="P6">
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>1402.0</v>
+        <v>12982.0</v>
       </c>
       <c r="Q6">
         <f>M6-P6</f>
-        <v>4283.0</v>
+        <v>-2902.0</v>
       </c>
     </row>
     <row r="7" ht="27.75" customHeight="1" s="331">
@@ -20515,33 +20548,72 @@
       <c r="AB143" s="292" t="n"/>
     </row>
     <row r="144" ht="16.5" customHeight="1" s="331">
-      <c r="B144" s="34" t="n"/>
-      <c r="C144" s="35" t="n"/>
-      <c r="D144" s="36" t="n"/>
-      <c r="E144" s="37" t="n"/>
-      <c r="F144" s="38" t="n"/>
-      <c r="G144" s="39" t="n"/>
-      <c r="H144" s="40" t="n"/>
-      <c r="I144" s="41" t="n"/>
-      <c r="J144" s="42" t="n"/>
-      <c r="K144" s="43" t="n"/>
-      <c r="L144" s="9" t="n"/>
-      <c r="M144" s="12" t="n"/>
-      <c r="N144" s="44" t="n"/>
-      <c r="O144" s="45" t="n"/>
-      <c r="P144" s="46" t="n"/>
-      <c r="Q144" s="44" t="n"/>
-      <c r="R144" s="44" t="n"/>
-      <c r="S144" s="44" t="n"/>
-      <c r="T144" s="44" t="n"/>
-      <c r="U144" s="44" t="n"/>
-      <c r="V144" s="44" t="n"/>
-      <c r="W144" s="44" t="n"/>
-      <c r="X144" s="44" t="n"/>
-      <c r="Y144" s="44" t="n"/>
-      <c r="Z144" s="44" t="n"/>
-      <c r="AA144" s="44" t="n"/>
-      <c r="AB144" s="44" t="n"/>
+      <c r="B144" s="427" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C144" s="270" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D144" s="271" t="n">
+        <v>2565</v>
+      </c>
+      <c r="E144" s="37" t="n">
+        <v>1830</v>
+      </c>
+      <c r="F144" s="38">
+        <f>IFERROR(D144+E144+G144+U144+Y144,0)</f>
+        <v>4395.0</v>
+      </c>
+      <c r="G144" s="272" t="n">
+        <v>0</v>
+      </c>
+      <c r="H144" s="273">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B144,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B144+1))</f>
+        <v>11580.0</v>
+      </c>
+      <c r="I144" s="274">
+        <f>IFERROR(F144-H144,0)</f>
+        <v>-7185.0</v>
+      </c>
+      <c r="J144" s="275">
+        <f>IFERROR(I144/F144,0)</f>
+        <v>-1.634812</v>
+      </c>
+      <c r="K144" s="250" t="n"/>
+      <c r="L144" s="276" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
+      <c r="M144" s="323" t="n"/>
+      <c r="N144" s="324" t="n"/>
+      <c r="O144" s="325" t="n"/>
+      <c r="P144" s="326" t="n"/>
+      <c r="Q144" s="324" t="n"/>
+      <c r="R144" s="428">
+        <f>IFERROR(D144*$T$7,0)</f>
+        <v>104.14</v>
+      </c>
+      <c r="S144" s="324" t="n"/>
+      <c r="T144" s="324" t="n"/>
+      <c r="U144" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="V144" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="W144" s="324" t="n"/>
+      <c r="X144" s="324" t="n"/>
+      <c r="Y144" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z144" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA144" s="324" t="n"/>
+      <c r="AB144" s="324" t="n"/>
     </row>
     <row r="145" ht="16.5" customHeight="1" s="331">
       <c r="B145" s="34" t="n"/>
@@ -27157,8 +27229,8 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="I2:P2"/>
-    <mergeCell ref="A2:H2"/>
     <mergeCell ref="B5:P5"/>
     <mergeCell ref="A3:P3"/>
   </mergeCells>
@@ -27182,7 +27254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J882"/>
+  <dimension ref="A1:J891"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="4" customWidth="1" style="331" min="1" max="1"/>
@@ -64609,6 +64681,393 @@
         </is>
       </c>
       <c r="J882" s="423" t="inlineStr">
+        <is>
+          <t>Pagado por Lohith (bolsillo); reembolsable via Owner Ledger</t>
+        </is>
+      </c>
+    </row>
+    <row r="883">
+      <c r="B883" s="429" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C883" s="297" t="inlineStr">
+        <is>
+          <t>Oxxo Arroz</t>
+        </is>
+      </c>
+      <c r="D883" s="298" t="inlineStr">
+        <is>
+          <t>OXXO</t>
+        </is>
+      </c>
+      <c r="E883" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Pantry</t>
+        </is>
+      </c>
+      <c r="F883" s="299" t="n">
+        <v>260</v>
+      </c>
+      <c r="G883" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H883" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I883" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J883" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="884">
+      <c r="B884" s="429" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C884" s="297" t="inlineStr">
+        <is>
+          <t>Oxxo Arroz</t>
+        </is>
+      </c>
+      <c r="D884" s="298" t="inlineStr">
+        <is>
+          <t>OXXO</t>
+        </is>
+      </c>
+      <c r="E884" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Pantry</t>
+        </is>
+      </c>
+      <c r="F884" s="299" t="n">
+        <v>26</v>
+      </c>
+      <c r="G884" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H884" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I884" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J884" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="885">
+      <c r="B885" s="429" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C885" s="297" t="inlineStr">
+        <is>
+          <t>Carne</t>
+        </is>
+      </c>
+      <c r="D885" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E885" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat</t>
+        </is>
+      </c>
+      <c r="F885" s="299" t="n">
+        <v>570</v>
+      </c>
+      <c r="G885" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H885" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I885" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J885" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="886">
+      <c r="B886" s="429" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C886" s="297" t="inlineStr">
+        <is>
+          <t>Pan Real</t>
+        </is>
+      </c>
+      <c r="D886" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E886" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Bread</t>
+        </is>
+      </c>
+      <c r="F886" s="299" t="n">
+        <v>1576</v>
+      </c>
+      <c r="G886" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H886" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I886" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J886" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="887">
+      <c r="B887" s="429" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C887" s="297" t="inlineStr">
+        <is>
+          <t>Sams Club</t>
+        </is>
+      </c>
+      <c r="D887" s="298" t="inlineStr">
+        <is>
+          <t>Sam's Club</t>
+        </is>
+      </c>
+      <c r="E887" s="297" t="inlineStr">
+        <is>
+          <t>Supermarket/General</t>
+        </is>
+      </c>
+      <c r="F887" s="299" t="n">
+        <v>1154</v>
+      </c>
+      <c r="G887" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H887" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I887" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J887" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="888">
+      <c r="B888" s="429" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C888" s="297" t="inlineStr">
+        <is>
+          <t>Chedraui</t>
+        </is>
+      </c>
+      <c r="D888" s="298" t="inlineStr">
+        <is>
+          <t>Chedraui</t>
+        </is>
+      </c>
+      <c r="E888" s="297" t="inlineStr">
+        <is>
+          <t>Supermarket/General</t>
+        </is>
+      </c>
+      <c r="F888" s="299" t="n">
+        <v>104</v>
+      </c>
+      <c r="G888" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H888" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I888" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J888" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="889">
+      <c r="B889" s="429" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C889" s="297" t="inlineStr">
+        <is>
+          <t>Julio Contador</t>
+        </is>
+      </c>
+      <c r="D889" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E889" s="297" t="inlineStr">
+        <is>
+          <t>Professional Services</t>
+        </is>
+      </c>
+      <c r="F889" s="299" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G889" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H889" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I889" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J889" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="890">
+      <c r="B890" s="429" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C890" s="297" t="inlineStr">
+        <is>
+          <t>Taxes</t>
+        </is>
+      </c>
+      <c r="D890" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E890" s="297" t="inlineStr">
+        <is>
+          <t>Taxes</t>
+        </is>
+      </c>
+      <c r="F890" s="299" t="n">
+        <v>4756</v>
+      </c>
+      <c r="G890" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H890" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I890" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J890" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="891">
+      <c r="B891" s="429" t="n">
+        <v>46315</v>
+      </c>
+      <c r="C891" s="297" t="inlineStr">
+        <is>
+          <t>Pollo</t>
+        </is>
+      </c>
+      <c r="D891" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E891" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat</t>
+        </is>
+      </c>
+      <c r="F891" s="299" t="n">
+        <v>1334</v>
+      </c>
+      <c r="G891" s="300" t="inlineStr">
+        <is>
+          <t>Lohith</t>
+        </is>
+      </c>
+      <c r="H891" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I891" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J891" s="423" t="inlineStr">
         <is>
           <t>Pagado por Lohith (bolsillo); reembolsable via Owner Ledger</t>
         </is>
@@ -75411,7 +75870,7 @@
     <row r="22">
       <c r="A22" s="439" t="inlineStr">
         <is>
-          <t>Utilities/Electricity</t>
+          <t>Taxes</t>
         </is>
       </c>
       <c r="B22" s="437">
@@ -75447,7 +75906,7 @@
     <row r="23">
       <c r="A23" s="439" t="inlineStr">
         <is>
-          <t>Taxes</t>
+          <t>Utilities/Electricity</t>
         </is>
       </c>
       <c r="B23" s="437">
@@ -75519,7 +75978,7 @@
     <row r="25">
       <c r="A25" s="439" t="inlineStr">
         <is>
-          <t>Ingredients - Beverages</t>
+          <t>Ingredients - Bread</t>
         </is>
       </c>
       <c r="B25" s="437">
@@ -75555,7 +76014,7 @@
     <row r="26">
       <c r="A26" s="439" t="inlineStr">
         <is>
-          <t>Ingredients - Dairy</t>
+          <t>Ingredients - Beverages</t>
         </is>
       </c>
       <c r="B26" s="437">
@@ -75591,7 +76050,7 @@
     <row r="27">
       <c r="A27" s="439" t="inlineStr">
         <is>
-          <t>Ingredients - Bread</t>
+          <t>Ingredients - Dairy</t>
         </is>
       </c>
       <c r="B27" s="437">
@@ -75807,7 +76266,7 @@
     <row r="33">
       <c r="A33" s="439" t="inlineStr">
         <is>
-          <t>Kitchen Supplies</t>
+          <t>Professional Services</t>
         </is>
       </c>
       <c r="B33" s="437">
@@ -75843,7 +76302,7 @@
     <row r="34">
       <c r="A34" s="439" t="inlineStr">
         <is>
-          <t>Professional Services</t>
+          <t>Kitchen Supplies</t>
         </is>
       </c>
       <c r="B34" s="437">

</xml_diff>

<commit_message>
LOKA 21-Oct-2026 | EOD | day 2026-10-21: rev $4,950 exp $3,501 net $1,449 | bal vs capital $-14,754
Changed: LOKA_Restaurant_Manager.xlsx, categories.json, dashboard.html, today.txt
+ 3 backup/day file(s)
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -5871,7 +5871,7 @@
         </is>
       </c>
       <c r="C172" s="455" t="n">
-        <v>-16094.43</v>
+        <v>-14753.63</v>
       </c>
       <c r="E172" s="423" t="inlineStr">
         <is>
@@ -5886,7 +5886,7 @@
         </is>
       </c>
       <c r="C173" s="457" t="n">
-        <v>109839.57</v>
+        <v>111180.37</v>
       </c>
       <c r="E173" s="423" t="inlineStr">
         <is>
@@ -11573,7 +11573,7 @@
       <c r="E6" s="29" t="n"/>
       <c r="F6" s="30">
         <f>SUMIFS($D$8:$D$5000,$B$8:$B$5000,TODAY())+SUMIFS($E$8:$E$5000,$B$8:$B$5000,TODAY())+SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())+SUMIFS($U$8:$U$5000,$B$8:$B$5000,TODAY())+SUMIFS($Y$8:$Y$5000,$B$8:$B$5000,TODAY())</f>
-        <v>4395.0</v>
+        <v>4950.0</v>
       </c>
       <c r="G6" s="31">
         <f>SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())</f>
@@ -11581,37 +11581,37 @@
       </c>
       <c r="H6" s="28">
         <f>SUMIFS($H$8:$H$5000,$B$8:$B$5000,TODAY())</f>
-        <v>11580.0</v>
+        <v>3501.0</v>
       </c>
       <c r="I6" s="32">
         <f>F6-H6</f>
-        <v>-7185.0</v>
+        <v>1449.0</v>
       </c>
       <c r="J6">
         <f>IFERROR(I6/F6,0)</f>
-        <v>-1.634812</v>
+        <v>0.292727</v>
       </c>
       <c r="K6" s="28" t="n"/>
       <c r="L6" s="31" t="n"/>
       <c r="M6" s="28">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>10080.0</v>
+        <v>15030.0</v>
       </c>
       <c r="N6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>10080.0</v>
+        <v>15030.0</v>
       </c>
       <c r="O6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),$B$8:$B$5000,"&lt;"&amp;DATE(YEAR(TODAY()),MONTH(TODAY())+1,1))</f>
-        <v>66550.0</v>
+        <v>71500.0</v>
       </c>
       <c r="P6">
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>12982.0</v>
+        <v>16483.0</v>
       </c>
       <c r="Q6">
         <f>M6-P6</f>
-        <v>-2902.0</v>
+        <v>-1453.0</v>
       </c>
     </row>
     <row r="7" ht="27.75" customHeight="1" s="331">
@@ -20616,33 +20616,72 @@
       <c r="AB144" s="324" t="n"/>
     </row>
     <row r="145" ht="16.5" customHeight="1" s="331">
-      <c r="B145" s="34" t="n"/>
-      <c r="C145" s="47" t="n"/>
-      <c r="D145" s="48" t="n"/>
-      <c r="E145" s="49" t="n"/>
-      <c r="F145" s="50" t="n"/>
-      <c r="G145" s="51" t="n"/>
-      <c r="H145" s="52" t="n"/>
-      <c r="I145" s="53" t="n"/>
-      <c r="J145" s="54" t="n"/>
-      <c r="K145" s="55" t="n"/>
-      <c r="L145" s="18" t="n"/>
-      <c r="M145" s="21" t="n"/>
-      <c r="N145" s="56" t="n"/>
-      <c r="O145" s="57" t="n"/>
-      <c r="P145" s="58" t="n"/>
-      <c r="Q145" s="56" t="n"/>
-      <c r="R145" s="56" t="n"/>
-      <c r="S145" s="56" t="n"/>
-      <c r="T145" s="56" t="n"/>
-      <c r="U145" s="56" t="n"/>
-      <c r="V145" s="56" t="n"/>
-      <c r="W145" s="56" t="n"/>
-      <c r="X145" s="56" t="n"/>
-      <c r="Y145" s="56" t="n"/>
-      <c r="Z145" s="56" t="n"/>
-      <c r="AA145" s="56" t="n"/>
-      <c r="AB145" s="56" t="n"/>
+      <c r="B145" s="427" t="n">
+        <v>46316</v>
+      </c>
+      <c r="C145" s="255" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="D145" s="256" t="n">
+        <v>2665</v>
+      </c>
+      <c r="E145" s="49" t="n">
+        <v>2285</v>
+      </c>
+      <c r="F145" s="50">
+        <f>IFERROR(D145+E145+G145+U145+Y145,0)</f>
+        <v>4950.0</v>
+      </c>
+      <c r="G145" s="257" t="n">
+        <v>0</v>
+      </c>
+      <c r="H145" s="258">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B145,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B145+1))</f>
+        <v>3501.0</v>
+      </c>
+      <c r="I145" s="259">
+        <f>IFERROR(F145-H145,0)</f>
+        <v>1449.0</v>
+      </c>
+      <c r="J145" s="260">
+        <f>IFERROR(I145/F145,0)</f>
+        <v>0.292727</v>
+      </c>
+      <c r="K145" s="254" t="n"/>
+      <c r="L145" s="261" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
+      <c r="M145" s="291" t="n"/>
+      <c r="N145" s="292" t="n"/>
+      <c r="O145" s="293" t="n"/>
+      <c r="P145" s="294" t="n"/>
+      <c r="Q145" s="292" t="n"/>
+      <c r="R145" s="443">
+        <f>IFERROR(D145*$T$7,0)</f>
+        <v>108.2</v>
+      </c>
+      <c r="S145" s="292" t="n"/>
+      <c r="T145" s="292" t="n"/>
+      <c r="U145" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="V145" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="W145" s="292" t="n"/>
+      <c r="X145" s="292" t="n"/>
+      <c r="Y145" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z145" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA145" s="292" t="n"/>
+      <c r="AB145" s="292" t="n"/>
     </row>
     <row r="146" ht="16.5" customHeight="1" s="331">
       <c r="B146" s="34" t="n"/>
@@ -27229,8 +27268,8 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="I2:P2"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="I2:P2"/>
     <mergeCell ref="B5:P5"/>
     <mergeCell ref="A3:P3"/>
   </mergeCells>
@@ -27254,7 +27293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J891"/>
+  <dimension ref="A1:J895"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="4" customWidth="1" style="331" min="1" max="1"/>
@@ -65070,6 +65109,178 @@
       <c r="J891" s="423" t="inlineStr">
         <is>
           <t>Pagado por Lohith (bolsillo); reembolsable via Owner Ledger</t>
+        </is>
+      </c>
+    </row>
+    <row r="892">
+      <c r="B892" s="429" t="n">
+        <v>46316</v>
+      </c>
+      <c r="C892" s="297" t="inlineStr">
+        <is>
+          <t>Pescado</t>
+        </is>
+      </c>
+      <c r="D892" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E892" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat &amp; Fish</t>
+        </is>
+      </c>
+      <c r="F892" s="299" t="n">
+        <v>325</v>
+      </c>
+      <c r="G892" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H892" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I892" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J892" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="893">
+      <c r="B893" s="429" t="n">
+        <v>46316</v>
+      </c>
+      <c r="C893" s="297" t="inlineStr">
+        <is>
+          <t>Carne</t>
+        </is>
+      </c>
+      <c r="D893" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E893" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat</t>
+        </is>
+      </c>
+      <c r="F893" s="299" t="n">
+        <v>570</v>
+      </c>
+      <c r="G893" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H893" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I893" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J893" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="894">
+      <c r="B894" s="429" t="n">
+        <v>46316</v>
+      </c>
+      <c r="C894" s="297" t="inlineStr">
+        <is>
+          <t>Etrusca</t>
+        </is>
+      </c>
+      <c r="D894" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E894" s="297" t="inlineStr">
+        <is>
+          <t>Supplies/Other</t>
+        </is>
+      </c>
+      <c r="F894" s="299" t="n">
+        <v>1796</v>
+      </c>
+      <c r="G894" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H894" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I894" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J894" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="B895" s="429" t="n">
+        <v>46316</v>
+      </c>
+      <c r="C895" s="297" t="inlineStr">
+        <is>
+          <t>Soft App</t>
+        </is>
+      </c>
+      <c r="D895" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E895" s="297" t="inlineStr">
+        <is>
+          <t>Software/Subscription</t>
+        </is>
+      </c>
+      <c r="F895" s="299" t="n">
+        <v>810</v>
+      </c>
+      <c r="G895" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H895" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I895" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J895" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
         </is>
       </c>
     </row>
@@ -76086,7 +76297,7 @@
     <row r="28">
       <c r="A28" s="439" t="inlineStr">
         <is>
-          <t>Ingredients - Meat &amp; Fish</t>
+          <t>Supplies/Other</t>
         </is>
       </c>
       <c r="B28" s="437">
@@ -76122,7 +76333,7 @@
     <row r="29">
       <c r="A29" s="439" t="inlineStr">
         <is>
-          <t>Supplies/Other</t>
+          <t>Ingredients - Meat &amp; Fish</t>
         </is>
       </c>
       <c r="B29" s="437">
@@ -76338,7 +76549,7 @@
     <row r="35">
       <c r="A35" s="439" t="inlineStr">
         <is>
-          <t>Ingredients - Fruit</t>
+          <t>Software/Subscription</t>
         </is>
       </c>
       <c r="B35" s="437">
@@ -76374,7 +76585,7 @@
     <row r="36">
       <c r="A36" s="439" t="inlineStr">
         <is>
-          <t>Utilities/Internet</t>
+          <t>Ingredients - Fruit</t>
         </is>
       </c>
       <c r="B36" s="437">
@@ -76410,7 +76621,7 @@
     <row r="37">
       <c r="A37" s="439" t="inlineStr">
         <is>
-          <t>Software/Subscription</t>
+          <t>Utilities/Internet</t>
         </is>
       </c>
       <c r="B37" s="437">

</xml_diff>

<commit_message>
LOKA 22-Oct-2026 | EOD | day 2026-10-22: rev $4,690 exp $1,294 net $3,396 | bal vs capital $-11,462
Changed: LOKA_Restaurant_Manager.xlsx, dashboard.html, today.txt
+ 2 backup/day file(s)
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -5871,7 +5871,7 @@
         </is>
       </c>
       <c r="C172" s="455" t="n">
-        <v>-14753.63</v>
+        <v>-11461.74</v>
       </c>
       <c r="E172" s="423" t="inlineStr">
         <is>
@@ -5886,7 +5886,7 @@
         </is>
       </c>
       <c r="C173" s="457" t="n">
-        <v>111180.37</v>
+        <v>114472.26</v>
       </c>
       <c r="E173" s="423" t="inlineStr">
         <is>
@@ -11573,7 +11573,7 @@
       <c r="E6" s="29" t="n"/>
       <c r="F6" s="30">
         <f>SUMIFS($D$8:$D$5000,$B$8:$B$5000,TODAY())+SUMIFS($E$8:$E$5000,$B$8:$B$5000,TODAY())+SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())+SUMIFS($U$8:$U$5000,$B$8:$B$5000,TODAY())+SUMIFS($Y$8:$Y$5000,$B$8:$B$5000,TODAY())</f>
-        <v>4950.0</v>
+        <v>4690.0</v>
       </c>
       <c r="G6" s="31">
         <f>SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())</f>
@@ -11581,37 +11581,37 @@
       </c>
       <c r="H6" s="28">
         <f>SUMIFS($H$8:$H$5000,$B$8:$B$5000,TODAY())</f>
-        <v>3501.0</v>
+        <v>1294.0</v>
       </c>
       <c r="I6" s="32">
         <f>F6-H6</f>
-        <v>1449.0</v>
+        <v>3396.0</v>
       </c>
       <c r="J6">
         <f>IFERROR(I6/F6,0)</f>
-        <v>0.292727</v>
+        <v>0.724094</v>
       </c>
       <c r="K6" s="28" t="n"/>
       <c r="L6" s="31" t="n"/>
       <c r="M6" s="28">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>15030.0</v>
+        <v>19720.0</v>
       </c>
       <c r="N6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>15030.0</v>
+        <v>19720.0</v>
       </c>
       <c r="O6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),$B$8:$B$5000,"&lt;"&amp;DATE(YEAR(TODAY()),MONTH(TODAY())+1,1))</f>
-        <v>71500.0</v>
+        <v>76190.0</v>
       </c>
       <c r="P6">
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>16483.0</v>
+        <v>17777.0</v>
       </c>
       <c r="Q6">
         <f>M6-P6</f>
-        <v>-1453.0</v>
+        <v>1943.0</v>
       </c>
     </row>
     <row r="7" ht="27.75" customHeight="1" s="331">
@@ -20684,33 +20684,72 @@
       <c r="AB145" s="292" t="n"/>
     </row>
     <row r="146" ht="16.5" customHeight="1" s="331">
-      <c r="B146" s="34" t="n"/>
-      <c r="C146" s="35" t="n"/>
-      <c r="D146" s="36" t="n"/>
-      <c r="E146" s="37" t="n"/>
-      <c r="F146" s="38" t="n"/>
-      <c r="G146" s="39" t="n"/>
-      <c r="H146" s="40" t="n"/>
-      <c r="I146" s="41" t="n"/>
-      <c r="J146" s="42" t="n"/>
-      <c r="K146" s="43" t="n"/>
-      <c r="L146" s="9" t="n"/>
-      <c r="M146" s="12" t="n"/>
-      <c r="N146" s="44" t="n"/>
-      <c r="O146" s="45" t="n"/>
-      <c r="P146" s="46" t="n"/>
-      <c r="Q146" s="44" t="n"/>
-      <c r="R146" s="44" t="n"/>
-      <c r="S146" s="44" t="n"/>
-      <c r="T146" s="44" t="n"/>
-      <c r="U146" s="44" t="n"/>
-      <c r="V146" s="44" t="n"/>
-      <c r="W146" s="44" t="n"/>
-      <c r="X146" s="44" t="n"/>
-      <c r="Y146" s="44" t="n"/>
-      <c r="Z146" s="44" t="n"/>
-      <c r="AA146" s="44" t="n"/>
-      <c r="AB146" s="44" t="n"/>
+      <c r="B146" s="427" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C146" s="270" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D146" s="271" t="n">
+        <v>1895</v>
+      </c>
+      <c r="E146" s="37" t="n">
+        <v>1365</v>
+      </c>
+      <c r="F146" s="38">
+        <f>IFERROR(D146+E146+G146+U146+Y146,0)</f>
+        <v>4690.0</v>
+      </c>
+      <c r="G146" s="272" t="n">
+        <v>0</v>
+      </c>
+      <c r="H146" s="273">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B146,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B146+1))</f>
+        <v>1294.0</v>
+      </c>
+      <c r="I146" s="274">
+        <f>IFERROR(F146-H146,0)</f>
+        <v>3396.0</v>
+      </c>
+      <c r="J146" s="275">
+        <f>IFERROR(I146/F146,0)</f>
+        <v>0.724094</v>
+      </c>
+      <c r="K146" s="250" t="n"/>
+      <c r="L146" s="276" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
+      <c r="M146" s="323" t="n"/>
+      <c r="N146" s="324" t="n"/>
+      <c r="O146" s="325" t="n"/>
+      <c r="P146" s="326" t="n"/>
+      <c r="Q146" s="324" t="n"/>
+      <c r="R146" s="428">
+        <f>IFERROR(D146*$T$7,0)</f>
+        <v>76.94</v>
+      </c>
+      <c r="S146" s="324" t="n"/>
+      <c r="T146" s="324" t="n"/>
+      <c r="U146" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="V146" s="428" t="n">
+        <v>0</v>
+      </c>
+      <c r="W146" s="324" t="n"/>
+      <c r="X146" s="324" t="n"/>
+      <c r="Y146" s="428" t="n">
+        <v>1430</v>
+      </c>
+      <c r="Z146" s="428" t="n">
+        <v>27.17</v>
+      </c>
+      <c r="AA146" s="324" t="n"/>
+      <c r="AB146" s="324" t="n"/>
     </row>
     <row r="147" ht="16.5" customHeight="1" s="331">
       <c r="B147" s="34" t="n"/>
@@ -27268,9 +27307,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="B5:P5"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="I2:P2"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="B5:P5"/>
     <mergeCell ref="A3:P3"/>
   </mergeCells>
   <conditionalFormatting sqref="I8:I372">
@@ -27293,7 +27332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J895"/>
+  <dimension ref="A1:J902"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="4" customWidth="1" style="331" min="1" max="1"/>
@@ -65279,6 +65318,307 @@
         </is>
       </c>
       <c r="J895" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="896">
+      <c r="B896" s="429" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C896" s="297" t="inlineStr">
+        <is>
+          <t>Chedraui</t>
+        </is>
+      </c>
+      <c r="D896" s="298" t="inlineStr">
+        <is>
+          <t>Chedraui</t>
+        </is>
+      </c>
+      <c r="E896" s="297" t="inlineStr">
+        <is>
+          <t>Supermarket/General</t>
+        </is>
+      </c>
+      <c r="F896" s="299" t="n">
+        <v>252</v>
+      </c>
+      <c r="G896" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H896" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I896" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J896" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="B897" s="429" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C897" s="297" t="inlineStr">
+        <is>
+          <t>Vegetables</t>
+        </is>
+      </c>
+      <c r="D897" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E897" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Vegetables</t>
+        </is>
+      </c>
+      <c r="F897" s="299" t="n">
+        <v>118</v>
+      </c>
+      <c r="G897" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H897" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I897" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J897" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="B898" s="429" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C898" s="297" t="inlineStr">
+        <is>
+          <t>Mango</t>
+        </is>
+      </c>
+      <c r="D898" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E898" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Vegetables</t>
+        </is>
+      </c>
+      <c r="F898" s="299" t="n">
+        <v>425</v>
+      </c>
+      <c r="G898" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H898" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I898" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J898" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="B899" s="429" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C899" s="297" t="inlineStr">
+        <is>
+          <t>Pan Dulce</t>
+        </is>
+      </c>
+      <c r="D899" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E899" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Bread</t>
+        </is>
+      </c>
+      <c r="F899" s="299" t="n">
+        <v>64</v>
+      </c>
+      <c r="G899" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H899" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I899" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J899" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="900">
+      <c r="B900" s="429" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C900" s="297" t="inlineStr">
+        <is>
+          <t>Pollo</t>
+        </is>
+      </c>
+      <c r="D900" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E900" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat</t>
+        </is>
+      </c>
+      <c r="F900" s="299" t="n">
+        <v>185</v>
+      </c>
+      <c r="G900" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H900" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I900" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J900" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="901">
+      <c r="B901" s="429" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C901" s="297" t="inlineStr">
+        <is>
+          <t>Molino</t>
+        </is>
+      </c>
+      <c r="D901" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E901" s="297" t="inlineStr">
+        <is>
+          <t>Supermarket/General</t>
+        </is>
+      </c>
+      <c r="F901" s="299" t="n">
+        <v>138</v>
+      </c>
+      <c r="G901" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H901" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I901" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J901" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="902">
+      <c r="B902" s="429" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C902" s="297" t="inlineStr">
+        <is>
+          <t>Oxxo Aceite</t>
+        </is>
+      </c>
+      <c r="D902" s="298" t="inlineStr">
+        <is>
+          <t>OXXO</t>
+        </is>
+      </c>
+      <c r="E902" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Pantry</t>
+        </is>
+      </c>
+      <c r="F902" s="299" t="n">
+        <v>112</v>
+      </c>
+      <c r="G902" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H902" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I902" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J902" s="423" t="inlineStr">
         <is>
           <t>No receipt; cash</t>
         </is>

</xml_diff>

<commit_message>
LOKA 28-Oct-2026 | EOD | day 7170-10-23: rev $7,170 exp $2,619 net $4,551 | bal vs capital $-7,047
Changed: LOKA_Restaurant_Manager.xlsx, dashboard.html, today.txt
+ 2 backup/day file(s)
</commit_message>
<xml_diff>
--- a/LOKA_Restaurant_Manager.xlsx
+++ b/LOKA_Restaurant_Manager.xlsx
@@ -5871,7 +5871,7 @@
         </is>
       </c>
       <c r="C172" s="455" t="n">
-        <v>-11461.74</v>
+        <v>-7046.87</v>
       </c>
       <c r="E172" s="423" t="inlineStr">
         <is>
@@ -5886,7 +5886,7 @@
         </is>
       </c>
       <c r="C173" s="457" t="n">
-        <v>114472.26</v>
+        <v>118887.13</v>
       </c>
       <c r="E173" s="423" t="inlineStr">
         <is>
@@ -11573,7 +11573,7 @@
       <c r="E6" s="29" t="n"/>
       <c r="F6" s="30">
         <f>SUMIFS($D$8:$D$5000,$B$8:$B$5000,TODAY())+SUMIFS($E$8:$E$5000,$B$8:$B$5000,TODAY())+SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())+SUMIFS($U$8:$U$5000,$B$8:$B$5000,TODAY())+SUMIFS($Y$8:$Y$5000,$B$8:$B$5000,TODAY())</f>
-        <v>4690.0</v>
+        <v>7170.0</v>
       </c>
       <c r="G6" s="31">
         <f>SUMIFS($G$8:$G$5000,$B$8:$B$5000,TODAY())</f>
@@ -11581,37 +11581,37 @@
       </c>
       <c r="H6" s="28">
         <f>SUMIFS($H$8:$H$5000,$B$8:$B$5000,TODAY())</f>
-        <v>1294.0</v>
+        <v>2619.0</v>
       </c>
       <c r="I6" s="32">
         <f>F6-H6</f>
-        <v>3396.0</v>
+        <v>4551.0</v>
       </c>
       <c r="J6">
         <f>IFERROR(I6/F6,0)</f>
-        <v>0.724094</v>
+        <v>0.634728</v>
       </c>
       <c r="K6" s="28" t="n"/>
       <c r="L6" s="31" t="n"/>
       <c r="M6" s="28">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>19720.0</v>
+        <v>7170.0</v>
       </c>
       <c r="N6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>19720.0</v>
+        <v>7170.0</v>
       </c>
       <c r="O6" s="33">
         <f>SUMIFS($F$8:$F$5000,$B$8:$B$5000,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),$B$8:$B$5000,"&lt;"&amp;DATE(YEAR(TODAY()),MONTH(TODAY())+1,1))</f>
-        <v>76190.0</v>
+        <v>7170.0</v>
       </c>
       <c r="P6">
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),2)+1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(TODAY()-WEEKDAY(TODAY(),2)+8))</f>
-        <v>17777.0</v>
+        <v>2619.0</v>
       </c>
       <c r="Q6">
         <f>M6-P6</f>
-        <v>1943.0</v>
+        <v>4551.0</v>
       </c>
     </row>
     <row r="7" ht="27.75" customHeight="1" s="331">
@@ -20752,33 +20752,72 @@
       <c r="AB146" s="324" t="n"/>
     </row>
     <row r="147" ht="16.5" customHeight="1" s="331">
-      <c r="B147" s="34" t="n"/>
-      <c r="C147" s="47" t="n"/>
-      <c r="D147" s="48" t="n"/>
-      <c r="E147" s="49" t="n"/>
-      <c r="F147" s="50" t="n"/>
-      <c r="G147" s="51" t="n"/>
-      <c r="H147" s="52" t="n"/>
-      <c r="I147" s="53" t="n"/>
-      <c r="J147" s="54" t="n"/>
-      <c r="K147" s="55" t="n"/>
-      <c r="L147" s="18" t="n"/>
-      <c r="M147" s="21" t="n"/>
-      <c r="N147" s="56" t="n"/>
-      <c r="O147" s="57" t="n"/>
-      <c r="P147" s="58" t="n"/>
-      <c r="Q147" s="56" t="n"/>
-      <c r="R147" s="56" t="n"/>
-      <c r="S147" s="56" t="n"/>
-      <c r="T147" s="56" t="n"/>
-      <c r="U147" s="56" t="n"/>
-      <c r="V147" s="56" t="n"/>
-      <c r="W147" s="56" t="n"/>
-      <c r="X147" s="56" t="n"/>
-      <c r="Y147" s="56" t="n"/>
-      <c r="Z147" s="56" t="n"/>
-      <c r="AA147" s="56" t="n"/>
-      <c r="AB147" s="56" t="n"/>
+      <c r="B147" s="427" t="n">
+        <v>1925125</v>
+      </c>
+      <c r="C147" s="255" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D147" s="256" t="n">
+        <v>2155</v>
+      </c>
+      <c r="E147" s="49" t="n">
+        <v>2455</v>
+      </c>
+      <c r="F147" s="50">
+        <f>IFERROR(D147+E147+G147+U147+Y147,0)</f>
+        <v>7170.0</v>
+      </c>
+      <c r="G147" s="257" t="n">
+        <v>0</v>
+      </c>
+      <c r="H147" s="258">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;B147,'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;(B147+1))</f>
+        <v>2619.0</v>
+      </c>
+      <c r="I147" s="259">
+        <f>IFERROR(F147-H147,0)</f>
+        <v>4551.0</v>
+      </c>
+      <c r="J147" s="260">
+        <f>IFERROR(I147/F147,0)</f>
+        <v>0.634728</v>
+      </c>
+      <c r="K147" s="254" t="n"/>
+      <c r="L147" s="261" t="inlineStr">
+        <is>
+          <t>Cierre via loka.py</t>
+        </is>
+      </c>
+      <c r="M147" s="291" t="n"/>
+      <c r="N147" s="292" t="n"/>
+      <c r="O147" s="293" t="n"/>
+      <c r="P147" s="294" t="n"/>
+      <c r="Q147" s="292" t="n"/>
+      <c r="R147" s="443">
+        <f>IFERROR(D147*$T$7,0)</f>
+        <v>87.49</v>
+      </c>
+      <c r="S147" s="292" t="n"/>
+      <c r="T147" s="292" t="n"/>
+      <c r="U147" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="V147" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="W147" s="292" t="n"/>
+      <c r="X147" s="292" t="n"/>
+      <c r="Y147" s="443" t="n">
+        <v>2560</v>
+      </c>
+      <c r="Z147" s="443" t="n">
+        <v>48.64</v>
+      </c>
+      <c r="AA147" s="292" t="n"/>
+      <c r="AB147" s="292" t="n"/>
     </row>
     <row r="148" ht="16.5" customHeight="1" s="331">
       <c r="B148" s="34" t="n"/>
@@ -27307,9 +27346,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="B5:P5"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="I2:P2"/>
+    <mergeCell ref="B5:P5"/>
     <mergeCell ref="A3:P3"/>
   </mergeCells>
   <conditionalFormatting sqref="I8:I372">
@@ -27332,7 +27371,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J902"/>
+  <dimension ref="A1:J907"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="4" customWidth="1" style="331" min="1" max="1"/>
@@ -65621,6 +65660,221 @@
       <c r="J902" s="423" t="inlineStr">
         <is>
           <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="903">
+      <c r="B903" s="429" t="n">
+        <v>1925125</v>
+      </c>
+      <c r="C903" s="297" t="inlineStr">
+        <is>
+          <t>Pan Real</t>
+        </is>
+      </c>
+      <c r="D903" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E903" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Bread</t>
+        </is>
+      </c>
+      <c r="F903" s="299" t="n">
+        <v>288</v>
+      </c>
+      <c r="G903" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H903" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I903" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J903" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="904">
+      <c r="B904" s="429" t="n">
+        <v>1925125</v>
+      </c>
+      <c r="C904" s="297" t="inlineStr">
+        <is>
+          <t>Oxxo</t>
+        </is>
+      </c>
+      <c r="D904" s="298" t="inlineStr">
+        <is>
+          <t>OXXO</t>
+        </is>
+      </c>
+      <c r="E904" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Pantry</t>
+        </is>
+      </c>
+      <c r="F904" s="299" t="n">
+        <v>108</v>
+      </c>
+      <c r="G904" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H904" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I904" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J904" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="905">
+      <c r="B905" s="429" t="n">
+        <v>1925125</v>
+      </c>
+      <c r="C905" s="297" t="inlineStr">
+        <is>
+          <t>Carne</t>
+        </is>
+      </c>
+      <c r="D905" s="298" t="inlineStr">
+        <is>
+          <t>No bill</t>
+        </is>
+      </c>
+      <c r="E905" s="297" t="inlineStr">
+        <is>
+          <t>Ingredients - Meat</t>
+        </is>
+      </c>
+      <c r="F905" s="299" t="n">
+        <v>292</v>
+      </c>
+      <c r="G905" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H905" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I905" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J905" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="906">
+      <c r="B906" s="429" t="n">
+        <v>1925125</v>
+      </c>
+      <c r="C906" s="297" t="inlineStr">
+        <is>
+          <t>Sams club</t>
+        </is>
+      </c>
+      <c r="D906" s="298" t="inlineStr">
+        <is>
+          <t>Sam's Club</t>
+        </is>
+      </c>
+      <c r="E906" s="297" t="inlineStr">
+        <is>
+          <t>Supermarket/General</t>
+        </is>
+      </c>
+      <c r="F906" s="299" t="n">
+        <v>471</v>
+      </c>
+      <c r="G906" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H906" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I906" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J906" s="423" t="inlineStr">
+        <is>
+          <t>No receipt; cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="907">
+      <c r="B907" s="429" t="n">
+        <v>1925125</v>
+      </c>
+      <c r="C907" s="297" t="inlineStr">
+        <is>
+          <t>Duvi - salary</t>
+        </is>
+      </c>
+      <c r="D907" s="298" t="inlineStr">
+        <is>
+          <t>Payroll</t>
+        </is>
+      </c>
+      <c r="E907" s="297" t="inlineStr">
+        <is>
+          <t>Staff - Salary</t>
+        </is>
+      </c>
+      <c r="F907" s="299" t="n">
+        <v>1460</v>
+      </c>
+      <c r="G907" s="300" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="H907" s="300" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I907" s="301" t="inlineStr">
+        <is>
+          <t>✅ Paid</t>
+        </is>
+      </c>
+      <c r="J907" s="423" t="inlineStr">
+        <is>
+          <t>Weekly salary</t>
         </is>
       </c>
     </row>
@@ -75719,7 +75973,7 @@
     <col width="15" customWidth="1" style="331" min="5" max="5"/>
     <col width="15" customWidth="1" style="331" min="6" max="14"/>
     <col width="15" customWidth="1" style="331" min="7" max="7"/>
-    <col width="9" customWidth="1" style="331" min="8" max="8"/>
+    <col width="15" customWidth="1" style="331" min="8" max="8"/>
     <col width="9" customWidth="1" style="331" min="9" max="9"/>
     <col width="9" customWidth="1" style="331" min="10" max="10"/>
     <col width="9" customWidth="1" style="331" min="11" max="11"/>
@@ -75740,7 +75994,7 @@
       <c r="E1" s="423" t="n"/>
       <c r="F1" s="423" t="n"/>
       <c r="G1" s="423" t="n"/>
-      <c r="H1" s="433" t="n"/>
+      <c r="H1" s="423" t="n"/>
       <c r="I1" s="433" t="n"/>
       <c r="J1" s="433" t="n"/>
       <c r="K1" s="433" t="n"/>
@@ -75796,7 +76050,11 @@
           <t>Oct 2026</t>
         </is>
       </c>
-      <c r="H3" s="433" t="n"/>
+      <c r="H3" s="435" t="inlineStr">
+        <is>
+          <t>Oct 7170</t>
+        </is>
+      </c>
       <c r="I3" s="433" t="n"/>
       <c r="J3" s="433" t="n"/>
       <c r="K3" s="433" t="n"/>
@@ -75832,7 +76090,10 @@
         <f>SUMIFS('📅 Daily Log'!$F$8:$F$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H4" s="433" t="n"/>
+      <c r="H4" s="437">
+        <f>SUMIFS('📅 Daily Log'!$F$8:$F$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I4" s="433" t="n"/>
       <c r="J4" s="433" t="n"/>
       <c r="K4" s="433" t="n"/>
@@ -75868,7 +76129,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H5" s="433" t="n"/>
+      <c r="H5" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I5" s="433" t="n"/>
       <c r="J5" s="433" t="n"/>
       <c r="K5" s="433" t="n"/>
@@ -75904,7 +76168,10 @@
         <f>G4-G5</f>
         <v/>
       </c>
-      <c r="H6" s="433" t="n"/>
+      <c r="H6" s="438">
+        <f>H4-H5</f>
+        <v/>
+      </c>
       <c r="I6" s="433" t="n"/>
       <c r="J6" s="433" t="n"/>
       <c r="K6" s="433" t="n"/>
@@ -75940,7 +76207,10 @@
         <f>COUNTIFS('📅 Daily Log'!$F$8:$F$5000,"&gt;0",'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H7" s="433" t="n"/>
+      <c r="H7" s="440">
+        <f>COUNTIFS('📅 Daily Log'!$F$8:$F$5000,"&gt;0",'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I7" s="433" t="n"/>
       <c r="J7" s="433" t="n"/>
       <c r="K7" s="433" t="n"/>
@@ -75976,7 +76246,10 @@
         <f>IFERROR(G4/G7,0)</f>
         <v/>
       </c>
-      <c r="H8" s="433" t="n"/>
+      <c r="H8" s="437">
+        <f>IFERROR(H4/H7,0)</f>
+        <v/>
+      </c>
       <c r="I8" s="433" t="n"/>
       <c r="J8" s="433" t="n"/>
       <c r="K8" s="433" t="n"/>
@@ -76032,7 +76305,11 @@
           <t>Oct 2026</t>
         </is>
       </c>
-      <c r="H10" s="433" t="n"/>
+      <c r="H10" s="435" t="inlineStr">
+        <is>
+          <t>Oct 7170</t>
+        </is>
+      </c>
       <c r="I10" s="433" t="n"/>
       <c r="J10" s="433" t="n"/>
       <c r="K10" s="433" t="n"/>
@@ -76068,7 +76345,10 @@
         <f>SUMIFS('📅 Daily Log'!$D$8:$D$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))+SUMIFS('📅 Daily Log'!$U$8:$U$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))+SUMIFS('📅 Daily Log'!$Y$8:$Y$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H11" s="433" t="n"/>
+      <c r="H11" s="437">
+        <f>SUMIFS('📅 Daily Log'!$D$8:$D$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))+SUMIFS('📅 Daily Log'!$U$8:$U$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))+SUMIFS('📅 Daily Log'!$Y$8:$Y$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I11" s="433" t="n"/>
       <c r="J11" s="433" t="n"/>
       <c r="K11" s="433" t="n"/>
@@ -76104,7 +76384,10 @@
         <f>SUMIFS('📅 Daily Log'!$E$8:$E$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H12" s="433" t="n"/>
+      <c r="H12" s="437">
+        <f>SUMIFS('📅 Daily Log'!$E$8:$E$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I12" s="433" t="n"/>
       <c r="J12" s="433" t="n"/>
       <c r="K12" s="433" t="n"/>
@@ -76140,7 +76423,10 @@
         <f>SUMIFS('📅 Daily Log'!$G$8:$G$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H13" s="433" t="n"/>
+      <c r="H13" s="437">
+        <f>SUMIFS('📅 Daily Log'!$G$8:$G$5000,'📅 Daily Log'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'📅 Daily Log'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I13" s="433" t="n"/>
       <c r="J13" s="433" t="n"/>
       <c r="K13" s="433" t="n"/>
@@ -76176,7 +76462,10 @@
         <f>G11+G12+G13</f>
         <v/>
       </c>
-      <c r="H14" s="433" t="n"/>
+      <c r="H14" s="438">
+        <f>H11+H12+H13</f>
+        <v/>
+      </c>
       <c r="I14" s="433" t="n"/>
       <c r="J14" s="433" t="n"/>
       <c r="K14" s="433" t="n"/>
@@ -76232,7 +76521,11 @@
           <t>Oct 2026</t>
         </is>
       </c>
-      <c r="H16" s="433" t="n"/>
+      <c r="H16" s="435" t="inlineStr">
+        <is>
+          <t>Oct 7170</t>
+        </is>
+      </c>
       <c r="I16" s="433" t="n"/>
       <c r="J16" s="433" t="n"/>
       <c r="K16" s="433" t="n"/>
@@ -76268,7 +76561,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A17,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H17" s="433" t="n"/>
+      <c r="H17" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A17,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I17" s="433" t="n"/>
       <c r="J17" s="433" t="n"/>
       <c r="K17" s="433" t="n"/>
@@ -76304,7 +76600,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A18,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H18" s="433" t="n"/>
+      <c r="H18" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A18,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I18" s="433" t="n"/>
       <c r="J18" s="433" t="n"/>
       <c r="K18" s="433" t="n"/>
@@ -76340,7 +76639,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A19,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H19" s="433" t="n"/>
+      <c r="H19" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A19,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I19" s="433" t="n"/>
       <c r="J19" s="433" t="n"/>
       <c r="K19" s="433" t="n"/>
@@ -76376,7 +76678,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A20,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H20" s="433" t="n"/>
+      <c r="H20" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A20,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I20" s="433" t="n"/>
       <c r="J20" s="433" t="n"/>
       <c r="K20" s="433" t="n"/>
@@ -76412,7 +76717,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A21,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H21" s="433" t="n"/>
+      <c r="H21" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A21,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I21" s="433" t="n"/>
       <c r="J21" s="433" t="n"/>
       <c r="K21" s="433" t="n"/>
@@ -76448,7 +76756,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A22,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H22" s="433" t="n"/>
+      <c r="H22" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A22,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I22" s="433" t="n"/>
       <c r="J22" s="433" t="n"/>
       <c r="K22" s="433" t="n"/>
@@ -76484,7 +76795,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A23,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H23" s="433" t="n"/>
+      <c r="H23" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A23,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I23" s="433" t="n"/>
       <c r="J23" s="433" t="n"/>
       <c r="K23" s="433" t="n"/>
@@ -76520,7 +76834,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A24,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H24" s="433" t="n"/>
+      <c r="H24" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A24,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I24" s="433" t="n"/>
       <c r="J24" s="433" t="n"/>
       <c r="K24" s="433" t="n"/>
@@ -76556,7 +76873,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A25,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H25" s="433" t="n"/>
+      <c r="H25" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A25,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I25" s="433" t="n"/>
       <c r="J25" s="433" t="n"/>
       <c r="K25" s="433" t="n"/>
@@ -76592,7 +76912,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A26,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H26" s="433" t="n"/>
+      <c r="H26" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A26,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I26" s="433" t="n"/>
       <c r="J26" s="433" t="n"/>
       <c r="K26" s="433" t="n"/>
@@ -76628,7 +76951,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A27,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H27" s="433" t="n"/>
+      <c r="H27" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A27,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I27" s="433" t="n"/>
       <c r="J27" s="433" t="n"/>
       <c r="K27" s="433" t="n"/>
@@ -76664,7 +76990,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A28,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H28" s="433" t="n"/>
+      <c r="H28" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A28,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I28" s="433" t="n"/>
       <c r="J28" s="433" t="n"/>
       <c r="K28" s="433" t="n"/>
@@ -76700,7 +77029,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A29,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H29" s="433" t="n"/>
+      <c r="H29" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A29,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I29" s="433" t="n"/>
       <c r="J29" s="433" t="n"/>
       <c r="K29" s="433" t="n"/>
@@ -76736,7 +77068,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A30,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H30" s="433" t="n"/>
+      <c r="H30" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A30,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I30" s="433" t="n"/>
       <c r="J30" s="433" t="n"/>
       <c r="K30" s="433" t="n"/>
@@ -76772,7 +77107,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A31,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H31" s="433" t="n"/>
+      <c r="H31" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A31,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I31" s="433" t="n"/>
       <c r="J31" s="433" t="n"/>
       <c r="K31" s="433" t="n"/>
@@ -76808,7 +77146,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A32,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H32" s="433" t="n"/>
+      <c r="H32" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A32,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I32" s="433" t="n"/>
       <c r="J32" s="433" t="n"/>
       <c r="K32" s="433" t="n"/>
@@ -76844,7 +77185,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A33,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H33" s="433" t="n"/>
+      <c r="H33" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A33,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I33" s="433" t="n"/>
       <c r="J33" s="433" t="n"/>
       <c r="K33" s="433" t="n"/>
@@ -76880,7 +77224,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A34,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H34" s="433" t="n"/>
+      <c r="H34" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A34,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I34" s="433" t="n"/>
       <c r="J34" s="433" t="n"/>
       <c r="K34" s="433" t="n"/>
@@ -76916,7 +77263,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A35,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H35" s="433" t="n"/>
+      <c r="H35" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A35,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I35" s="433" t="n"/>
       <c r="J35" s="433" t="n"/>
       <c r="K35" s="433" t="n"/>
@@ -76952,7 +77302,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A36,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H36" s="433" t="n"/>
+      <c r="H36" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A36,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I36" s="433" t="n"/>
       <c r="J36" s="433" t="n"/>
       <c r="K36" s="433" t="n"/>
@@ -76988,7 +77341,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A37,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H37" s="433" t="n"/>
+      <c r="H37" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A37,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I37" s="433" t="n"/>
       <c r="J37" s="433" t="n"/>
       <c r="K37" s="433" t="n"/>
@@ -77024,7 +77380,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A38,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H38" s="433" t="n"/>
+      <c r="H38" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A38,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I38" s="433" t="n"/>
       <c r="J38" s="433" t="n"/>
       <c r="K38" s="433" t="n"/>
@@ -77060,7 +77419,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A39,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H39" s="433" t="n"/>
+      <c r="H39" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A39,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I39" s="433" t="n"/>
       <c r="J39" s="433" t="n"/>
       <c r="K39" s="433" t="n"/>
@@ -77096,7 +77458,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A40,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H40" s="433" t="n"/>
+      <c r="H40" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A40,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I40" s="433" t="n"/>
       <c r="J40" s="433" t="n"/>
       <c r="K40" s="433" t="n"/>
@@ -77132,7 +77497,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A41,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H41" s="433" t="n"/>
+      <c r="H41" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A41,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I41" s="433" t="n"/>
       <c r="J41" s="433" t="n"/>
       <c r="K41" s="433" t="n"/>
@@ -77168,7 +77536,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A42,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H42" s="433" t="n"/>
+      <c r="H42" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A42,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I42" s="433" t="n"/>
       <c r="J42" s="433" t="n"/>
       <c r="K42" s="433" t="n"/>
@@ -77204,7 +77575,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A43,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H43" s="433" t="n"/>
+      <c r="H43" s="437">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$E$8:$E$5000,$A43,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I43" s="433" t="n"/>
       <c r="J43" s="433" t="n"/>
       <c r="K43" s="433" t="n"/>
@@ -77240,7 +77614,10 @@
         <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(2026,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(2026,11,1))</f>
         <v/>
       </c>
-      <c r="H44" s="433" t="n"/>
+      <c r="H44" s="438">
+        <f>SUMIFS('💸 Expenses'!$F$8:$F$5000,'💸 Expenses'!$B$8:$B$5000,"&gt;="&amp;DATE(7170,10,1),'💸 Expenses'!$B$8:$B$5000,"&lt;"&amp;DATE(7170,11,1))</f>
+        <v/>
+      </c>
       <c r="I44" s="433" t="n"/>
       <c r="J44" s="433" t="n"/>
       <c r="K44" s="433" t="n"/>
@@ -77276,7 +77653,10 @@
         <f>G4-G44</f>
         <v/>
       </c>
-      <c r="H45" s="433" t="n"/>
+      <c r="H45" s="438">
+        <f>H4-H44</f>
+        <v/>
+      </c>
       <c r="I45" s="433" t="n"/>
       <c r="J45" s="433" t="n"/>
       <c r="K45" s="433" t="n"/>
@@ -77494,7 +77874,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>